<commit_message>
docs: record verified GitHub repository handoff
</commit_message>
<xml_diff>
--- a/docs/project-control/So-quan-ly-tai-lieu.xlsx
+++ b/docs/project-control/So-quan-ly-tai-lieu.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bat dau" sheetId="1" r:id="Re1b17fa0ffdf433d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh muc" sheetId="2" r:id="R94c0da200428471f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anh huong" sheetId="3" r:id="R8cc99b7aa1dc4d52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quyet dinh" sheetId="4" r:id="R2f1a707825a6454d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dong bo" sheetId="5" r:id="R03dda1f0684b43d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quy trinh" sheetId="6" r:id="Reca33850a899469c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bat dau" sheetId="1" r:id="R8a8a9de6fdf34576"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh muc" sheetId="2" r:id="Re0f21705b2124758"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anh huong" sheetId="3" r:id="Rac27ff509c0f4e40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quyet dinh" sheetId="4" r:id="R41ed8e731b0a4b86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dong bo" sheetId="5" r:id="R1d163119f8ec4369"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quy trinh" sheetId="6" r:id="Ra5ddeda82f274795"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -489,7 +489,7 @@
     <x:row r="3">
       <x:c r="A3" s="1"/>
       <x:c r="B3" s="1" t="str">
-        <x:v>Dịch vụ quanh bạn — phiên bản 1.30, 28/09/2026</x:v>
+        <x:v>Dịch vụ quanh bạn — phiên bản 1.31, 28/09/2026</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>
@@ -537,7 +537,7 @@
       </x:c>
       <x:c r="C7" s="13" t="n">
         <x:f>COUNTA('Dong bo'!A6:A1000)-COUNTIFS('Dong bo'!L6:L1000,"Hoàn tất")-COUNTIFS('Dong bo'!L6:L1000,"Không áp dụng có lý do")</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D7" s="1"/>
       <x:c r="E7" s="1"/>
@@ -550,7 +550,7 @@
       </x:c>
       <x:c r="C8" s="13" t="n">
         <x:f>COUNTIFS('Dong bo'!L6:L1000,"Hoàn tất")</x:f>
-        <x:v>315</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="D8" s="1"/>
       <x:c r="E8" s="1"/>
@@ -751,7 +751,7 @@
     <x:hyperlink ref="B14" location="'Quyet dinh'!A1"/>
     <x:hyperlink ref="B15" location="'Dong bo'!A1"/>
     <x:hyperlink ref="B16" location="'Quy trinh'!A1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="Rc720501b49604dde"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="Rf358efb959044fde"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -887,7 +887,7 @@
         <x:v>Quản lý hồ sơ</x:v>
       </x:c>
       <x:c r="D6" s="8" t="str">
-        <x:v>v1.30</x:v>
+        <x:v>v1.31</x:v>
       </x:c>
       <x:c r="E6" s="8" t="str">
         <x:v>Sổ quản lý chính</x:v>
@@ -906,7 +906,7 @@
       </x:c>
       <x:c r="J6" s="8" t="str"/>
       <x:c r="K6" s="8" t="str">
-        <x:v>REPO-01: repo GitHub được chỉ định; Git local riêng; README/DOC-065 v1.1 và ZIP đồng bộ. Push chờ xác thực GitHub; không force-push, chưa kích hoạt CI.</x:v>
+        <x:v>REPO-01: repo private anhthaingd/dich-vu-quanh-ban; push main thành công commit 1f07065. DOC-065 v1.2 và ZIP đối chiếu Drive; CI chưa kích hoạt.</x:v>
       </x:c>
       <x:c r="L6" s="10" t="n">
         <x:v>46293</x:v>
@@ -1558,7 +1558,7 @@
       </x:c>
       <x:c r="J24" s="8" t="str"/>
       <x:c r="K24" s="8" t="str">
-        <x:v>REPO-01: repo GitHub được chỉ định; Git local riêng; README/DOC-065 v1.1 và ZIP đồng bộ. Push chờ xác thực GitHub; không force-push, chưa kích hoạt CI.</x:v>
+        <x:v>REPO-01: repo private anhthaingd/dich-vu-quanh-ban; push main thành công commit 1f07065. DOC-065 v1.2 và ZIP đối chiếu Drive; CI chưa kích hoạt.</x:v>
       </x:c>
       <x:c r="L24" s="10" t="n">
         <x:v>46293</x:v>
@@ -2674,7 +2674,7 @@
         <x:v>Bản trên Drive</x:v>
       </x:c>
       <x:c r="K55" s="20" t="str">
-        <x:v>REPO-01: repo GitHub được chỉ định; Git local riêng; README/DOC-065 v1.1 và ZIP đồng bộ. Push chờ xác thực GitHub; không force-push, chưa kích hoạt CI.</x:v>
+        <x:v>REPO-01: repo private anhthaingd/dich-vu-quanh-ban; push main thành công commit 1f07065. DOC-065 v1.2 và ZIP đối chiếu Drive; CI chưa kích hoạt.</x:v>
       </x:c>
       <x:c r="L55" s="21" t="n">
         <x:v>46293</x:v>
@@ -3206,7 +3206,7 @@
         <x:v>React/Storybook; UI-UX-v0.19.zip</x:v>
       </x:c>
       <x:c r="K69" s="24" t="str">
-        <x:v>REPO-01: repo GitHub được chỉ định; Git local riêng; README/DOC-065 v1.1 và ZIP đồng bộ. Push chờ xác thực GitHub; không force-push, chưa kích hoạt CI.</x:v>
+        <x:v>REPO-01: repo private anhthaingd/dich-vu-quanh-ban; push main thành công commit 1f07065. DOC-065 v1.2 và ZIP đối chiếu Drive; CI chưa kích hoạt.</x:v>
       </x:c>
       <x:c r="L69" s="24" t="n">
         <x:v>46293</x:v>
@@ -3603,7 +3603,7 @@
         <x:v>Triển khai</x:v>
       </x:c>
       <x:c r="D80" s="24" t="str">
-        <x:v>v1.1</x:v>
+        <x:v>v1.2</x:v>
       </x:c>
       <x:c r="E80" s="24" t="str">
         <x:v>Nguồn hiện trạng và kết quả local</x:v>
@@ -3624,7 +3624,7 @@
         <x:v>docs/implementation/evidence; technical-design ZIP</x:v>
       </x:c>
       <x:c r="K80" s="24" t="str">
-        <x:v>REPO-01: repo GitHub được chỉ định; Git local riêng; README/DOC-065 v1.1 và ZIP đồng bộ. Push chờ xác thực GitHub; không force-push, chưa kích hoạt CI.</x:v>
+        <x:v>REPO-01: repo private anhthaingd/dich-vu-quanh-ban; push main thành công commit 1f07065. DOC-065 v1.2 và ZIP đối chiếu Drive; CI chưa kích hoạt.</x:v>
       </x:c>
       <x:c r="L80" s="24" t="n">
         <x:v>46293</x:v>
@@ -3752,81 +3752,81 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="Rfc5bee286977423c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R63c9785f87ca435a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="R1a2f2a11f2a0495f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="R1f45e9912ffd4495"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="R9bec97ccacd74b5a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="R16a0c1095e8e4742"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="R7217b0736e174c4a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R160e372270874e52"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="Ra95130749fad4ef1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="R1aa932d0060045a0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="R30cccaf1f100438b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="R98da1a7b93f74bd9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="Rd6728f4b36264d8e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="Rd135473f0a414976"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="R346d1aa43c004849"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="R0c6441ead7044b61"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="Rfb23edea01414865"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="Rbc13dc060cfd4497"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="R71c42ebede1b4b51"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="R84ef922a403b4541"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="R8d92b73d1c4c4520"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="R666f277228124a62"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="R4fc409b18b99440c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="Rf5e7bfc4c5b142b2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="R6ae87af468e841bb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="Rca77a63e8059405a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="R44d71095e8bb4cd7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="Rc2460e21c945476c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="R4e5f248443ba41a1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R787ad2f7fb6a47c3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="R4c125e27355f49f6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="R26ac4c09450c47f6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R95aaa9ae8f5a4761"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R52b4de5bf8fa46f3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="R8fb89d1d1606453e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="Ra86537cf337b4b93"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="R6f52394fb10c4508"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="Rb11d1d1ef59d44e3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="Rcd08a6f918744a56"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="Ra5032974510f4df7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="R886897ec89e44085"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="Rb19a300a5afd49d3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="R2007845c909b466c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="Rf2dd9e8b6fff4532"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="R1fcdb2f9e00b4654"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="Rbe7e686a0d6a4ad8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="R41be55b567574142"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="Rad9c7f16dcde4340"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="R5cf5482f635d451b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="Rb2ecf78cdefa4231"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="Rc439fead09f84ac7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="R1d5790dd58504fb7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="Rbe82201723014d90"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="R028e8e31b77b4992"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="R9f26885f8cbc4a0d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="Rb6c6b35736514b9c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="R0404923f07384d93"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="R4ceb876b463e4c27"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="R8993cc6a7cf64b6a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="Raab142b00fe242c7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="R9d47c528a4e24053"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="R471898aa19714b9c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="Rfe0e4358673b44b4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="Rec0b67a0ebae44e0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="R93be6577ed5e42cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="R8ef24b7d64f040a8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="R3c007b281bef45e0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="Rdeb3d1de2e364625"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="R3222629127854fe9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="Ra3056876336f49a1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="R42fab58f2a4c437e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="R3bfb8b542ba948bd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R90e8f8cadd5a4a31"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="Rff13854e95ef486f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="Raa40edc5153849e0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="Re31d90a295724192"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="R8b05a5c0cac24c29"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="Rbd4da0d774294f9e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R2797de5ed5664496"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="R8327b7db10e54f58"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="Rfb181db4e9e8482e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="Re13a7670c9f54f8a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="R3ceb301323964d3e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="R6bf663f1e6134a74"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="R073c5a54f0da49c6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="Rf317f75b58f0467d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="R5673a7b3d9a34b26"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="R09d211447ae44e43"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="Rab448c5834e144ea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="Rdb22b4c057f54e1e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="R1e1c8ebc10d742c3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="Rcf069d82cf564852"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="R12cecd4c176c4ec2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="R99a41aae61714cb6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="Ra4122904c9284635"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="Rd278aedd602749ce"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="Rf6f6f1a7010948b1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="R698c1015bf08450e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="R3861919cee164503"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="R602be373e7aa4a8c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="Rab8dd8c5ad884ae8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="Rfbe536ad88694a4f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="Rdc6aab794baf4f43"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R811781f3eb2c437d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="Rac0aaa5910bb4e9a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="R436c11a8d0e84b29"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="Rdc6663a48a1045ca"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="Rb4df92c73d5346c9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="R5e2cd171d5854f41"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="R2d1102e892dd496b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="R88e04be7926a40c8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="R89bd24ccdb394e91"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="R82eb2fd25ae545ab"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="Ra6be5fba70bc4803"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="R78f2d58d8efb4570"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="Rbaea0ec0e42e4d8e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="R9047fa5f0d9b4175"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="R8a72e1092b964f96"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="R814b96e28a484509"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="R9969d724e0924304"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="R35035a9c17b94049"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="R966de9f703e4406e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="R513f06d1b4394c2d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="Ra94f6ac1f8da4565"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="R1ba44f791d56487a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="Rbb0bb346fdd74c3a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="R71ff83ce6e3d4baa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="Rff8a1b1817e44218"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="R09370944a69c4014"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="Ra1d31eb104e84c88"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="Rcfd04fdc6bc445de"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="R4226b2934c4a42a9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="R5616c754bdc04b28"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="R53d26bc0a5884dbc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="Rde58ebc803d74ebc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="R10c25084ff214c9b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="Raae97f50fc694b7b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="R8ec99cb898fe4148"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="R0605d6bcb5be48b1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="R8500af7296e54e07"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="Ra48dadf901b54365"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="R5d00e157ef7c4b89"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R333b3706905d46c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9625b3821294854"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19882,7 +19882,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R457fb38ac93b41e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28b146e11e994690"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20989,7 +20989,7 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="D51" s="24" t="str">
-        <x:v>Native còn thiếu simctl/adb/thiết bị. Repository đã chỉ định theo REPO-01; remote CI chưa kích hoạt. Push hiện chờ tài khoản GitHub có quyền ghi.</x:v>
+        <x:v>Native còn thiếu simctl/adb/thiết bị. Repository đã chỉ định theo REPO-01 và push main thành công; remote CI chưa kích hoạt.</x:v>
       </x:c>
       <x:c r="E51" s="24" t="str">
         <x:v>F18</x:v>
@@ -21018,7 +21018,7 @@
         <x:v>F18/F20</x:v>
       </x:c>
       <x:c r="F52" s="24" t="str">
-        <x:v>Yêu cầu trực tiếp 28/09/2026; README; DOC-065 v1.1. Push chờ xác thực GitHub.</x:v>
+        <x:v>Yêu cầu trực tiếp 28/09/2026; README; DOC-065 v1.2; origin/main: 1f070655aad0a0487b8d600e84554daa95b5465d. Repo private, không force-push.</x:v>
       </x:c>
       <x:c r="G52" s="25" t="n">
         <x:v>46293</x:v>
@@ -23871,7 +23871,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ef25fdb08f84f5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98c1015395ee4a79"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36930,7 +36930,7 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J343" s="24" t="str">
-        <x:v>DOC-065 v1.1: thiếu native; repo đã chọn REPO-01, CI template chưa kích hoạt; push chờ xác thực.</x:v>
+        <x:v>DOC-065 v1.2: thiếu native; repo đã push REPO-01; CI template chưa kích hoạt.</x:v>
       </x:c>
       <x:c r="K343" s="24" t="str">
         <x:v>Chưa kiểm native và remote CI; không dùng web/mock để đánh dấu đạt.</x:v>
@@ -36968,10 +36968,10 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J344" s="24" t="str">
-        <x:v>README/DOC-065 v1.1; Git root riêng; symlink tương đối; nguồn và ZIP đối chiếu Drive cùng ID.</x:v>
+        <x:v>DOC-065 v1.2; Git root riêng, symlink tương đối; push 1f07065 lên origin/main thành công; Drive cùng ID đọc lại.</x:v>
       </x:c>
       <x:c r="K344" s="24" t="str">
-        <x:v>Chưa push do thiếu quyền truy cập; CI chưa kích hoạt.</x:v>
+        <x:v>Repo private, xác thực anhthaingd qua Keychain; không force-push. CI chưa kích hoạt; native chưa kiểm.</x:v>
       </x:c>
       <x:c r="L344" s="24" t="str">
         <x:v>Hoàn tất</x:v>
@@ -37006,10 +37006,10 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J345" s="24" t="str">
-        <x:v>README/DOC-065 v1.1; Git root riêng; symlink tương đối; nguồn và ZIP đối chiếu Drive cùng ID.</x:v>
+        <x:v>DOC-065 v1.2; Git root riêng, symlink tương đối; push 1f07065 lên origin/main thành công; Drive cùng ID đọc lại.</x:v>
       </x:c>
       <x:c r="K345" s="24" t="str">
-        <x:v>Chưa push do thiếu quyền truy cập; CI chưa kích hoạt.</x:v>
+        <x:v>Repo private, xác thực anhthaingd qua Keychain; không force-push. CI chưa kích hoạt; native chưa kiểm.</x:v>
       </x:c>
       <x:c r="L345" s="24" t="str">
         <x:v>Hoàn tất</x:v>
@@ -37044,10 +37044,10 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J346" s="24" t="str">
-        <x:v>README/DOC-065 v1.1; Git root riêng; symlink tương đối; nguồn và ZIP đối chiếu Drive cùng ID.</x:v>
+        <x:v>DOC-065 v1.2; Git root riêng, symlink tương đối; push 1f07065 lên origin/main thành công; Drive cùng ID đọc lại.</x:v>
       </x:c>
       <x:c r="K346" s="24" t="str">
-        <x:v>Chưa push do thiếu quyền truy cập; CI chưa kích hoạt.</x:v>
+        <x:v>Repo private, xác thực anhthaingd qua Keychain; không force-push. CI chưa kích hoạt; native chưa kiểm.</x:v>
       </x:c>
       <x:c r="L346" s="24" t="str">
         <x:v>Hoàn tất</x:v>
@@ -37082,10 +37082,10 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J347" s="24" t="str">
-        <x:v>README/DOC-065 v1.1; Git root riêng; symlink tương đối; nguồn và ZIP đối chiếu Drive cùng ID.</x:v>
+        <x:v>DOC-065 v1.2; Git root riêng, symlink tương đối; push 1f07065 lên origin/main thành công; Drive cùng ID đọc lại.</x:v>
       </x:c>
       <x:c r="K347" s="24" t="str">
-        <x:v>Chưa push do thiếu quyền truy cập; CI chưa kích hoạt.</x:v>
+        <x:v>Repo private, xác thực anhthaingd qua Keychain; không force-push. CI chưa kích hoạt; native chưa kiểm.</x:v>
       </x:c>
       <x:c r="L347" s="24" t="str">
         <x:v>Hoàn tất</x:v>
@@ -37120,10 +37120,10 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J348" s="24" t="str">
-        <x:v>README/DOC-065 v1.1; Git root riêng; symlink tương đối; nguồn và ZIP đối chiếu Drive cùng ID.</x:v>
+        <x:v>DOC-065 v1.2; Git root riêng, symlink tương đối; push 1f07065 lên origin/main thành công; Drive cùng ID đọc lại.</x:v>
       </x:c>
       <x:c r="K348" s="24" t="str">
-        <x:v>Chưa push do thiếu quyền truy cập; CI chưa kích hoạt.</x:v>
+        <x:v>Repo private, xác thực anhthaingd qua Keychain; không force-push. CI chưa kích hoạt; native chưa kiểm.</x:v>
       </x:c>
       <x:c r="L348" s="24" t="str">
         <x:v>Hoàn tất</x:v>
@@ -37146,10 +37146,10 @@
         <x:v>Push code lên repo chủ dự án</x:v>
       </x:c>
       <x:c r="F349" s="24" t="str">
-        <x:v>Chưa cập nhật</x:v>
+        <x:v>Đã cập nhật</x:v>
       </x:c>
       <x:c r="G349" s="24" t="str">
-        <x:v>Không</x:v>
+        <x:v>Có</x:v>
       </x:c>
       <x:c r="H349" s="24" t="str">
         <x:v>Codex</x:v>
@@ -37158,13 +37158,13 @@
         <x:v>46293</x:v>
       </x:c>
       <x:c r="J349" s="24" t="str">
-        <x:v>gh: token invalid; SSH: thainda-0252, Repository not found.</x:v>
+        <x:v>DOC-065 v1.2; Git root riêng, symlink tương đối; push 1f07065 lên origin/main thành công; Drive cùng ID đọc lại.</x:v>
       </x:c>
       <x:c r="K349" s="24" t="str">
-        <x:v>Chờ đăng nhập tài khoản có quyền ghi; chưa kiểm lịch sử remote.</x:v>
+        <x:v>Repo private, xác thực anhthaingd qua Keychain; không force-push. CI chưa kích hoạt; native chưa kiểm.</x:v>
       </x:c>
       <x:c r="L349" s="24" t="str">
-        <x:v>Chưa hoàn tất</x:v>
+        <x:v>Hoàn tất</x:v>
       </x:c>
     </x:row>
     <x:row r="350">
@@ -39134,7 +39134,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e44ff59b75044a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a0c8cfeecb947c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39376,7 +39376,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd0055d4d3c74efa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23100ab2ff084ac0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: organize workspace and add structured logging and quality gates
</commit_message>
<xml_diff>
--- a/docs/project-control/So-quan-ly-tai-lieu.xlsx
+++ b/docs/project-control/So-quan-ly-tai-lieu.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bat dau" sheetId="1" r:id="R8a8a9de6fdf34576"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh muc" sheetId="2" r:id="Re0f21705b2124758"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anh huong" sheetId="3" r:id="Rac27ff509c0f4e40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quyet dinh" sheetId="4" r:id="R41ed8e731b0a4b86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dong bo" sheetId="5" r:id="R1d163119f8ec4369"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quy trinh" sheetId="6" r:id="Ra5ddeda82f274795"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bat dau" sheetId="1" r:id="Rfe4fd5fde09041f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh muc" sheetId="2" r:id="R6f2998d7706d4bff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anh huong" sheetId="3" r:id="R74b817679b1748f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quyet dinh" sheetId="4" r:id="R144fd33092614f35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dong bo" sheetId="5" r:id="R07e4f31a5c484ec1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quy trinh" sheetId="6" r:id="R85834ea87e8c4d61"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -181,7 +181,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="86" name="Tbl1" displayName="Tbl1" ref="A5:L83" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="86" name="Tbl1" displayName="Tbl1" ref="A5:L86" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Mã tài liệu"/>
     <x:tableColumn id="2" name="Tài liệu"/>
@@ -201,7 +201,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="89" name="Tbl2" displayName="Tbl2" ref="A5:F804" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="89" name="Tbl2" displayName="Tbl2" ref="A5:F813" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Mã chức năng"/>
     <x:tableColumn id="2" name="Chức năng"/>
@@ -215,7 +215,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="87" name="Tbl3" displayName="Tbl3" ref="A5:G52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="87" name="Tbl3" displayName="Tbl3" ref="A5:G56" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Mã quyết định"/>
     <x:tableColumn id="2" name="Chủ đề"/>
@@ -230,7 +230,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="88" name="Tbl4" displayName="Tbl4" ref="A5:L349" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="88" name="Tbl4" displayName="Tbl4" ref="A5:L388" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Mã đợt"/>
     <x:tableColumn id="2" name="Quyết định"/>
@@ -489,7 +489,7 @@
     <x:row r="3">
       <x:c r="A3" s="1"/>
       <x:c r="B3" s="1" t="str">
-        <x:v>Dịch vụ quanh bạn — phiên bản 1.31, 28/09/2026</x:v>
+        <x:v>Phiên bản 1.34 · 28/09/2026 · LOGTEST-01: phương án A đã triển khai/kiểm local; native/remoteCI còn thiếu</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>
@@ -511,7 +511,7 @@
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>COUNTA('Danh muc'!A6:A1000)-COUNTIFS('Danh muc'!F6:F1000,"Chưa có")</x:f>
-        <x:v>76</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D5" s="1"/>
       <x:c r="E5" s="1"/>
@@ -537,7 +537,7 @@
       </x:c>
       <x:c r="C7" s="13" t="n">
         <x:f>COUNTA('Dong bo'!A6:A1000)-COUNTIFS('Dong bo'!L6:L1000,"Hoàn tất")-COUNTIFS('Dong bo'!L6:L1000,"Không áp dụng có lý do")</x:f>
-        <x:v>3</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D7" s="1"/>
       <x:c r="E7" s="1"/>
@@ -550,7 +550,7 @@
       </x:c>
       <x:c r="C8" s="13" t="n">
         <x:f>COUNTIFS('Dong bo'!L6:L1000,"Hoàn tất")</x:f>
-        <x:v>316</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="D8" s="1"/>
       <x:c r="E8" s="1"/>
@@ -751,7 +751,7 @@
     <x:hyperlink ref="B14" location="'Quyet dinh'!A1"/>
     <x:hyperlink ref="B15" location="'Dong bo'!A1"/>
     <x:hyperlink ref="B16" location="'Quy trinh'!A1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="Rf358efb959044fde"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="R72a03738674442a4"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -887,7 +887,7 @@
         <x:v>Quản lý hồ sơ</x:v>
       </x:c>
       <x:c r="D6" s="8" t="str">
-        <x:v>v1.31</x:v>
+        <x:v>v1.34</x:v>
       </x:c>
       <x:c r="E6" s="8" t="str">
         <x:v>Sổ quản lý chính</x:v>
@@ -896,7 +896,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G6" s="8" t="str">
-        <x:v>RULE-01</x:v>
+        <x:v>RULE-01; STRUCTURE-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H6" s="9" t="str">
         <x:v>Mở tài liệu</x:v>
@@ -906,7 +906,7 @@
       </x:c>
       <x:c r="J6" s="8" t="str"/>
       <x:c r="K6" s="8" t="str">
-        <x:v>REPO-01: repo private anhthaingd/dich-vu-quanh-ban; push main thành công commit 1f07065. DOC-065 v1.2 và ZIP đối chiếu Drive; CI chưa kích hoạt.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L6" s="10" t="n">
         <x:v>46293</x:v>
@@ -1465,7 +1465,7 @@
         <x:v>Kiến trúc trực quan</x:v>
       </x:c>
       <x:c r="D22" s="8" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.1 / LOGTEST-01</x:v>
       </x:c>
       <x:c r="E22" s="8" t="str">
         <x:v>Bản xuất</x:v>
@@ -1474,7 +1474,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G22" s="8" t="str">
-        <x:v>Quyết định theo chức năng; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Quyết định theo chức năng; IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H22" s="9" t="str">
         <x:v>Mở tài liệu</x:v>
@@ -1486,7 +1486,7 @@
         <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/ui-ux/wireframes/architecture.html</x:v>
       </x:c>
       <x:c r="K22" s="8" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L22" s="10" t="n">
         <x:v>46293</x:v>
@@ -1503,7 +1503,7 @@
         <x:v>Kiến trúc tổng hợp</x:v>
       </x:c>
       <x:c r="D23" s="8" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.1 / LOGTEST-01</x:v>
       </x:c>
       <x:c r="E23" s="8" t="str">
         <x:v>Bản xuất</x:v>
@@ -1512,7 +1512,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G23" s="8" t="str">
-        <x:v>Quyết định theo chức năng; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Quyết định theo chức năng; IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H23" s="9" t="str">
         <x:v>Mở tài liệu</x:v>
@@ -1522,7 +1522,7 @@
       </x:c>
       <x:c r="J23" s="8" t="str"/>
       <x:c r="K23" s="8" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L23" s="10" t="n">
         <x:v>46293</x:v>
@@ -1539,7 +1539,7 @@
         <x:v>Gói nguồn hồ sơ</x:v>
       </x:c>
       <x:c r="D24" s="8" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.1 / LOGTEST-01</x:v>
       </x:c>
       <x:c r="E24" s="8" t="str">
         <x:v>Gói xuất</x:v>
@@ -1548,7 +1548,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G24" s="8" t="str">
-        <x:v>Quyết định theo chức năng; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Quyết định theo chức năng; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H24" s="9" t="str">
         <x:v>Mở tài liệu</x:v>
@@ -1558,7 +1558,7 @@
       </x:c>
       <x:c r="J24" s="8" t="str"/>
       <x:c r="K24" s="8" t="str">
-        <x:v>REPO-01: repo private anhthaingd/dich-vu-quanh-ban; push main thành công commit 1f07065. DOC-065 v1.2 và ZIP đối chiếu Drive; CI chưa kích hoạt.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L24" s="10" t="n">
         <x:v>46293</x:v>
@@ -1948,7 +1948,7 @@
         <x:v>46288</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="38" customHeight="1">
+    <x:row r="36" ht="105" customHeight="1">
       <x:c r="A36" s="8" t="str">
         <x:v>DOC-030</x:v>
       </x:c>
@@ -1959,7 +1959,7 @@
         <x:v>Nguồn kiến trúc</x:v>
       </x:c>
       <x:c r="D36" s="8" t="str">
-        <x:v>v0.1 + 22/09</x:v>
+        <x:v>v0.1.1 / LOGTEST-01</x:v>
       </x:c>
       <x:c r="E36" s="8" t="str">
         <x:v>Nguồn bổ trợ</x:v>
@@ -1968,20 +1968,22 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G36" s="8" t="str">
-        <x:v>Q01; Q02; Q03; Q04</x:v>
+        <x:v>Q01; Q02; Q03; Q04; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H36" s="9" t="str">
-        <x:v>Chưa có</x:v>
+        <x:v>https://drive.google.com/file/d/1QFvCWLng19VPnOoXcCZ2i0PUCsmlexMC/view</x:v>
       </x:c>
       <x:c r="I36" s="9" t="str">
         <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/project-docs/architecture/10-sequence-API.md</x:v>
       </x:c>
-      <x:c r="J36" s="8" t="str"/>
+      <x:c r="J36" s="8" t="str">
+        <x:v>Thành phần trong DOC-018 architecture-source ZIP; không có file Drive riêng</x:v>
+      </x:c>
       <x:c r="K36" s="8" t="str">
-        <x:v>Đồng bộ JOB-01/02 chốt 23/09: tự thuê và việc không tự hết hạn. Tài liệu thiết kế; chưa triển khai sản phẩm.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L36" s="10" t="n">
-        <x:v>46288</x:v>
+        <x:v>46293</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="105" customHeight="1">
@@ -2067,7 +2069,7 @@
         <x:v>Nguồn kiến trúc</x:v>
       </x:c>
       <x:c r="D39" s="8" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.1 / LOGTEST-01</x:v>
       </x:c>
       <x:c r="E39" s="8" t="str">
         <x:v>Nguồn bổ trợ</x:v>
@@ -2076,7 +2078,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G39" s="8" t="str">
-        <x:v>Q01; Q02; Q03; Q04; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Q01; Q02; Q03; Q04; IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H39" s="9" t="str">
         <x:v>https://drive.google.com/file/d/1QFvCWLng19VPnOoXcCZ2i0PUCsmlexMC/view</x:v>
@@ -2086,7 +2088,7 @@
       </x:c>
       <x:c r="J39" s="8" t="str"/>
       <x:c r="K39" s="8" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L39" s="10" t="n">
         <x:v>46293</x:v>
@@ -2245,7 +2247,7 @@
         <x:v>Thiết kế kỹ thuật</x:v>
       </x:c>
       <x:c r="D44" s="8" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.2</x:v>
       </x:c>
       <x:c r="E44" s="8" t="str">
         <x:v>Nguồn thiết kế; chi tiết chờ review</x:v>
@@ -2254,7 +2256,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G44" s="8" t="str">
-        <x:v>Q03; nghiệp vụ đã chốt; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Q03; nghiệp vụ đã chốt; IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H44" s="9" t="str">
         <x:v>https://drive.google.com/file/d/1XtwMHGx2jBE491-E7rCaJHulQ2XrneR5/view?usp=drivesdk</x:v>
@@ -2266,7 +2268,7 @@
         <x:v>Viewer, JSON và ZIP cùng phiên bản</x:v>
       </x:c>
       <x:c r="K44" s="8" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L44" s="10" t="n">
         <x:v>46293</x:v>
@@ -2283,7 +2285,7 @@
         <x:v>Thiết kế kỹ thuật</x:v>
       </x:c>
       <x:c r="D45" s="8" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.2</x:v>
       </x:c>
       <x:c r="E45" s="8" t="str">
         <x:v>Nguồn thiết kế; chi tiết chờ review</x:v>
@@ -2292,7 +2294,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G45" s="8" t="str">
-        <x:v>Q03; nghiệp vụ đã chốt; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Q03; nghiệp vụ đã chốt; IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H45" s="9" t="str">
         <x:v>https://drive.google.com/file/d/1eE5IvNzIMPson4PO2uwqQ9GGEHky_Cp6/view?usp=drivesdk</x:v>
@@ -2304,7 +2306,7 @@
         <x:v>Viewer, JSON và ZIP cùng phiên bản</x:v>
       </x:c>
       <x:c r="K45" s="8" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L45" s="10" t="n">
         <x:v>46293</x:v>
@@ -2321,28 +2323,28 @@
         <x:v>Hồ sơ còn thiếu</x:v>
       </x:c>
       <x:c r="D46" s="8" t="str">
-        <x:v>v0.1 local</x:v>
+        <x:v>v1.0 local / DOC-071</x:v>
       </x:c>
       <x:c r="E46" s="8" t="str">
-        <x:v>Runbook local/CI trong DOC-065; deploy/backup production chưa có</x:v>
+        <x:v>Runbook local/log/test/CI đã có; deploy/backup production chưa hoàn thành</x:v>
       </x:c>
       <x:c r="F46" s="8" t="str">
         <x:v>Cần đồng bộ</x:v>
       </x:c>
       <x:c r="G46" s="8" t="str">
-        <x:v>IMPLEMENT-01; TECH-01</x:v>
+        <x:v>IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H46" s="9" t="str">
-        <x:v>https://drive.google.com/file/d/1JjfKtYYgYGHlLSZCKZ21hqWiscQxoFpT/view</x:v>
+        <x:v>https://drive.google.com/file/d/1m7nrDRbwKj7HPH3TQoWUIsT4zSKn_ldK/view</x:v>
       </x:c>
       <x:c r="I46" s="9" t="str">
-        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/implementation/dot-1.md</x:v>
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/implementation/logging-testing.md</x:v>
       </x:c>
       <x:c r="J46" s="8" t="str">
-        <x:v>infra/compose.yaml; infra/ci/github-actions.yml</x:v>
+        <x:v>DOC-065; DOC-071; .github/workflows/quality.yml</x:v>
       </x:c>
       <x:c r="K46" s="8" t="str">
-        <x:v>Đã có hướng dẫn dựng/dừng/local/test/CI template. Production deploy/backup và remote CI ngoài Đợt 1, chưa hoàn thành PLAN-004 toàn bộ.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. PLAN-004 còn native/remote CI, deploy/backup production ngoài phạm vi.</x:v>
       </x:c>
       <x:c r="L46" s="10" t="n">
         <x:v>46293</x:v>
@@ -2465,7 +2467,7 @@
         <x:v>Thiết kế kỹ thuật</x:v>
       </x:c>
       <x:c r="D50" s="8" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.2</x:v>
       </x:c>
       <x:c r="E50" s="8" t="str">
         <x:v>Nguồn thiết kế; chi tiết chờ review</x:v>
@@ -2474,7 +2476,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G50" s="8" t="str">
-        <x:v>Q03; nghiệp vụ đã chốt; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Q03; nghiệp vụ đã chốt; IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H50" s="9" t="str">
         <x:v>https://drive.google.com/file/d/1pJieipNm0-CL8furUSqQFYjoaGNa4Kjo/view?usp=drivesdk</x:v>
@@ -2486,7 +2488,7 @@
         <x:v>Viewer, JSON và ZIP cùng phiên bản</x:v>
       </x:c>
       <x:c r="K50" s="8" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L50" s="10" t="n">
         <x:v>46293</x:v>
@@ -2539,7 +2541,7 @@
         <x:v>Thiết kế kỹ thuật</x:v>
       </x:c>
       <x:c r="D52" s="20" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.2</x:v>
       </x:c>
       <x:c r="E52" s="20" t="str">
         <x:v>Nguồn / bản tra cứu</x:v>
@@ -2548,7 +2550,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G52" s="20" t="str">
-        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H52" s="20" t="str">
         <x:v>https://drive.google.com/file/d/15EgWqgGgTsG11r9BBF7boNAL0jY2Wi_a/view?usp=drivesdk</x:v>
@@ -2560,7 +2562,7 @@
         <x:v>Bản trên Drive</x:v>
       </x:c>
       <x:c r="K52" s="20" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L52" s="21" t="n">
         <x:v>46293</x:v>
@@ -2615,7 +2617,7 @@
         <x:v>Thiết kế kỹ thuật</x:v>
       </x:c>
       <x:c r="D54" s="20" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.2</x:v>
       </x:c>
       <x:c r="E54" s="20" t="str">
         <x:v>Nguồn / bản tra cứu</x:v>
@@ -2624,7 +2626,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G54" s="20" t="str">
-        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H54" s="20" t="str">
         <x:v>https://drive.google.com/file/d/1aO9fJeNj78rOpQwhgWCeiWJSnRz5FXl6/view?usp=drivesdk</x:v>
@@ -2636,7 +2638,7 @@
         <x:v>Bản trên Drive</x:v>
       </x:c>
       <x:c r="K54" s="20" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L54" s="21" t="n">
         <x:v>46293</x:v>
@@ -2653,7 +2655,7 @@
         <x:v>Thiết kế kỹ thuật</x:v>
       </x:c>
       <x:c r="D55" s="20" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.1 / LOGTEST-01</x:v>
       </x:c>
       <x:c r="E55" s="20" t="str">
         <x:v>Gói hiện hành</x:v>
@@ -2662,7 +2664,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G55" s="20" t="str">
-        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H55" s="20" t="str">
         <x:v>https://drive.google.com/file/d/18z-ReFxGP-RhX5_cOVTidcHJJGFfB48D/view?usp=drivesdk</x:v>
@@ -2674,7 +2676,7 @@
         <x:v>Bản trên Drive</x:v>
       </x:c>
       <x:c r="K55" s="20" t="str">
-        <x:v>REPO-01: repo private anhthaingd/dich-vu-quanh-ban; push main thành công commit 1f07065. DOC-065 v1.2 và ZIP đối chiếu Drive; CI chưa kích hoạt.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L55" s="21" t="n">
         <x:v>46293</x:v>
@@ -2691,7 +2693,7 @@
         <x:v>Thiết kế kỹ thuật</x:v>
       </x:c>
       <x:c r="D56" s="20" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.2</x:v>
       </x:c>
       <x:c r="E56" s="20" t="str">
         <x:v>Nguồn / bản tra cứu</x:v>
@@ -2700,7 +2702,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G56" s="20" t="str">
-        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H56" s="20" t="str">
         <x:v>https://drive.google.com/file/d/18z-ReFxGP-RhX5_cOVTidcHJJGFfB48D/view?usp=drivesdk</x:v>
@@ -2712,7 +2714,7 @@
         <x:v>Thành phần trong ZIP trên Drive</x:v>
       </x:c>
       <x:c r="K56" s="20" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L56" s="21" t="n">
         <x:v>46293</x:v>
@@ -2767,7 +2769,7 @@
         <x:v>Thiết kế kỹ thuật</x:v>
       </x:c>
       <x:c r="D58" s="20" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.2</x:v>
       </x:c>
       <x:c r="E58" s="20" t="str">
         <x:v>Nguồn / bản tra cứu</x:v>
@@ -2776,7 +2778,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G58" s="20" t="str">
-        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H58" s="20" t="str">
         <x:v>https://drive.google.com/file/d/18z-ReFxGP-RhX5_cOVTidcHJJGFfB48D/view?usp=drivesdk</x:v>
@@ -2788,7 +2790,7 @@
         <x:v>Thành phần trong ZIP trên Drive</x:v>
       </x:c>
       <x:c r="K58" s="20" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L58" s="21" t="n">
         <x:v>46293</x:v>
@@ -2843,7 +2845,7 @@
         <x:v>Thiết kế kỹ thuật</x:v>
       </x:c>
       <x:c r="D60" s="20" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.2</x:v>
       </x:c>
       <x:c r="E60" s="20" t="str">
         <x:v>Nguồn / bản tra cứu</x:v>
@@ -2852,7 +2854,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G60" s="20" t="str">
-        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H60" s="20" t="str">
         <x:v>https://drive.google.com/file/d/18z-ReFxGP-RhX5_cOVTidcHJJGFfB48D/view?usp=drivesdk</x:v>
@@ -2864,7 +2866,7 @@
         <x:v>Thành phần trong ZIP trên Drive</x:v>
       </x:c>
       <x:c r="K60" s="20" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L60" s="21" t="n">
         <x:v>46293</x:v>
@@ -2881,7 +2883,7 @@
         <x:v>Thiết kế kỹ thuật</x:v>
       </x:c>
       <x:c r="D61" s="20" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.2</x:v>
       </x:c>
       <x:c r="E61" s="20" t="str">
         <x:v>Nguồn / bản tra cứu</x:v>
@@ -2890,7 +2892,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G61" s="20" t="str">
-        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H61" s="20" t="str">
         <x:v>https://drive.google.com/file/d/18z-ReFxGP-RhX5_cOVTidcHJJGFfB48D/view?usp=drivesdk</x:v>
@@ -2902,7 +2904,7 @@
         <x:v>Thành phần trong ZIP trên Drive</x:v>
       </x:c>
       <x:c r="K61" s="20" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L61" s="21" t="n">
         <x:v>46293</x:v>
@@ -2919,7 +2921,7 @@
         <x:v>Thiết kế kỹ thuật</x:v>
       </x:c>
       <x:c r="D62" s="20" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.2</x:v>
       </x:c>
       <x:c r="E62" s="20" t="str">
         <x:v>Nguồn / bản tra cứu</x:v>
@@ -2928,7 +2930,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G62" s="20" t="str">
-        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H62" s="20" t="str">
         <x:v>https://drive.google.com/file/d/18z-ReFxGP-RhX5_cOVTidcHJJGFfB48D/view?usp=drivesdk</x:v>
@@ -2940,7 +2942,7 @@
         <x:v>Thành phần trong ZIP trên Drive</x:v>
       </x:c>
       <x:c r="K62" s="20" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L62" s="21" t="n">
         <x:v>46293</x:v>
@@ -2957,7 +2959,7 @@
         <x:v>Thiết kế kỹ thuật</x:v>
       </x:c>
       <x:c r="D63" s="20" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+        <x:v>v0.1.2</x:v>
       </x:c>
       <x:c r="E63" s="20" t="str">
         <x:v>Nguồn / bản tra cứu</x:v>
@@ -2966,7 +2968,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G63" s="20" t="str">
-        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H63" s="20" t="str">
         <x:v>https://drive.google.com/file/d/18z-ReFxGP-RhX5_cOVTidcHJJGFfB48D/view?usp=drivesdk</x:v>
@@ -2978,7 +2980,7 @@
         <x:v>Thành phần trong ZIP trên Drive</x:v>
       </x:c>
       <x:c r="K63" s="20" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L63" s="21" t="n">
         <x:v>46293</x:v>
@@ -3185,7 +3187,7 @@
         <x:v>Quản lý dự án</x:v>
       </x:c>
       <x:c r="D69" s="24" t="str">
-        <x:v>v0.16 / Đợt 1</x:v>
+        <x:v>v0.3 / LOGTEST-01</x:v>
       </x:c>
       <x:c r="E69" s="24" t="str">
         <x:v>Hướng dẫn hiện hành</x:v>
@@ -3194,7 +3196,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G69" s="24" t="str">
-        <x:v>ORG-01/UI-21; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>ORG-01/UI-21; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H69" s="24" t="str">
         <x:v>https://drive.google.com/file/d/18z-ReFxGP-RhX5_cOVTidcHJJGFfB48D/view</x:v>
@@ -3206,7 +3208,7 @@
         <x:v>React/Storybook; UI-UX-v0.19.zip</x:v>
       </x:c>
       <x:c r="K69" s="24" t="str">
-        <x:v>REPO-01: repo private anhthaingd/dich-vu-quanh-ban; push main thành công commit 1f07065. DOC-065 v1.2 và ZIP đối chiếu Drive; CI chưa kích hoạt.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L69" s="24" t="n">
         <x:v>46293</x:v>
@@ -3565,7 +3567,7 @@
         <x:v>Bàn giao triển khai</x:v>
       </x:c>
       <x:c r="D79" s="24" t="str">
-        <x:v>v1.1</x:v>
+        <x:v>v1.3</x:v>
       </x:c>
       <x:c r="E79" s="24" t="str">
         <x:v>Prompt bàn giao; đã kích hoạt Đợt 1, hiện trạng ở DOC-065</x:v>
@@ -3574,7 +3576,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G79" s="24" t="str">
-        <x:v>HANDOFF-01; IMPLEMENT-01; TECH-01</x:v>
+        <x:v>HANDOFF-01; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H79" s="24" t="str">
         <x:v>https://drive.google.com/file/d/1WnXV2mRTBnYePYztiKJvvfS6tCAjeTrW/view</x:v>
@@ -3586,7 +3588,7 @@
         <x:v>Markdown nguồn local và Drive cùng nội dung</x:v>
       </x:c>
       <x:c r="K79" s="24" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L79" s="24" t="n">
         <x:v>46293</x:v>
@@ -3603,7 +3605,7 @@
         <x:v>Triển khai</x:v>
       </x:c>
       <x:c r="D80" s="24" t="str">
-        <x:v>v1.2</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="E80" s="24" t="str">
         <x:v>Nguồn hiện trạng và kết quả local</x:v>
@@ -3612,7 +3614,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G80" s="24" t="str">
-        <x:v>IMPLEMENT-01; TECH-01</x:v>
+        <x:v>IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H80" s="24" t="str">
         <x:v>https://drive.google.com/file/d/1JjfKtYYgYGHlLSZCKZ21hqWiscQxoFpT/view</x:v>
@@ -3624,7 +3626,7 @@
         <x:v>docs/implementation/evidence; technical-design ZIP</x:v>
       </x:c>
       <x:c r="K80" s="24" t="str">
-        <x:v>REPO-01: repo private anhthaingd/dich-vu-quanh-ban; push main thành công commit 1f07065. DOC-065 v1.2 và ZIP đối chiếu Drive; CI chưa kích hoạt.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L80" s="24" t="n">
         <x:v>46293</x:v>
@@ -3641,7 +3643,7 @@
         <x:v>Kiến trúc</x:v>
       </x:c>
       <x:c r="D81" s="24" t="str">
-        <x:v>v1.0</x:v>
+        <x:v>v1.2</x:v>
       </x:c>
       <x:c r="E81" s="24" t="str">
         <x:v>Quyết định kỹ thuật trong phạm vi được giao</x:v>
@@ -3650,7 +3652,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G81" s="24" t="str">
-        <x:v>IMPLEMENT-01; TECH-01</x:v>
+        <x:v>IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01</x:v>
       </x:c>
       <x:c r="H81" s="24" t="str">
         <x:v>https://drive.google.com/file/d/13DeYIW4Nt-qA1kw7K_NXInowM5huLNH6/view</x:v>
@@ -3662,7 +3664,7 @@
         <x:v>technical-design ZIP</x:v>
       </x:c>
       <x:c r="K81" s="24" t="str">
-        <x:v>Không phê duyệt toàn bộ roadmap hoặc production.</x:v>
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
       </x:c>
       <x:c r="L81" s="24" t="n">
         <x:v>46293</x:v>
@@ -3739,6 +3741,120 @@
         <x:v>Giữ nguyên snapshot cũ; không dùng làm nguồn hiện hành.</x:v>
       </x:c>
       <x:c r="L83" s="24"/>
+    </x:row>
+    <x:row r="84" ht="105" customHeight="1">
+      <x:c r="A84" s="24" t="str">
+        <x:v>DOC-069</x:v>
+      </x:c>
+      <x:c r="B84" s="24" t="str">
+        <x:v>Thiết kế log và kiểm thử nền tảng</x:v>
+      </x:c>
+      <x:c r="C84" s="24" t="str">
+        <x:v>Thiết kế kỹ thuật</x:v>
+      </x:c>
+      <x:c r="D84" s="24" t="str">
+        <x:v>v0.3</x:v>
+      </x:c>
+      <x:c r="E84" s="24" t="str">
+        <x:v>Thiết kế đã duyệt; triển khai local theo DOC-071</x:v>
+      </x:c>
+      <x:c r="F84" s="24" t="str">
+        <x:v>Mới nhất</x:v>
+      </x:c>
+      <x:c r="G84" s="24" t="str">
+        <x:v>LOGTEST-REQ-01; LOGTEST-DESIGN-01; STRUCTURE-01; LOGTEST-01</x:v>
+      </x:c>
+      <x:c r="H84" s="24" t="str">
+        <x:v>https://drive.google.com/file/d/1cJtBn_wcwXd6GAAy752RMWrl9cUaqaf1/view</x:v>
+      </x:c>
+      <x:c r="I84" s="24" t="str">
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/specs/2026-09-28-logging-testing-design.md</x:v>
+      </x:c>
+      <x:c r="J84" s="24" t="str">
+        <x:v>Nguồn Markdown, Drive cùng ID; kèm hai ZIP hiện hành</x:v>
+      </x:c>
+      <x:c r="K84" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
+      </x:c>
+      <x:c r="L84" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="105" customHeight="1">
+      <x:c r="A85" s="24" t="str">
+        <x:v>DOC-070</x:v>
+      </x:c>
+      <x:c r="B85" s="24" t="str">
+        <x:v>Khung cấu trúc dự án</x:v>
+      </x:c>
+      <x:c r="C85" s="24" t="str">
+        <x:v>Kiến trúc / triển khai</x:v>
+      </x:c>
+      <x:c r="D85" s="24" t="str">
+        <x:v>v1.1</x:v>
+      </x:c>
+      <x:c r="E85" s="24" t="str">
+        <x:v>Bản đồ code, trách nhiệm folder và quy tắc mở rộng</x:v>
+      </x:c>
+      <x:c r="F85" s="24" t="str">
+        <x:v>Mới nhất</x:v>
+      </x:c>
+      <x:c r="G85" s="24" t="str">
+        <x:v>STRUCTURE-01; LOGTEST-DESIGN-01; LOGTEST-01</x:v>
+      </x:c>
+      <x:c r="H85" s="24" t="str">
+        <x:v>https://drive.google.com/file/d/1pWijvZgP7U3mpjq5Wualaa1mdPCDk_Ge/view</x:v>
+      </x:c>
+      <x:c r="I85" s="24" t="str">
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/implementation/project-structure.md</x:v>
+      </x:c>
+      <x:c r="J85" s="24" t="str">
+        <x:v>README; hai ZIP kỹ thuật hiện hành</x:v>
+      </x:c>
+      <x:c r="K85" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
+      </x:c>
+      <x:c r="L85" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="130" customHeight="1">
+      <x:c r="A86" s="24" t="str">
+        <x:v>DOC-071</x:v>
+      </x:c>
+      <x:c r="B86" s="24" t="str">
+        <x:v>Vận hành log và kiểm thử phương án A</x:v>
+      </x:c>
+      <x:c r="C86" s="24" t="str">
+        <x:v>Triển khai / vận hành</x:v>
+      </x:c>
+      <x:c r="D86" s="24" t="str">
+        <x:v>v1.0</x:v>
+      </x:c>
+      <x:c r="E86" s="24" t="str">
+        <x:v>Runbook và bằng chứng kiểm local; giới hạn native/remoteCI</x:v>
+      </x:c>
+      <x:c r="F86" s="24" t="str">
+        <x:v>Mới nhất</x:v>
+      </x:c>
+      <x:c r="G86" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="H86" s="24" t="str">
+        <x:v>https://drive.google.com/file/d/1m7nrDRbwKj7HPH3TQoWUIsT4zSKn_ldK/view</x:v>
+      </x:c>
+      <x:c r="I86" s="24" t="str">
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/implementation/logging-testing.md</x:v>
+      </x:c>
+      <x:c r="J86" s="24" t="str">
+        <x:v>Hai ZIP hiện hành; coverage/test-results local ignored</x:v>
+      </x:c>
+      <x:c r="K86" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
+      </x:c>
+      <x:c r="L86" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F6:F1000">
@@ -3752,81 +3868,81 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="R3bfb8b542ba948bd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R90e8f8cadd5a4a31"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="Rff13854e95ef486f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="Raa40edc5153849e0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="Re31d90a295724192"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="R8b05a5c0cac24c29"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="Rbd4da0d774294f9e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R2797de5ed5664496"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="R8327b7db10e54f58"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="Rfb181db4e9e8482e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="Re13a7670c9f54f8a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="R3ceb301323964d3e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="R6bf663f1e6134a74"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="R073c5a54f0da49c6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="Rf317f75b58f0467d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="R5673a7b3d9a34b26"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="R09d211447ae44e43"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="Rab448c5834e144ea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="Rdb22b4c057f54e1e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="R1e1c8ebc10d742c3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="Rcf069d82cf564852"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="R12cecd4c176c4ec2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="R99a41aae61714cb6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="Ra4122904c9284635"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="Rd278aedd602749ce"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="Rf6f6f1a7010948b1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="R698c1015bf08450e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="R3861919cee164503"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="R602be373e7aa4a8c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="Rab8dd8c5ad884ae8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="Rfbe536ad88694a4f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="Rdc6aab794baf4f43"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R811781f3eb2c437d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="Rac0aaa5910bb4e9a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="R436c11a8d0e84b29"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="Rdc6663a48a1045ca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="Rb4df92c73d5346c9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="R5e2cd171d5854f41"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="R2d1102e892dd496b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="R88e04be7926a40c8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="R89bd24ccdb394e91"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="R82eb2fd25ae545ab"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="Ra6be5fba70bc4803"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="R78f2d58d8efb4570"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="Rbaea0ec0e42e4d8e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="R9047fa5f0d9b4175"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="R8a72e1092b964f96"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="R814b96e28a484509"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="R9969d724e0924304"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="R35035a9c17b94049"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="R966de9f703e4406e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="R513f06d1b4394c2d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="Ra94f6ac1f8da4565"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="R1ba44f791d56487a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="Rbb0bb346fdd74c3a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="R71ff83ce6e3d4baa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="Rff8a1b1817e44218"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="R09370944a69c4014"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="Ra1d31eb104e84c88"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="Rcfd04fdc6bc445de"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="R4226b2934c4a42a9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="R5616c754bdc04b28"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="R53d26bc0a5884dbc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="Rde58ebc803d74ebc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="R10c25084ff214c9b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="Raae97f50fc694b7b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="R8ec99cb898fe4148"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="R0605d6bcb5be48b1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="R8500af7296e54e07"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="Ra48dadf901b54365"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="R5d00e157ef7c4b89"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="R0e0ea06ec95c4239"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R2993c2dbee8e4715"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="Rcf90c67a09ee4043"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="R232f18a296134ce7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="R4241635c91b94b6d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="R9aa1f91a70d94b77"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="Rb2bf539e90b1427e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R9190cd05b2154498"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="Rf487ec837be54c5f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="Rd98212fe91c34289"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="R893c6c418c9d40a7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="Re54f25b39d334383"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="R75f4ab2ca0c744c7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="R5c4ce04a77584ee5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="R45321951c6a94376"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="R31364b6ccb3f4ad5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="Rf8138b5102304ca5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="R5f4ff2cc4cb740cd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="R4868f0de14e04889"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="Rb9bf8ce3dace43cb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="Reb618d44f0b94542"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="Rb684c77e2a454938"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="R921917e0de114691"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="R39eb590dd3f940d0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="Rc6432f6c91684f0b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="R774b7a5197fa4410"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="R5c10ff1bfb2a43d4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="Rb8a3e5a3aebb49b4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="Rd21c7647f4be48e8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R32907f91bb274c21"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="Rb9b190d707f84dbd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="R22442571d2d44659"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R25da1f2869254ef2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R02f17c9b37604197"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="R55e26d7c82ae438c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="Rf7e92801cb7b4645"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="Rd00f54816bc94f2b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="R60a0885ad05d407d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="Rdd06caccbb294bc0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="R8351a58771074bf5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="R6291422096e84392"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="Rcbd18d5341694662"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="R40d934ed533d4f80"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="Rb70ea6e1d3e442f8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="R497efdc7f828445c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="Rd00a986aff2448ca"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="Ra628313e15a84dcc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="R5d98a45f99f7404c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="R6e867fb3b67e4414"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="R69b5807c1ea84587"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="Ra19e1489d6a24bfa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="R100d05fa27d64085"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="R6568905699e84bf2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="Re24ebcf213874499"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="Rfb3d5a6e04274816"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="R43ee00299f6f4da9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="R07aa0f19dd374a3f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="R3b11d0160e93489c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="Reaf8da3b54ca408f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="R62cbbae323e64842"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="Rf2e06fb4e3cb4173"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="R2248801f36934993"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="R5a128e7800c642e1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="R546b11a001ff40e5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="R7d26d799820c42c6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="Ra68e7370228f4ba2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="R173e5f8156c84d37"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="Rd15ff254ae2a4c1b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="Rc3e2fe4cbef24c31"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="Rddace0a9895149bd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="R4784433d490a459c"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9625b3821294854"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bdb21b069874527"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19879,10 +19995,190 @@
         <x:v>Đối chiếu code/migration/test, DOC-065/066, technical JSON/MD/viewer/ZIP và registry</x:v>
       </x:c>
     </x:row>
+    <x:row r="805" ht="90" customHeight="1">
+      <x:c r="A805" s="24" t="str">
+        <x:v>F18</x:v>
+      </x:c>
+      <x:c r="B805" s="24" t="str">
+        <x:v>Log / test / CI / bằng chứng</x:v>
+      </x:c>
+      <x:c r="C805" s="24" t="str">
+        <x:v>DOC-069</x:v>
+      </x:c>
+      <x:c r="D805" s="24" t="str">
+        <x:v>LOGTEST-REQ-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="E805" s="24" t="str">
+        <x:v>Khi duyệt hoặc sửa thiết kế log/test</x:v>
+      </x:c>
+      <x:c r="F805" s="24" t="str">
+        <x:v>Phương án A đã triển khai local (DOC-071); khi sửa log/test cập nhật contract/QA/ADR/runbook/source/export/registry.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="806" ht="90" customHeight="1">
+      <x:c r="A806" s="24" t="str">
+        <x:v>F20</x:v>
+      </x:c>
+      <x:c r="B806" s="24" t="str">
+        <x:v>Log / test / CI / bằng chứng</x:v>
+      </x:c>
+      <x:c r="C806" s="24" t="str">
+        <x:v>DOC-069</x:v>
+      </x:c>
+      <x:c r="D806" s="24" t="str">
+        <x:v>LOGTEST-REQ-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="E806" s="24" t="str">
+        <x:v>Khi duyệt hoặc sửa thiết kế log/test</x:v>
+      </x:c>
+      <x:c r="F806" s="24" t="str">
+        <x:v>Phương án A đã triển khai local (DOC-071); khi sửa log/test cập nhật contract/QA/ADR/runbook/source/export/registry.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="807" ht="72" customHeight="1">
+      <x:c r="A807" s="24" t="str">
+        <x:v>F17</x:v>
+      </x:c>
+      <x:c r="B807" s="24" t="str">
+        <x:v>Khung source và hướng dẫn phát triển</x:v>
+      </x:c>
+      <x:c r="C807" s="24" t="str">
+        <x:v>DOC-070</x:v>
+      </x:c>
+      <x:c r="D807" s="24" t="str">
+        <x:v>STRUCTURE-01</x:v>
+      </x:c>
+      <x:c r="E807" s="24" t="str">
+        <x:v>Khi đổi vị trí code/module/workspace</x:v>
+      </x:c>
+      <x:c r="F807" s="24" t="str">
+        <x:v>Đối chiếu imports/scripts/build/test, README, runbook, ADR, handoff, ZIP và registry</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="808" ht="72" customHeight="1">
+      <x:c r="A808" s="24" t="str">
+        <x:v>F18</x:v>
+      </x:c>
+      <x:c r="B808" s="24" t="str">
+        <x:v>Khung source và hướng dẫn phát triển</x:v>
+      </x:c>
+      <x:c r="C808" s="24" t="str">
+        <x:v>DOC-070</x:v>
+      </x:c>
+      <x:c r="D808" s="24" t="str">
+        <x:v>STRUCTURE-01</x:v>
+      </x:c>
+      <x:c r="E808" s="24" t="str">
+        <x:v>Khi đổi vị trí code/module/workspace</x:v>
+      </x:c>
+      <x:c r="F808" s="24" t="str">
+        <x:v>Đối chiếu imports/scripts/build/test, README, runbook, ADR, handoff, ZIP và registry</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="809" ht="72" customHeight="1">
+      <x:c r="A809" s="24" t="str">
+        <x:v>F20</x:v>
+      </x:c>
+      <x:c r="B809" s="24" t="str">
+        <x:v>Khung source và hướng dẫn phát triển</x:v>
+      </x:c>
+      <x:c r="C809" s="24" t="str">
+        <x:v>DOC-070</x:v>
+      </x:c>
+      <x:c r="D809" s="24" t="str">
+        <x:v>STRUCTURE-01</x:v>
+      </x:c>
+      <x:c r="E809" s="24" t="str">
+        <x:v>Khi đổi vị trí code/module/workspace</x:v>
+      </x:c>
+      <x:c r="F809" s="24" t="str">
+        <x:v>Đối chiếu imports/scripts/build/test, README, runbook, ADR, handoff, ZIP và registry</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="810" ht="75" customHeight="1">
+      <x:c r="A810" s="24" t="str">
+        <x:v>F02</x:v>
+      </x:c>
+      <x:c r="B810" s="24" t="str">
+        <x:v>Log/test/correlation/CI</x:v>
+      </x:c>
+      <x:c r="C810" s="24" t="str">
+        <x:v>DOC-071</x:v>
+      </x:c>
+      <x:c r="D810" s="24" t="str">
+        <x:v>LOGTEST-01</x:v>
+      </x:c>
+      <x:c r="E810" s="24" t="str">
+        <x:v>Khi đổi log/error/test hoặc cách vận hành</x:v>
+      </x:c>
+      <x:c r="F810" s="24" t="str">
+        <x:v>Đối chiếu source/test/reports, OpenAPI/QA/RTM/backlog, DOC-065/066/069/070 và ZIP/Drive</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="811" ht="75" customHeight="1">
+      <x:c r="A811" s="24" t="str">
+        <x:v>F17</x:v>
+      </x:c>
+      <x:c r="B811" s="24" t="str">
+        <x:v>Log/test/correlation/CI</x:v>
+      </x:c>
+      <x:c r="C811" s="24" t="str">
+        <x:v>DOC-071</x:v>
+      </x:c>
+      <x:c r="D811" s="24" t="str">
+        <x:v>LOGTEST-01</x:v>
+      </x:c>
+      <x:c r="E811" s="24" t="str">
+        <x:v>Khi đổi log/error/test hoặc cách vận hành</x:v>
+      </x:c>
+      <x:c r="F811" s="24" t="str">
+        <x:v>Đối chiếu source/test/reports, OpenAPI/QA/RTM/backlog, DOC-065/066/069/070 và ZIP/Drive</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="812" ht="75" customHeight="1">
+      <x:c r="A812" s="24" t="str">
+        <x:v>F18</x:v>
+      </x:c>
+      <x:c r="B812" s="24" t="str">
+        <x:v>Log/test/correlation/CI</x:v>
+      </x:c>
+      <x:c r="C812" s="24" t="str">
+        <x:v>DOC-071</x:v>
+      </x:c>
+      <x:c r="D812" s="24" t="str">
+        <x:v>LOGTEST-01</x:v>
+      </x:c>
+      <x:c r="E812" s="24" t="str">
+        <x:v>Khi đổi log/error/test hoặc cách vận hành</x:v>
+      </x:c>
+      <x:c r="F812" s="24" t="str">
+        <x:v>Đối chiếu source/test/reports, OpenAPI/QA/RTM/backlog, DOC-065/066/069/070 và ZIP/Drive</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="813" ht="75" customHeight="1">
+      <x:c r="A813" s="24" t="str">
+        <x:v>F20</x:v>
+      </x:c>
+      <x:c r="B813" s="24" t="str">
+        <x:v>Log/test/correlation/CI</x:v>
+      </x:c>
+      <x:c r="C813" s="24" t="str">
+        <x:v>DOC-071</x:v>
+      </x:c>
+      <x:c r="D813" s="24" t="str">
+        <x:v>LOGTEST-01</x:v>
+      </x:c>
+      <x:c r="E813" s="24" t="str">
+        <x:v>Khi đổi log/error/test hoặc cách vận hành</x:v>
+      </x:c>
+      <x:c r="F813" s="24" t="str">
+        <x:v>Đối chiếu source/test/reports, OpenAPI/QA/RTM/backlog, DOC-065/066/069/070 và ZIP/Drive</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28b146e11e994690"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd945b1a595a4fe6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21024,17 +21320,97 @@
         <x:v>46293</x:v>
       </x:c>
     </x:row>
-    <x:row r="53">
-      <x:c r="G53" s="11"/>
-    </x:row>
-    <x:row r="54">
-      <x:c r="G54" s="11"/>
-    </x:row>
-    <x:row r="55">
-      <x:c r="G55" s="11"/>
-    </x:row>
-    <x:row r="56">
-      <x:c r="G56" s="11"/>
+    <x:row r="53" ht="100" customHeight="1">
+      <x:c r="A53" s="24" t="str">
+        <x:v>LOGTEST-REQ-01</x:v>
+      </x:c>
+      <x:c r="B53" s="24" t="str">
+        <x:v>Làm log/test chỉn chu từ dự án thực tế</x:v>
+      </x:c>
+      <x:c r="C53" s="24" t="str">
+        <x:v>Đã chốt</x:v>
+      </x:c>
+      <x:c r="D53" s="24" t="str">
+        <x:v>Chủ dự án yêu cầu tham khảo bộ log/test của các dự án nổi tiếng để áp dụng cho dự án. Không mở production/tiền thật.</x:v>
+      </x:c>
+      <x:c r="E53" s="24" t="str">
+        <x:v>F18/F20</x:v>
+      </x:c>
+      <x:c r="F53" s="24" t="str">
+        <x:v>Yêu cầu trực tiếp 28/09/2026; DOC-069 v0.1</x:v>
+      </x:c>
+      <x:c r="G53" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="100" customHeight="1">
+      <x:c r="A54" s="24" t="str">
+        <x:v>LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="B54" s="24" t="str">
+        <x:v>Thiết kế phương án A log/test</x:v>
+      </x:c>
+      <x:c r="C54" s="24" t="str">
+        <x:v>Đã chốt</x:v>
+      </x:c>
+      <x:c r="D54" s="24" t="str">
+        <x:v>Chủ dự án duyệt phương án A theo DOC-069 v0.2. Ưu tiên hoàn thiện khung STRUCTURE-01 trước rồi triển khai log/test; chưa production hoặc tiền thật.</x:v>
+      </x:c>
+      <x:c r="E54" s="24" t="str">
+        <x:v>F18/F20</x:v>
+      </x:c>
+      <x:c r="F54" s="24" t="str">
+        <x:v>DOC-069 v0.3 đã duyệt; LOGTEST-01 triển khai/kiểm local tại DOC-071 v1.0; native/remoteCI chưa nghiệm thu</x:v>
+      </x:c>
+      <x:c r="G54" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="125" customHeight="1">
+      <x:c r="A55" s="24" t="str">
+        <x:v>STRUCTURE-01</x:v>
+      </x:c>
+      <x:c r="B55" s="24" t="str">
+        <x:v>Hoàn thiện khung trước chức năng</x:v>
+      </x:c>
+      <x:c r="C55" s="24" t="str">
+        <x:v>Đã chốt</x:v>
+      </x:c>
+      <x:c r="D55" s="24" t="str">
+        <x:v>Tổ chức mobile theo feature, API theo module; dành chỗ các miền và shared packages bằng .gitkeep, tách scripts/test/infra. Giữ nghiệp vụ danh mục hiện hành; chưa mở production/tiền thật.</x:v>
+      </x:c>
+      <x:c r="E55" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="F55" s="24" t="str">
+        <x:v>Chủ dự án yêu cầu trực tiếp 28/09/2026; DOC-070 v1.0; tham khảo Expo/Mattermost/Immich/Vendure.</x:v>
+      </x:c>
+      <x:c r="G55" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="115" customHeight="1">
+      <x:c r="A56" s="24" t="str">
+        <x:v>LOGTEST-01</x:v>
+      </x:c>
+      <x:c r="B56" s="24" t="str">
+        <x:v>Triển khai log/test phương án A</x:v>
+      </x:c>
+      <x:c r="C56" s="24" t="str">
+        <x:v>Đã chốt</x:v>
+      </x:c>
+      <x:c r="D56" s="24" t="str">
+        <x:v>Chủ dự án giao triển khai phương án A đã duyệt sau khung STRUCTURE-01. Đã kiểm local; native BLOCKED và remoteCI chưa chạy, không production/tiền thật/telemetry ngoài.</x:v>
+      </x:c>
+      <x:c r="E56" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="F56" s="24" t="str">
+        <x:v>Yêu cầu trực tiếp28/09/2026; DOC-069 v0.3 và DOC-071 v1.0; không commit/push mới.</x:v>
+      </x:c>
+      <x:c r="G56" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="G57" s="11"/>
@@ -23871,7 +24247,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98c1015395ee4a79"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c0bb58d82ef44fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37167,122 +37543,1487 @@
         <x:v>Hoàn tất</x:v>
       </x:c>
     </x:row>
-    <x:row r="350">
-      <x:c r="I350" s="11"/>
-    </x:row>
-    <x:row r="351">
-      <x:c r="I351" s="11"/>
-    </x:row>
-    <x:row r="352">
-      <x:c r="I352" s="11"/>
-    </x:row>
-    <x:row r="353">
-      <x:c r="I353" s="11"/>
-    </x:row>
-    <x:row r="354">
-      <x:c r="I354" s="11"/>
-    </x:row>
-    <x:row r="355">
-      <x:c r="I355" s="11"/>
-    </x:row>
-    <x:row r="356">
-      <x:c r="I356" s="11"/>
-    </x:row>
-    <x:row r="357">
-      <x:c r="I357" s="11"/>
-    </x:row>
-    <x:row r="358">
-      <x:c r="I358" s="11"/>
-    </x:row>
-    <x:row r="359">
-      <x:c r="I359" s="11"/>
-    </x:row>
-    <x:row r="360">
-      <x:c r="I360" s="11"/>
-    </x:row>
-    <x:row r="361">
-      <x:c r="I361" s="11"/>
-    </x:row>
-    <x:row r="362">
-      <x:c r="I362" s="11"/>
-    </x:row>
-    <x:row r="363">
-      <x:c r="I363" s="11"/>
-    </x:row>
-    <x:row r="364">
-      <x:c r="I364" s="11"/>
-    </x:row>
-    <x:row r="365">
-      <x:c r="I365" s="11"/>
-    </x:row>
-    <x:row r="366">
-      <x:c r="I366" s="11"/>
-    </x:row>
-    <x:row r="367">
-      <x:c r="I367" s="11"/>
-    </x:row>
-    <x:row r="368">
-      <x:c r="I368" s="11"/>
-    </x:row>
-    <x:row r="369">
-      <x:c r="I369" s="11"/>
-    </x:row>
-    <x:row r="370">
-      <x:c r="I370" s="11"/>
-    </x:row>
-    <x:row r="371">
-      <x:c r="I371" s="11"/>
-    </x:row>
-    <x:row r="372">
-      <x:c r="I372" s="11"/>
-    </x:row>
-    <x:row r="373">
-      <x:c r="I373" s="11"/>
-    </x:row>
-    <x:row r="374">
-      <x:c r="I374" s="11"/>
-    </x:row>
-    <x:row r="375">
-      <x:c r="I375" s="11"/>
-    </x:row>
-    <x:row r="376">
-      <x:c r="I376" s="11"/>
-    </x:row>
-    <x:row r="377">
-      <x:c r="I377" s="11"/>
-    </x:row>
-    <x:row r="378">
-      <x:c r="I378" s="11"/>
-    </x:row>
-    <x:row r="379">
-      <x:c r="I379" s="11"/>
-    </x:row>
-    <x:row r="380">
-      <x:c r="I380" s="11"/>
-    </x:row>
-    <x:row r="381">
-      <x:c r="I381" s="11"/>
-    </x:row>
-    <x:row r="382">
-      <x:c r="I382" s="11"/>
-    </x:row>
-    <x:row r="383">
-      <x:c r="I383" s="11"/>
-    </x:row>
-    <x:row r="384">
-      <x:c r="I384" s="11"/>
-    </x:row>
-    <x:row r="385">
-      <x:c r="I385" s="11"/>
-    </x:row>
-    <x:row r="386">
-      <x:c r="I386" s="11"/>
-    </x:row>
-    <x:row r="387">
-      <x:c r="I387" s="11"/>
-    </x:row>
-    <x:row r="388">
-      <x:c r="I388" s="11"/>
+    <x:row r="350" ht="100" customHeight="1">
+      <x:c r="A350" s="24" t="str">
+        <x:v>LOGTEST-DESIGN-20260928</x:v>
+      </x:c>
+      <x:c r="B350" s="24" t="str">
+        <x:v>LOGTEST-REQ-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C350" s="24" t="str">
+        <x:v>F18/F20</x:v>
+      </x:c>
+      <x:c r="D350" s="24" t="str">
+        <x:v>DOC-069</x:v>
+      </x:c>
+      <x:c r="E350" s="24" t="str">
+        <x:v>Nghiên cứu và đăng ký đề xuất log/test</x:v>
+      </x:c>
+      <x:c r="F350" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G350" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H350" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I350" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J350" s="24" t="str">
+        <x:v>DOC-069 v0.1 source/permalink pin commit; chạy lại 7 unit/app +8 PostgreSQL integration PASS; local/Drive đọc lại.</x:v>
+      </x:c>
+      <x:c r="K350" s="24" t="str">
+        <x:v>Chỉ hoàn tất tài liệu đề xuất; thiết kế chưa duyệt, chưa triển khai log/test mới. Native/remote CI chưa kiểm.</x:v>
+      </x:c>
+      <x:c r="L350" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="351" ht="100" customHeight="1">
+      <x:c r="A351" s="24" t="str">
+        <x:v>LOGTEST-DESIGN-20260928</x:v>
+      </x:c>
+      <x:c r="B351" s="24" t="str">
+        <x:v>LOGTEST-REQ-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C351" s="24" t="str">
+        <x:v>F18/F20</x:v>
+      </x:c>
+      <x:c r="D351" s="24" t="str">
+        <x:v>DOC-000</x:v>
+      </x:c>
+      <x:c r="E351" s="24" t="str">
+        <x:v>Nghiên cứu và đăng ký đề xuất log/test</x:v>
+      </x:c>
+      <x:c r="F351" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G351" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H351" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I351" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J351" s="24" t="str">
+        <x:v>DOC-069 v0.1 source/permalink pin commit; chạy lại 7 unit/app +8 PostgreSQL integration PASS; local/Drive đọc lại.</x:v>
+      </x:c>
+      <x:c r="K351" s="24" t="str">
+        <x:v>Chỉ hoàn tất tài liệu đề xuất; thiết kế chưa duyệt, chưa triển khai log/test mới. Native/remote CI chưa kiểm.</x:v>
+      </x:c>
+      <x:c r="L351" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="352" ht="115" customHeight="1">
+      <x:c r="A352" s="24" t="str">
+        <x:v>STRUCTURE-20260928</x:v>
+      </x:c>
+      <x:c r="B352" s="24" t="str">
+        <x:v>STRUCTURE-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C352" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D352" s="24" t="str">
+        <x:v>DOC-054</x:v>
+      </x:c>
+      <x:c r="E352" s="24" t="str">
+        <x:v>Khung trước chức năng</x:v>
+      </x:c>
+      <x:c r="F352" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G352" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H352" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I352" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J352" s="24" t="str">
+        <x:v>STRUCTURE-01: DOC-070 v1.0; lint/types, 7 unit/mobile +8 DB, API/Expo bundles và web smoke PASS. Khung miền khác chỉ .gitkeep. Native/remote CI và bộ log/test A chưa triển khai. Nguồn/ZIP/Drive đọc lại cùng ID.</x:v>
+      </x:c>
+      <x:c r="K352" s="24" t="str">
+        <x:v>Không commit/push mới; native và remote CI chưa nghiệm thu.</x:v>
+      </x:c>
+      <x:c r="L352" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="353" ht="115" customHeight="1">
+      <x:c r="A353" s="24" t="str">
+        <x:v>STRUCTURE-20260928</x:v>
+      </x:c>
+      <x:c r="B353" s="24" t="str">
+        <x:v>STRUCTURE-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C353" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D353" s="24" t="str">
+        <x:v>DOC-064</x:v>
+      </x:c>
+      <x:c r="E353" s="24" t="str">
+        <x:v>Khung trước chức năng</x:v>
+      </x:c>
+      <x:c r="F353" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G353" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H353" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I353" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J353" s="24" t="str">
+        <x:v>STRUCTURE-01: DOC-070 v1.0; lint/types, 7 unit/mobile +8 DB, API/Expo bundles và web smoke PASS. Khung miền khác chỉ .gitkeep. Native/remote CI và bộ log/test A chưa triển khai. Nguồn/ZIP/Drive đọc lại cùng ID.</x:v>
+      </x:c>
+      <x:c r="K353" s="24" t="str">
+        <x:v>Không commit/push mới; native và remote CI chưa nghiệm thu.</x:v>
+      </x:c>
+      <x:c r="L353" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="354" ht="115" customHeight="1">
+      <x:c r="A354" s="24" t="str">
+        <x:v>STRUCTURE-20260928</x:v>
+      </x:c>
+      <x:c r="B354" s="24" t="str">
+        <x:v>STRUCTURE-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C354" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D354" s="24" t="str">
+        <x:v>DOC-065</x:v>
+      </x:c>
+      <x:c r="E354" s="24" t="str">
+        <x:v>Khung trước chức năng</x:v>
+      </x:c>
+      <x:c r="F354" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G354" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H354" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I354" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J354" s="24" t="str">
+        <x:v>STRUCTURE-01: DOC-070 v1.0; lint/types, 7 unit/mobile +8 DB, API/Expo bundles và web smoke PASS. Khung miền khác chỉ .gitkeep. Native/remote CI và bộ log/test A chưa triển khai. Nguồn/ZIP/Drive đọc lại cùng ID.</x:v>
+      </x:c>
+      <x:c r="K354" s="24" t="str">
+        <x:v>Không commit/push mới; native và remote CI chưa nghiệm thu.</x:v>
+      </x:c>
+      <x:c r="L354" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="355" ht="115" customHeight="1">
+      <x:c r="A355" s="24" t="str">
+        <x:v>STRUCTURE-20260928</x:v>
+      </x:c>
+      <x:c r="B355" s="24" t="str">
+        <x:v>STRUCTURE-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C355" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D355" s="24" t="str">
+        <x:v>DOC-066</x:v>
+      </x:c>
+      <x:c r="E355" s="24" t="str">
+        <x:v>Khung trước chức năng</x:v>
+      </x:c>
+      <x:c r="F355" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G355" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H355" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I355" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J355" s="24" t="str">
+        <x:v>STRUCTURE-01: DOC-070 v1.0; lint/types, 7 unit/mobile +8 DB, API/Expo bundles và web smoke PASS. Khung miền khác chỉ .gitkeep. Native/remote CI và bộ log/test A chưa triển khai. Nguồn/ZIP/Drive đọc lại cùng ID.</x:v>
+      </x:c>
+      <x:c r="K355" s="24" t="str">
+        <x:v>Không commit/push mới; native và remote CI chưa nghiệm thu.</x:v>
+      </x:c>
+      <x:c r="L355" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="356" ht="115" customHeight="1">
+      <x:c r="A356" s="24" t="str">
+        <x:v>STRUCTURE-20260928</x:v>
+      </x:c>
+      <x:c r="B356" s="24" t="str">
+        <x:v>STRUCTURE-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C356" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D356" s="24" t="str">
+        <x:v>DOC-069</x:v>
+      </x:c>
+      <x:c r="E356" s="24" t="str">
+        <x:v>Khung trước chức năng</x:v>
+      </x:c>
+      <x:c r="F356" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G356" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H356" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I356" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J356" s="24" t="str">
+        <x:v>STRUCTURE-01: DOC-070 v1.0; lint/types, 7 unit/mobile +8 DB, API/Expo bundles và web smoke PASS. Khung miền khác chỉ .gitkeep. Native/remote CI và bộ log/test A chưa triển khai. Nguồn/ZIP/Drive đọc lại cùng ID.</x:v>
+      </x:c>
+      <x:c r="K356" s="24" t="str">
+        <x:v>Không commit/push mới; native và remote CI chưa nghiệm thu.</x:v>
+      </x:c>
+      <x:c r="L356" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="357" ht="115" customHeight="1">
+      <x:c r="A357" s="24" t="str">
+        <x:v>STRUCTURE-20260928</x:v>
+      </x:c>
+      <x:c r="B357" s="24" t="str">
+        <x:v>STRUCTURE-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C357" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D357" s="24" t="str">
+        <x:v>DOC-070</x:v>
+      </x:c>
+      <x:c r="E357" s="24" t="str">
+        <x:v>Khung trước chức năng</x:v>
+      </x:c>
+      <x:c r="F357" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G357" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H357" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I357" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J357" s="24" t="str">
+        <x:v>STRUCTURE-01: DOC-070 v1.0; lint/types, 7 unit/mobile +8 DB, API/Expo bundles và web smoke PASS. Khung miền khác chỉ .gitkeep. Native/remote CI và bộ log/test A chưa triển khai. Nguồn/ZIP/Drive đọc lại cùng ID.</x:v>
+      </x:c>
+      <x:c r="K357" s="24" t="str">
+        <x:v>Không commit/push mới; native và remote CI chưa nghiệm thu.</x:v>
+      </x:c>
+      <x:c r="L357" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="358" ht="115" customHeight="1">
+      <x:c r="A358" s="24" t="str">
+        <x:v>STRUCTURE-20260928</x:v>
+      </x:c>
+      <x:c r="B358" s="24" t="str">
+        <x:v>STRUCTURE-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C358" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D358" s="24" t="str">
+        <x:v>DOC-018</x:v>
+      </x:c>
+      <x:c r="E358" s="24" t="str">
+        <x:v>Khung trước chức năng</x:v>
+      </x:c>
+      <x:c r="F358" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G358" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H358" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I358" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J358" s="24" t="str">
+        <x:v>STRUCTURE-01: DOC-070 v1.0; lint/types, 7 unit/mobile +8 DB, API/Expo bundles và web smoke PASS. Khung miền khác chỉ .gitkeep. Native/remote CI và bộ log/test A chưa triển khai. Nguồn/ZIP/Drive đọc lại cùng ID.</x:v>
+      </x:c>
+      <x:c r="K358" s="24" t="str">
+        <x:v>Không commit/push mới; native và remote CI chưa nghiệm thu.</x:v>
+      </x:c>
+      <x:c r="L358" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="359" ht="115" customHeight="1">
+      <x:c r="A359" s="24" t="str">
+        <x:v>STRUCTURE-20260928</x:v>
+      </x:c>
+      <x:c r="B359" s="24" t="str">
+        <x:v>STRUCTURE-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C359" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D359" s="24" t="str">
+        <x:v>DOC-040</x:v>
+      </x:c>
+      <x:c r="E359" s="24" t="str">
+        <x:v>Khung trước chức năng</x:v>
+      </x:c>
+      <x:c r="F359" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G359" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H359" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I359" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J359" s="24" t="str">
+        <x:v>STRUCTURE-01: DOC-070 v1.0; lint/types, 7 unit/mobile +8 DB, API/Expo bundles và web smoke PASS. Khung miền khác chỉ .gitkeep. Native/remote CI và bộ log/test A chưa triển khai. Nguồn/ZIP/Drive đọc lại cùng ID.</x:v>
+      </x:c>
+      <x:c r="K359" s="24" t="str">
+        <x:v>Không commit/push mới; native và remote CI chưa nghiệm thu.</x:v>
+      </x:c>
+      <x:c r="L359" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="360" ht="115" customHeight="1">
+      <x:c r="A360" s="24" t="str">
+        <x:v>STRUCTURE-20260928</x:v>
+      </x:c>
+      <x:c r="B360" s="24" t="str">
+        <x:v>STRUCTURE-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C360" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D360" s="24" t="str">
+        <x:v>DOC-000</x:v>
+      </x:c>
+      <x:c r="E360" s="24" t="str">
+        <x:v>Khung trước chức năng</x:v>
+      </x:c>
+      <x:c r="F360" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G360" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H360" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I360" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J360" s="24" t="str">
+        <x:v>STRUCTURE-01: DOC-070 v1.0; lint/types, 7 unit/mobile +8 DB, API/Expo bundles và web smoke PASS. Khung miền khác chỉ .gitkeep. Native/remote CI và bộ log/test A chưa triển khai. Nguồn/ZIP/Drive đọc lại cùng ID.</x:v>
+      </x:c>
+      <x:c r="K360" s="24" t="str">
+        <x:v>Không commit/push mới; native và remote CI chưa nghiệm thu.</x:v>
+      </x:c>
+      <x:c r="L360" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="361" ht="115" customHeight="1">
+      <x:c r="A361" s="24" t="str">
+        <x:v>STRUCTURE-20260928</x:v>
+      </x:c>
+      <x:c r="B361" s="24" t="str">
+        <x:v>STRUCTURE-01</x:v>
+      </x:c>
+      <x:c r="C361" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D361" s="24" t="str">
+        <x:v>BRD/PRD/FR/SRS/UX/API/ERD/QA/viewer</x:v>
+      </x:c>
+      <x:c r="E361" s="24" t="str">
+        <x:v>Rà phạm vi ảnh hưởng</x:v>
+      </x:c>
+      <x:c r="F361" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
+      <x:c r="G361" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H361" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I361" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J361" s="24" t="str">
+        <x:v>Đối chiếu nguồn và tìm đường dẫn cũ: contract, schema, nghiệp vụ và prototype không đổi. Không sửa JSON/viewer/UI ZIP; ZIP hồ sơ chứa runbook được làm mới.</x:v>
+      </x:c>
+      <x:c r="K361" s="24" t="str">
+        <x:v>Không coi folder rỗng là chức năng hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L361" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="362" ht="120" customHeight="1">
+      <x:c r="A362" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B362" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C362" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D362" s="24" t="str">
+        <x:v>DOC-000</x:v>
+      </x:c>
+      <x:c r="E362" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F362" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G362" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H362" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I362" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J362" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K362" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L362" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="363" ht="120" customHeight="1">
+      <x:c r="A363" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B363" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C363" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D363" s="24" t="str">
+        <x:v>DOC-054</x:v>
+      </x:c>
+      <x:c r="E363" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F363" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G363" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H363" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I363" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J363" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K363" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L363" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="364" ht="120" customHeight="1">
+      <x:c r="A364" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B364" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C364" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D364" s="24" t="str">
+        <x:v>DOC-064</x:v>
+      </x:c>
+      <x:c r="E364" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F364" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G364" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H364" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I364" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J364" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K364" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L364" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="365" ht="120" customHeight="1">
+      <x:c r="A365" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B365" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C365" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D365" s="24" t="str">
+        <x:v>DOC-065</x:v>
+      </x:c>
+      <x:c r="E365" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F365" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G365" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H365" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I365" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J365" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K365" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L365" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="366" ht="120" customHeight="1">
+      <x:c r="A366" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B366" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C366" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D366" s="24" t="str">
+        <x:v>DOC-066</x:v>
+      </x:c>
+      <x:c r="E366" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F366" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G366" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H366" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I366" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J366" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K366" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L366" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="367" ht="120" customHeight="1">
+      <x:c r="A367" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B367" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C367" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D367" s="24" t="str">
+        <x:v>DOC-069</x:v>
+      </x:c>
+      <x:c r="E367" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F367" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G367" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H367" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I367" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J367" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K367" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L367" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="368" ht="120" customHeight="1">
+      <x:c r="A368" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B368" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C368" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D368" s="24" t="str">
+        <x:v>DOC-070</x:v>
+      </x:c>
+      <x:c r="E368" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F368" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G368" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H368" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I368" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J368" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K368" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L368" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="369" ht="120" customHeight="1">
+      <x:c r="A369" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B369" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C369" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D369" s="24" t="str">
+        <x:v>PLAN-002</x:v>
+      </x:c>
+      <x:c r="E369" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F369" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G369" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H369" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I369" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J369" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K369" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L369" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="370" ht="120" customHeight="1">
+      <x:c r="A370" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B370" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C370" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D370" s="24" t="str">
+        <x:v>PLAN-003</x:v>
+      </x:c>
+      <x:c r="E370" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F370" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G370" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H370" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I370" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J370" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K370" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L370" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="371" ht="120" customHeight="1">
+      <x:c r="A371" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B371" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C371" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D371" s="24" t="str">
+        <x:v>PLAN-004</x:v>
+      </x:c>
+      <x:c r="E371" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F371" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G371" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H371" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I371" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J371" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K371" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L371" s="24" t="str">
+        <x:v>Một phần</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="372" ht="120" customHeight="1">
+      <x:c r="A372" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B372" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C372" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D372" s="24" t="str">
+        <x:v>PLAN-008</x:v>
+      </x:c>
+      <x:c r="E372" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F372" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G372" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H372" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I372" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J372" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K372" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L372" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="373" ht="120" customHeight="1">
+      <x:c r="A373" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B373" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C373" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D373" s="24" t="str">
+        <x:v>DOC-037</x:v>
+      </x:c>
+      <x:c r="E373" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F373" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G373" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H373" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I373" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J373" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K373" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L373" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="374" ht="120" customHeight="1">
+      <x:c r="A374" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B374" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C374" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D374" s="24" t="str">
+        <x:v>DOC-039</x:v>
+      </x:c>
+      <x:c r="E374" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F374" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G374" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H374" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I374" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J374" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K374" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L374" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="375" ht="120" customHeight="1">
+      <x:c r="A375" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B375" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C375" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D375" s="24" t="str">
+        <x:v>DOC-040</x:v>
+      </x:c>
+      <x:c r="E375" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F375" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G375" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H375" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I375" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J375" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K375" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L375" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="376" ht="120" customHeight="1">
+      <x:c r="A376" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B376" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C376" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D376" s="24" t="str">
+        <x:v>DOC-041</x:v>
+      </x:c>
+      <x:c r="E376" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F376" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G376" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H376" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I376" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J376" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K376" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L376" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="377" ht="120" customHeight="1">
+      <x:c r="A377" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B377" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C377" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D377" s="24" t="str">
+        <x:v>DOC-043</x:v>
+      </x:c>
+      <x:c r="E377" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F377" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G377" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H377" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I377" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J377" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K377" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L377" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="378" ht="120" customHeight="1">
+      <x:c r="A378" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B378" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C378" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D378" s="24" t="str">
+        <x:v>DOC-045</x:v>
+      </x:c>
+      <x:c r="E378" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F378" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G378" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H378" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I378" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J378" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K378" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L378" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="379" ht="120" customHeight="1">
+      <x:c r="A379" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B379" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C379" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D379" s="24" t="str">
+        <x:v>DOC-046</x:v>
+      </x:c>
+      <x:c r="E379" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F379" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G379" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H379" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I379" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J379" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K379" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L379" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="380" ht="120" customHeight="1">
+      <x:c r="A380" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B380" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C380" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D380" s="24" t="str">
+        <x:v>DOC-047</x:v>
+      </x:c>
+      <x:c r="E380" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F380" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G380" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H380" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I380" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J380" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K380" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L380" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="381" ht="120" customHeight="1">
+      <x:c r="A381" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B381" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C381" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D381" s="24" t="str">
+        <x:v>DOC-048</x:v>
+      </x:c>
+      <x:c r="E381" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F381" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G381" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H381" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I381" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J381" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K381" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L381" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="382" ht="120" customHeight="1">
+      <x:c r="A382" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B382" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C382" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D382" s="24" t="str">
+        <x:v>DOC-016</x:v>
+      </x:c>
+      <x:c r="E382" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F382" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G382" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H382" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I382" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J382" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K382" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L382" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="383" ht="120" customHeight="1">
+      <x:c r="A383" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B383" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C383" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D383" s="24" t="str">
+        <x:v>DOC-017</x:v>
+      </x:c>
+      <x:c r="E383" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F383" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G383" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H383" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I383" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J383" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K383" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L383" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="384" ht="120" customHeight="1">
+      <x:c r="A384" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B384" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C384" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D384" s="24" t="str">
+        <x:v>DOC-018</x:v>
+      </x:c>
+      <x:c r="E384" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F384" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G384" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H384" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I384" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J384" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K384" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L384" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="385" ht="120" customHeight="1">
+      <x:c r="A385" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B385" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C385" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D385" s="24" t="str">
+        <x:v>DOC-030</x:v>
+      </x:c>
+      <x:c r="E385" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F385" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G385" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H385" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I385" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J385" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K385" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L385" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="386" ht="120" customHeight="1">
+      <x:c r="A386" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B386" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C386" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D386" s="24" t="str">
+        <x:v>DOC-033</x:v>
+      </x:c>
+      <x:c r="E386" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F386" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G386" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H386" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I386" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J386" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K386" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L386" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="387" ht="120" customHeight="1">
+      <x:c r="A387" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B387" s="24" t="str">
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+      </x:c>
+      <x:c r="C387" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D387" s="24" t="str">
+        <x:v>DOC-071</x:v>
+      </x:c>
+      <x:c r="E387" s="24" t="str">
+        <x:v>Triển khai phương án A</x:v>
+      </x:c>
+      <x:c r="F387" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G387" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H387" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I387" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J387" s="24" t="str">
+        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. Nguồn/served/ZIP và Drive cùng ID đọc lại.</x:v>
+      </x:c>
+      <x:c r="K387" s="24" t="str">
+        <x:v>Native/remoteCI chưa nghiệm thu; PLAN-004 production chưa hoàn thành.</x:v>
+      </x:c>
+      <x:c r="L387" s="24" t="str">
+        <x:v>Hoàn tất phạm vi local</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="388" ht="120" customHeight="1">
+      <x:c r="A388" s="24" t="str">
+        <x:v>LOGTEST-20260928</x:v>
+      </x:c>
+      <x:c r="B388" s="24" t="str">
+        <x:v>LOGTEST-01</x:v>
+      </x:c>
+      <x:c r="C388" s="24" t="str">
+        <x:v>F02/F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D388" s="24" t="str">
+        <x:v>BRD/PRD/FR/SRS/ERD/UX</x:v>
+      </x:c>
+      <x:c r="E388" s="24" t="str">
+        <x:v>Rà phạm vi nghiệp vụ</x:v>
+      </x:c>
+      <x:c r="F388" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
+      <x:c r="G388" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H388" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I388" s="25" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="J388" s="24" t="str">
+        <x:v>Không đổi nghiệp vụ, quyền/trạng thái, SQL/seed, UI prototype hay ERD. Contract lỗi/header, kiến trúc API và QA được đồng bộ trong nguồn kỹ thuật.</x:v>
+      </x:c>
+      <x:c r="K388" s="24" t="str">
+        <x:v>Không cập nhật UI ZIP/nguồn nghiệp vụ chỉ vì thay hạ tầng log/test.</x:v>
+      </x:c>
+      <x:c r="L388" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
     </x:row>
     <x:row r="389">
       <x:c r="I389" s="11"/>
@@ -39134,7 +40875,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a0c8cfeecb947c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc79d16519e4a4bb4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39376,7 +41117,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23100ab2ff084ac0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a48a53dad144706"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: prepare mobile development builds and setup guides
</commit_message>
<xml_diff>
--- a/docs/project-control/So-quan-ly-tai-lieu.xlsx
+++ b/docs/project-control/So-quan-ly-tai-lieu.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bat dau" sheetId="1" r:id="Rfe4fd5fde09041f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh muc" sheetId="2" r:id="R6f2998d7706d4bff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anh huong" sheetId="3" r:id="R74b817679b1748f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quyet dinh" sheetId="4" r:id="R144fd33092614f35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dong bo" sheetId="5" r:id="R07e4f31a5c484ec1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quy trinh" sheetId="6" r:id="R85834ea87e8c4d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bat dau" sheetId="1" r:id="R0150bbbdf20e48e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh muc" sheetId="2" r:id="R8e59ba579f244fd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anh huong" sheetId="3" r:id="R8733cef6ebee4de4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quyet dinh" sheetId="4" r:id="Rb200d66dd94042c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dong bo" sheetId="5" r:id="R0bffdca58a61443a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quy trinh" sheetId="6" r:id="R8a5f932cac484ad4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -181,7 +181,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="86" name="Tbl1" displayName="Tbl1" ref="A5:L86" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="86" name="Tbl1" displayName="Tbl1" ref="A5:L96" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Mã tài liệu"/>
     <x:tableColumn id="2" name="Tài liệu"/>
@@ -201,7 +201,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="89" name="Tbl2" displayName="Tbl2" ref="A5:F813" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="89" name="Tbl2" displayName="Tbl2" ref="A5:F843" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Mã chức năng"/>
     <x:tableColumn id="2" name="Chức năng"/>
@@ -215,7 +215,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="87" name="Tbl3" displayName="Tbl3" ref="A5:G56" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="87" name="Tbl3" displayName="Tbl3" ref="A5:G59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Mã quyết định"/>
     <x:tableColumn id="2" name="Chủ đề"/>
@@ -230,7 +230,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="88" name="Tbl4" displayName="Tbl4" ref="A5:L388" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="88" name="Tbl4" displayName="Tbl4" ref="A5:L423" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Mã đợt"/>
     <x:tableColumn id="2" name="Quyết định"/>
@@ -489,7 +489,7 @@
     <x:row r="3">
       <x:c r="A3" s="1"/>
       <x:c r="B3" s="1" t="str">
-        <x:v>Phiên bản 1.34 · 28/09/2026 · LOGTEST-01: phương án A đã triển khai/kiểm local; native/remoteCI còn thiếu</x:v>
+        <x:v>Phiên bản 1.37 · 29/09/2026 · NATIVE-B-01: kiểm môi trường Android/iOS và triển khai phần B; giữ PATH-01</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>
@@ -511,7 +511,7 @@
       </x:c>
       <x:c r="C5" s="13" t="n">
         <x:f>COUNTA('Danh muc'!A6:A1000)-COUNTIFS('Danh muc'!F6:F1000,"Chưa có")</x:f>
-        <x:v>79</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="D5" s="1"/>
       <x:c r="E5" s="1"/>
@@ -537,7 +537,7 @@
       </x:c>
       <x:c r="C7" s="13" t="n">
         <x:f>COUNTA('Dong bo'!A6:A1000)-COUNTIFS('Dong bo'!L6:L1000,"Hoàn tất")-COUNTIFS('Dong bo'!L6:L1000,"Không áp dụng có lý do")</x:f>
-        <x:v>31</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D7" s="1"/>
       <x:c r="E7" s="1"/>
@@ -550,7 +550,7 @@
       </x:c>
       <x:c r="C8" s="13" t="n">
         <x:f>COUNTIFS('Dong bo'!L6:L1000,"Hoàn tất")</x:f>
-        <x:v>327</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="D8" s="1"/>
       <x:c r="E8" s="1"/>
@@ -587,7 +587,7 @@
     <x:row r="12" ht="28" customHeight="1">
       <x:c r="A12" s="1"/>
       <x:c r="B12" s="14" t="str">
-        <x:v>Danh muc</x:v>
+        <x:v>#gid=1174524789</x:v>
       </x:c>
       <x:c r="C12" s="1" t="str">
         <x:v>Tìm tài liệu, phiên bản, bản chính và bản cũ</x:v>
@@ -599,7 +599,7 @@
     <x:row r="13" ht="28" customHeight="1">
       <x:c r="A13" s="1"/>
       <x:c r="B13" s="14" t="str">
-        <x:v>Anh huong</x:v>
+        <x:v>#gid=1659053007</x:v>
       </x:c>
       <x:c r="C13" s="1" t="str">
         <x:v>Tìm tất cả tài liệu liên quan đến chức năng</x:v>
@@ -611,7 +611,7 @@
     <x:row r="14" ht="28" customHeight="1">
       <x:c r="A14" s="1"/>
       <x:c r="B14" s="14" t="str">
-        <x:v>Quyet dinh</x:v>
+        <x:v>#gid=1142207888</x:v>
       </x:c>
       <x:c r="C14" s="1" t="str">
         <x:v>Đọc đúng nội dung user đã chốt</x:v>
@@ -623,7 +623,7 @@
     <x:row r="15" ht="28" customHeight="1">
       <x:c r="A15" s="1"/>
       <x:c r="B15" s="14" t="str">
-        <x:v>Dong bo</x:v>
+        <x:v>#gid=1783723350</x:v>
       </x:c>
       <x:c r="C15" s="1" t="str">
         <x:v>Theo dõi sửa từng tài liệu và bằng chứng</x:v>
@@ -635,7 +635,7 @@
     <x:row r="16" ht="28" customHeight="1">
       <x:c r="A16" s="1"/>
       <x:c r="B16" s="14" t="str">
-        <x:v>Quy trinh</x:v>
+        <x:v>#gid=1416641078</x:v>
       </x:c>
       <x:c r="C16" s="1" t="str">
         <x:v>Thực hiện quy tắc cập nhật nhất quán</x:v>
@@ -751,7 +751,7 @@
     <x:hyperlink ref="B14" location="'Quyet dinh'!A1"/>
     <x:hyperlink ref="B15" location="'Dong bo'!A1"/>
     <x:hyperlink ref="B16" location="'Quy trinh'!A1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="R72a03738674442a4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="Rade9e0e4cbdd4596"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -887,7 +887,7 @@
         <x:v>Quản lý hồ sơ</x:v>
       </x:c>
       <x:c r="D6" s="8" t="str">
-        <x:v>v1.34</x:v>
+        <x:v>v1.37</x:v>
       </x:c>
       <x:c r="E6" s="8" t="str">
         <x:v>Sổ quản lý chính</x:v>
@@ -896,7 +896,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G6" s="8" t="str">
-        <x:v>RULE-01; STRUCTURE-01; LOGTEST-01</x:v>
+        <x:v>RULE-01; STRUCTURE-01; LOGTEST-01; MOBILE-GUIDE-01; PATH-01; NATIVE-B-01</x:v>
       </x:c>
       <x:c r="H6" s="9" t="str">
         <x:v>Mở tài liệu</x:v>
@@ -906,10 +906,10 @@
       </x:c>
       <x:c r="J6" s="8" t="str"/>
       <x:c r="K6" s="8" t="str">
-        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
       </x:c>
       <x:c r="L6" s="10" t="n">
-        <x:v>46293</x:v>
+        <x:v>46294</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="68" customHeight="1">
@@ -1282,8 +1282,10 @@
       <x:c r="C17" s="8" t="str">
         <x:v>Mục lục hồ sơ</x:v>
       </x:c>
-      <x:c r="D17" s="8" t="str">
-        <x:v>v0.1.1 / Đợt 1</x:v>
+      <x:c r="D17" s="8" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">v0.1.1 / PATH-01</x:t>
+        </x:is>
       </x:c>
       <x:c r="E17" s="8" t="str">
         <x:v>Nguồn bổ trợ</x:v>
@@ -1291,8 +1293,10 @@
       <x:c r="F17" s="8" t="str">
         <x:v>Mới nhất</x:v>
       </x:c>
-      <x:c r="G17" s="8" t="str">
-        <x:v>Quyết định theo chức năng; IMPLEMENT-01; TECH-01</x:v>
+      <x:c r="G17" s="8" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Quyết định theo chức năng; IMPLEMENT-01; TECH-01; PATH-01</x:t>
+        </x:is>
       </x:c>
       <x:c r="H17" s="9" t="str">
         <x:v>Mở tài liệu</x:v>
@@ -1301,11 +1305,13 @@
         <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/project-docs/01-danh-muc-ho-so.md</x:v>
       </x:c>
       <x:c r="J17" s="8" t="str"/>
-      <x:c r="K17" s="8" t="str">
-        <x:v>Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID.</x:v>
-      </x:c>
-      <x:c r="L17" s="10" t="n">
-        <x:v>46293</x:v>
+      <x:c r="K17" s="8" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Đợt 1 local danh mục đã kiểm; DOC-065/066. Giữ phần ngoài danh mục là thiết kế; native và CI từ xa chưa chạy. Nguồn/bản xuất/Drive đã đọc lại cùng ID. PATH-01: đã bỏ outputs; nội dung local/ZIP đã kiểm, Drive cập nhật cùng ID và đọc lại metadata/kích thước ngày 29/09/2026. Không đổi nghiệp vụ hoặc nghiệm thu native/CI.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L17" s="10">
+        <x:v>46294</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="68" customHeight="1">
@@ -1539,7 +1545,7 @@
         <x:v>Gói nguồn hồ sơ</x:v>
       </x:c>
       <x:c r="D24" s="8" t="str">
-        <x:v>v0.1.1 / LOGTEST-01</x:v>
+        <x:v>v0.1.1 / NATIVE-B-01</x:v>
       </x:c>
       <x:c r="E24" s="8" t="str">
         <x:v>Gói xuất</x:v>
@@ -1548,7 +1554,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G24" s="8" t="str">
-        <x:v>Quyết định theo chức năng; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01</x:v>
+        <x:v>Quyết định theo chức năng; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01; PATH-01; NATIVE-B-01</x:v>
       </x:c>
       <x:c r="H24" s="9" t="str">
         <x:v>Mở tài liệu</x:v>
@@ -1558,10 +1564,10 @@
       </x:c>
       <x:c r="J24" s="8" t="str"/>
       <x:c r="K24" s="8" t="str">
-        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
       </x:c>
       <x:c r="L24" s="10" t="n">
-        <x:v>46293</x:v>
+        <x:v>46294</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="38" customHeight="1">
@@ -2655,7 +2661,7 @@
         <x:v>Thiết kế kỹ thuật</x:v>
       </x:c>
       <x:c r="D55" s="20" t="str">
-        <x:v>v0.1.1 / LOGTEST-01</x:v>
+        <x:v>v0.1.1 / NATIVE-B-01</x:v>
       </x:c>
       <x:c r="E55" s="20" t="str">
         <x:v>Gói hiện hành</x:v>
@@ -2664,7 +2670,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G55" s="20" t="str">
-        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01</x:v>
+        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01; PATH-01; NATIVE-B-01</x:v>
       </x:c>
       <x:c r="H55" s="20" t="str">
         <x:v>https://drive.google.com/file/d/18z-ReFxGP-RhX5_cOVTidcHJJGFfB48D/view?usp=drivesdk</x:v>
@@ -2676,10 +2682,10 @@
         <x:v>Bản trên Drive</x:v>
       </x:c>
       <x:c r="K55" s="20" t="str">
-        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
       </x:c>
       <x:c r="L55" s="21" t="n">
-        <x:v>46293</x:v>
+        <x:v>46294</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="105" customHeight="1">
@@ -3034,8 +3040,10 @@
       <x:c r="C65" s="24" t="str">
         <x:v>Thiết kế UI</x:v>
       </x:c>
-      <x:c r="D65" s="24" t="str">
-        <x:v>v0.15</x:v>
+      <x:c r="D65" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">v0.15 / gói PATH-01</x:t>
+        </x:is>
       </x:c>
       <x:c r="E65" s="24" t="str">
         <x:v>Nhóm trước đã xem; đội ngũ mới để review</x:v>
@@ -3043,8 +3051,10 @@
       <x:c r="F65" s="24" t="str">
         <x:v>Mới nhất</x:v>
       </x:c>
-      <x:c r="G65" s="24" t="str">
-        <x:v>UI-05/06/07/08/09/10/11/12/13/14/15/16/UI-17/UI-18/UI-19/UI-20/UI-21</x:v>
+      <x:c r="G65" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">UI-05/06/07/08/09/10/11/12/13/14/15/16/UI-17/UI-18/UI-19/UI-20/UI-21; PATH-01</x:t>
+        </x:is>
       </x:c>
       <x:c r="H65" s="24" t="str">
         <x:v>https://drive.google.com/file/d/1Unjr9ELcli6zcOb-4U2z62EDZo8Q5iE7/view?usp=drivesdk</x:v>
@@ -3055,11 +3065,13 @@
       <x:c r="J65" s="24" t="str">
         <x:v>React/Storybook; UI-UX-v0.19.zip</x:v>
       </x:c>
-      <x:c r="K65" s="24" t="str">
-        <x:v>UI-21: sửa nối luồng; 49 tests, 52 stories. Ma trận chứng cứ và giới hạn DOC-063.</x:v>
-      </x:c>
-      <x:c r="L65" s="25" t="n">
-        <x:v>46288</x:v>
+      <x:c r="K65" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">UI-21: sửa nối luồng; 49 tests, 52 stories. Ma trận chứng cứ và giới hạn DOC-063. PATH-01: đã bỏ outputs; nội dung local/ZIP đã kiểm, Drive cập nhật cùng ID và đọc lại metadata/kích thước ngày 29/09/2026. Không đổi nghiệp vụ hoặc nghiệm thu native/CI.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L65" s="25">
+        <x:v>46294</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="104" customHeight="1">
@@ -3186,8 +3198,10 @@
       <x:c r="C69" s="24" t="str">
         <x:v>Quản lý dự án</x:v>
       </x:c>
-      <x:c r="D69" s="24" t="str">
-        <x:v>v0.3 / LOGTEST-01</x:v>
+      <x:c r="D69" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">v0.4 / PATH-01</x:t>
+        </x:is>
       </x:c>
       <x:c r="E69" s="24" t="str">
         <x:v>Hướng dẫn hiện hành</x:v>
@@ -3195,8 +3209,10 @@
       <x:c r="F69" s="24" t="str">
         <x:v>Mới nhất</x:v>
       </x:c>
-      <x:c r="G69" s="24" t="str">
-        <x:v>ORG-01/UI-21; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01</x:v>
+      <x:c r="G69" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ORG-01/UI-21; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01; PATH-01</x:t>
+        </x:is>
       </x:c>
       <x:c r="H69" s="24" t="str">
         <x:v>https://drive.google.com/file/d/18z-ReFxGP-RhX5_cOVTidcHJJGFfB48D/view</x:v>
@@ -3207,11 +3223,13 @@
       <x:c r="J69" s="24" t="str">
         <x:v>React/Storybook; UI-UX-v0.19.zip</x:v>
       </x:c>
-      <x:c r="K69" s="24" t="str">
-        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
-      </x:c>
-      <x:c r="L69" s="24" t="n">
-        <x:v>46293</x:v>
+      <x:c r="K69" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. PATH-01: đã bỏ outputs; nội dung local/ZIP đã kiểm, Drive cập nhật cùng ID và đọc lại metadata/kích thước ngày 29/09/2026. Không đổi nghiệp vụ hoặc nghiệm thu native/CI.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L69" s="24">
+        <x:v>46294</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="104" customHeight="1">
@@ -3566,8 +3584,10 @@
       <x:c r="C79" s="24" t="str">
         <x:v>Bàn giao triển khai</x:v>
       </x:c>
-      <x:c r="D79" s="24" t="str">
-        <x:v>v1.3</x:v>
+      <x:c r="D79" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">v1.4</x:t>
+        </x:is>
       </x:c>
       <x:c r="E79" s="24" t="str">
         <x:v>Prompt bàn giao; đã kích hoạt Đợt 1, hiện trạng ở DOC-065</x:v>
@@ -3575,8 +3595,10 @@
       <x:c r="F79" s="24" t="str">
         <x:v>Mới nhất</x:v>
       </x:c>
-      <x:c r="G79" s="24" t="str">
-        <x:v>HANDOFF-01; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01</x:v>
+      <x:c r="G79" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">HANDOFF-01; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01; PATH-01</x:t>
+        </x:is>
       </x:c>
       <x:c r="H79" s="24" t="str">
         <x:v>https://drive.google.com/file/d/1WnXV2mRTBnYePYztiKJvvfS6tCAjeTrW/view</x:v>
@@ -3587,11 +3609,13 @@
       <x:c r="J79" s="24" t="str">
         <x:v>Markdown nguồn local và Drive cùng nội dung</x:v>
       </x:c>
-      <x:c r="K79" s="24" t="str">
-        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
-      </x:c>
-      <x:c r="L79" s="24" t="n">
-        <x:v>46293</x:v>
+      <x:c r="K79" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy. PATH-01: đã bỏ outputs; nội dung local/ZIP đã kiểm, Drive cập nhật cùng ID và đọc lại metadata/kích thước ngày 29/09/2026. Không đổi nghiệp vụ hoặc nghiệm thu native/CI.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L79" s="24">
+        <x:v>46294</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="105" customHeight="1">
@@ -3605,7 +3629,7 @@
         <x:v>Triển khai</x:v>
       </x:c>
       <x:c r="D80" s="24" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.6</x:v>
       </x:c>
       <x:c r="E80" s="24" t="str">
         <x:v>Nguồn hiện trạng và kết quả local</x:v>
@@ -3614,7 +3638,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G80" s="24" t="str">
-        <x:v>IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01</x:v>
+        <x:v>IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01; PATH-01; NATIVE-B-01</x:v>
       </x:c>
       <x:c r="H80" s="24" t="str">
         <x:v>https://drive.google.com/file/d/1JjfKtYYgYGHlLSZCKZ21hqWiscQxoFpT/view</x:v>
@@ -3626,10 +3650,10 @@
         <x:v>docs/implementation/evidence; technical-design ZIP</x:v>
       </x:c>
       <x:c r="K80" s="24" t="str">
-        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
       </x:c>
       <x:c r="L80" s="24" t="n">
-        <x:v>46293</x:v>
+        <x:v>46294</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="105" customHeight="1">
@@ -3791,7 +3815,7 @@
         <x:v>Kiến trúc / triển khai</x:v>
       </x:c>
       <x:c r="D85" s="24" t="str">
-        <x:v>v1.1</x:v>
+        <x:v>v1.3</x:v>
       </x:c>
       <x:c r="E85" s="24" t="str">
         <x:v>Bản đồ code, trách nhiệm folder và quy tắc mở rộng</x:v>
@@ -3800,7 +3824,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G85" s="24" t="str">
-        <x:v>STRUCTURE-01; LOGTEST-DESIGN-01; LOGTEST-01</x:v>
+        <x:v>STRUCTURE-01; LOGTEST-DESIGN-01; LOGTEST-01; PATH-01; NATIVE-B-01</x:v>
       </x:c>
       <x:c r="H85" s="24" t="str">
         <x:v>https://drive.google.com/file/d/1pWijvZgP7U3mpjq5Wualaa1mdPCDk_Ge/view</x:v>
@@ -3812,10 +3836,10 @@
         <x:v>README; hai ZIP kỹ thuật hiện hành</x:v>
       </x:c>
       <x:c r="K85" s="24" t="str">
-        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
       </x:c>
       <x:c r="L85" s="25" t="n">
-        <x:v>46293</x:v>
+        <x:v>46294</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="130" customHeight="1">
@@ -3829,7 +3853,7 @@
         <x:v>Triển khai / vận hành</x:v>
       </x:c>
       <x:c r="D86" s="24" t="str">
-        <x:v>v1.0</x:v>
+        <x:v>v1.1</x:v>
       </x:c>
       <x:c r="E86" s="24" t="str">
         <x:v>Runbook và bằng chứng kiểm local; giới hạn native/remoteCI</x:v>
@@ -3838,7 +3862,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G86" s="24" t="str">
-        <x:v>LOGTEST-01; LOGTEST-DESIGN-01</x:v>
+        <x:v>LOGTEST-01; LOGTEST-DESIGN-01; NATIVE-B-01</x:v>
       </x:c>
       <x:c r="H86" s="24" t="str">
         <x:v>https://drive.google.com/file/d/1m7nrDRbwKj7HPH3TQoWUIsT4zSKn_ldK/view</x:v>
@@ -3850,10 +3874,390 @@
         <x:v>Hai ZIP hiện hành; coverage/test-results local ignored</x:v>
       </x:c>
       <x:c r="K86" s="24" t="str">
-        <x:v>LOGTEST-01/DOC-071:31 mobile+26 API+2 tooling+2 web E2E PASS; coverage core API100/91.53, mobile100/95.70; load200/concurrency20 PASS. Negative coverage/failure artifacts đã kiểm. Native BLOCKED; remoteCI chưa chạy.</x:v>
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
       </x:c>
       <x:c r="L86" s="25" t="n">
-        <x:v>46293</x:v>
+        <x:v>46294</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="110" customHeight="1">
+      <x:c r="A87" s="24" t="str">
+        <x:v>DOC-072</x:v>
+      </x:c>
+      <x:c r="B87" s="24" t="str">
+        <x:v>Bắt đầu phát triển app Android và iOS</x:v>
+      </x:c>
+      <x:c r="C87" s="24" t="str">
+        <x:v>Hướng dẫn phát triển</x:v>
+      </x:c>
+      <x:c r="D87" s="24" t="str">
+        <x:v>v1.1</x:v>
+      </x:c>
+      <x:c r="E87" s="24" t="str">
+        <x:v>Nguồn Markdown</x:v>
+      </x:c>
+      <x:c r="F87" s="24" t="str">
+        <x:v>Mới nhất</x:v>
+      </x:c>
+      <x:c r="G87" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01; NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="H87" s="24" t="str">
+        <x:v>https://drive.google.com/file/d/10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u/view?usp=drivesdk</x:v>
+      </x:c>
+      <x:c r="I87" s="24" t="str">
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/README.md</x:v>
+      </x:c>
+      <x:c r="J87" s="24" t="str">
+        <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
+      </x:c>
+      <x:c r="K87" s="24" t="str">
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+      </x:c>
+      <x:c r="L87" s="24" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="110" customHeight="1">
+      <x:c r="A88" s="24" t="str">
+        <x:v>DOC-073</x:v>
+      </x:c>
+      <x:c r="B88" s="24" t="str">
+        <x:v>01 — Chuẩn bị máy và dùng Terminal</x:v>
+      </x:c>
+      <x:c r="C88" s="24" t="str">
+        <x:v>Hướng dẫn phát triển</x:v>
+      </x:c>
+      <x:c r="D88" s="24" t="str">
+        <x:v>v1.0</x:v>
+      </x:c>
+      <x:c r="E88" s="24" t="str">
+        <x:v>Nguồn Markdown</x:v>
+      </x:c>
+      <x:c r="F88" s="24" t="str">
+        <x:v>Mới nhất</x:v>
+      </x:c>
+      <x:c r="G88" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="H88" s="24" t="str">
+        <x:v>https://drive.google.com/file/d/10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u/view?usp=drivesdk</x:v>
+      </x:c>
+      <x:c r="I88" s="24" t="str">
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/01-chuan-bi-may.md</x:v>
+      </x:c>
+      <x:c r="J88" s="24" t="str">
+        <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
+      </x:c>
+      <x:c r="K88" s="24" t="str">
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+      </x:c>
+      <x:c r="L88" s="24" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="110" customHeight="1">
+      <x:c r="A89" s="24" t="str">
+        <x:v>DOC-074</x:v>
+      </x:c>
+      <x:c r="B89" s="24" t="str">
+        <x:v>02 — Cài Android Studio và tạo máy ảo</x:v>
+      </x:c>
+      <x:c r="C89" s="24" t="str">
+        <x:v>Hướng dẫn phát triển</x:v>
+      </x:c>
+      <x:c r="D89" s="24" t="str">
+        <x:v>v1.0</x:v>
+      </x:c>
+      <x:c r="E89" s="24" t="str">
+        <x:v>Nguồn Markdown</x:v>
+      </x:c>
+      <x:c r="F89" s="24" t="str">
+        <x:v>Mới nhất</x:v>
+      </x:c>
+      <x:c r="G89" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="H89" s="24" t="str">
+        <x:v>https://drive.google.com/file/d/10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u/view?usp=drivesdk</x:v>
+      </x:c>
+      <x:c r="I89" s="24" t="str">
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/02-android.md</x:v>
+      </x:c>
+      <x:c r="J89" s="24" t="str">
+        <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
+      </x:c>
+      <x:c r="K89" s="24" t="str">
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+      </x:c>
+      <x:c r="L89" s="24" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="110" customHeight="1">
+      <x:c r="A90" s="24" t="str">
+        <x:v>DOC-075</x:v>
+      </x:c>
+      <x:c r="B90" s="24" t="str">
+        <x:v>03 — Cài Xcode và iOS Simulator trên macOS 27</x:v>
+      </x:c>
+      <x:c r="C90" s="24" t="str">
+        <x:v>Hướng dẫn phát triển</x:v>
+      </x:c>
+      <x:c r="D90" s="24" t="str">
+        <x:v>v1.1</x:v>
+      </x:c>
+      <x:c r="E90" s="24" t="str">
+        <x:v>Nguồn Markdown</x:v>
+      </x:c>
+      <x:c r="F90" s="24" t="str">
+        <x:v>Mới nhất</x:v>
+      </x:c>
+      <x:c r="G90" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01; NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="H90" s="24" t="str">
+        <x:v>https://drive.google.com/file/d/10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u/view?usp=drivesdk</x:v>
+      </x:c>
+      <x:c r="I90" s="24" t="str">
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/03-ios.md</x:v>
+      </x:c>
+      <x:c r="J90" s="24" t="str">
+        <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
+      </x:c>
+      <x:c r="K90" s="24" t="str">
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+      </x:c>
+      <x:c r="L90" s="24" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="110" customHeight="1">
+      <x:c r="A91" s="24" t="str">
+        <x:v>DOC-076</x:v>
+      </x:c>
+      <x:c r="B91" s="24" t="str">
+        <x:v>04 — Chạy API và app native</x:v>
+      </x:c>
+      <x:c r="C91" s="24" t="str">
+        <x:v>Hướng dẫn phát triển</x:v>
+      </x:c>
+      <x:c r="D91" s="24" t="str">
+        <x:v>v1.1</x:v>
+      </x:c>
+      <x:c r="E91" s="24" t="str">
+        <x:v>Nguồn Markdown</x:v>
+      </x:c>
+      <x:c r="F91" s="24" t="str">
+        <x:v>Mới nhất</x:v>
+      </x:c>
+      <x:c r="G91" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01; NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="H91" s="24" t="str">
+        <x:v>https://drive.google.com/file/d/10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u/view?usp=drivesdk</x:v>
+      </x:c>
+      <x:c r="I91" s="24" t="str">
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/04-chay-app.md</x:v>
+      </x:c>
+      <x:c r="J91" s="24" t="str">
+        <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
+      </x:c>
+      <x:c r="K91" s="24" t="str">
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+      </x:c>
+      <x:c r="L91" s="24" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="110" customHeight="1">
+      <x:c r="A92" s="24" t="str">
+        <x:v>DOC-077</x:v>
+      </x:c>
+      <x:c r="B92" s="24" t="str">
+        <x:v>05 — Kết nối MCP hỗ trợ phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C92" s="24" t="str">
+        <x:v>Hướng dẫn phát triển</x:v>
+      </x:c>
+      <x:c r="D92" s="24" t="str">
+        <x:v>v1.0</x:v>
+      </x:c>
+      <x:c r="E92" s="24" t="str">
+        <x:v>Nguồn Markdown</x:v>
+      </x:c>
+      <x:c r="F92" s="24" t="str">
+        <x:v>Mới nhất</x:v>
+      </x:c>
+      <x:c r="G92" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="H92" s="24" t="str">
+        <x:v>https://drive.google.com/file/d/10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u/view?usp=drivesdk</x:v>
+      </x:c>
+      <x:c r="I92" s="24" t="str">
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/05-mcp.md</x:v>
+      </x:c>
+      <x:c r="J92" s="24" t="str">
+        <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
+      </x:c>
+      <x:c r="K92" s="24" t="str">
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+      </x:c>
+      <x:c r="L92" s="24" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="110" customHeight="1">
+      <x:c r="A93" s="24" t="str">
+        <x:v>DOC-078</x:v>
+      </x:c>
+      <x:c r="B93" s="24" t="str">
+        <x:v>06 — Kiểm thử native, đọc log và ghi bằng chứng</x:v>
+      </x:c>
+      <x:c r="C93" s="24" t="str">
+        <x:v>Hướng dẫn phát triển</x:v>
+      </x:c>
+      <x:c r="D93" s="24" t="str">
+        <x:v>v1.0</x:v>
+      </x:c>
+      <x:c r="E93" s="24" t="str">
+        <x:v>Nguồn Markdown</x:v>
+      </x:c>
+      <x:c r="F93" s="24" t="str">
+        <x:v>Mới nhất</x:v>
+      </x:c>
+      <x:c r="G93" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="H93" s="24" t="str">
+        <x:v>https://drive.google.com/file/d/10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u/view?usp=drivesdk</x:v>
+      </x:c>
+      <x:c r="I93" s="24" t="str">
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/06-kiem-thu-log.md</x:v>
+      </x:c>
+      <x:c r="J93" s="24" t="str">
+        <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
+      </x:c>
+      <x:c r="K93" s="24" t="str">
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+      </x:c>
+      <x:c r="L93" s="24" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="110" customHeight="1">
+      <x:c r="A94" s="24" t="str">
+        <x:v>DOC-079</x:v>
+      </x:c>
+      <x:c r="B94" s="24" t="str">
+        <x:v>07 — Kế hoạch hoàn thiện khung app trước nghiệp vụ</x:v>
+      </x:c>
+      <x:c r="C94" s="24" t="str">
+        <x:v>Hướng dẫn phát triển</x:v>
+      </x:c>
+      <x:c r="D94" s="24" t="str">
+        <x:v>v1.1</x:v>
+      </x:c>
+      <x:c r="E94" s="24" t="str">
+        <x:v>Nguồn Markdown</x:v>
+      </x:c>
+      <x:c r="F94" s="24" t="str">
+        <x:v>Mới nhất</x:v>
+      </x:c>
+      <x:c r="G94" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01; NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="H94" s="24" t="str">
+        <x:v>https://drive.google.com/file/d/10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u/view?usp=drivesdk</x:v>
+      </x:c>
+      <x:c r="I94" s="24" t="str">
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/07-ke-hoach-khung-app.md</x:v>
+      </x:c>
+      <x:c r="J94" s="24" t="str">
+        <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
+      </x:c>
+      <x:c r="K94" s="24" t="str">
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+      </x:c>
+      <x:c r="L94" s="24" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="110" customHeight="1">
+      <x:c r="A95" s="24" t="str">
+        <x:v>DOC-080</x:v>
+      </x:c>
+      <x:c r="B95" s="24" t="str">
+        <x:v>08 — Xử lý lỗi theo nơi phát sinh</x:v>
+      </x:c>
+      <x:c r="C95" s="24" t="str">
+        <x:v>Hướng dẫn phát triển</x:v>
+      </x:c>
+      <x:c r="D95" s="24" t="str">
+        <x:v>v1.1</x:v>
+      </x:c>
+      <x:c r="E95" s="24" t="str">
+        <x:v>Nguồn Markdown</x:v>
+      </x:c>
+      <x:c r="F95" s="24" t="str">
+        <x:v>Mới nhất</x:v>
+      </x:c>
+      <x:c r="G95" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01; NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="H95" s="24" t="str">
+        <x:v>https://drive.google.com/file/d/10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u/view?usp=drivesdk</x:v>
+      </x:c>
+      <x:c r="I95" s="24" t="str">
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/08-xu-ly-loi.md</x:v>
+      </x:c>
+      <x:c r="J95" s="24" t="str">
+        <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
+      </x:c>
+      <x:c r="K95" s="24" t="str">
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+      </x:c>
+      <x:c r="L95" s="24" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="110" customHeight="1">
+      <x:c r="A96" s="24" t="str">
+        <x:v>DOC-081</x:v>
+      </x:c>
+      <x:c r="B96" s="24" t="str">
+        <x:v>Gói hướng dẫn phát triển mobile v1.1</x:v>
+      </x:c>
+      <x:c r="C96" s="24" t="str">
+        <x:v>Hướng dẫn phát triển</x:v>
+      </x:c>
+      <x:c r="D96" s="24" t="str">
+        <x:v>v1.1</x:v>
+      </x:c>
+      <x:c r="E96" s="24" t="str">
+        <x:v>Gói xuất</x:v>
+      </x:c>
+      <x:c r="F96" s="24" t="str">
+        <x:v>Mới nhất</x:v>
+      </x:c>
+      <x:c r="G96" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01; NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="H96" s="24" t="str">
+        <x:v>https://drive.google.com/file/d/10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u/view?usp=drivesdk</x:v>
+      </x:c>
+      <x:c r="I96" s="24" t="str">
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/huong-dan-mobile-v1.1.zip</x:v>
+      </x:c>
+      <x:c r="J96" s="24" t="str">
+        <x:v>9 Markdown hiện hành; v1.0 giữ lịch sử, đã thay thế</x:v>
+      </x:c>
+      <x:c r="K96" s="24" t="str">
+        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+      </x:c>
+      <x:c r="L96" s="24" t="n">
+        <x:v>46294</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3868,81 +4272,81 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="R0e0ea06ec95c4239"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R2993c2dbee8e4715"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="Rcf90c67a09ee4043"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="R232f18a296134ce7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="R4241635c91b94b6d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="R9aa1f91a70d94b77"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="Rb2bf539e90b1427e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R9190cd05b2154498"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="Rf487ec837be54c5f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="Rd98212fe91c34289"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="R893c6c418c9d40a7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="Re54f25b39d334383"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="R75f4ab2ca0c744c7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="R5c4ce04a77584ee5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="R45321951c6a94376"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="R31364b6ccb3f4ad5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="Rf8138b5102304ca5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="R5f4ff2cc4cb740cd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="R4868f0de14e04889"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="Rb9bf8ce3dace43cb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="Reb618d44f0b94542"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="Rb684c77e2a454938"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="R921917e0de114691"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="R39eb590dd3f940d0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="Rc6432f6c91684f0b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="R774b7a5197fa4410"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="R5c10ff1bfb2a43d4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="Rb8a3e5a3aebb49b4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="Rd21c7647f4be48e8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R32907f91bb274c21"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="Rb9b190d707f84dbd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="R22442571d2d44659"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R25da1f2869254ef2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R02f17c9b37604197"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="R55e26d7c82ae438c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="Rf7e92801cb7b4645"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="Rd00f54816bc94f2b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="R60a0885ad05d407d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="Rdd06caccbb294bc0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="R8351a58771074bf5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="R6291422096e84392"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="Rcbd18d5341694662"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="R40d934ed533d4f80"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="Rb70ea6e1d3e442f8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="R497efdc7f828445c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="Rd00a986aff2448ca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="Ra628313e15a84dcc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="R5d98a45f99f7404c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="R6e867fb3b67e4414"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="R69b5807c1ea84587"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="Ra19e1489d6a24bfa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="R100d05fa27d64085"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="R6568905699e84bf2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="Re24ebcf213874499"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="Rfb3d5a6e04274816"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="R43ee00299f6f4da9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="R07aa0f19dd374a3f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="R3b11d0160e93489c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="Reaf8da3b54ca408f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="R62cbbae323e64842"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="Rf2e06fb4e3cb4173"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="R2248801f36934993"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="R5a128e7800c642e1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="R546b11a001ff40e5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="R7d26d799820c42c6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="Ra68e7370228f4ba2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="R173e5f8156c84d37"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="Rd15ff254ae2a4c1b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="Rc3e2fe4cbef24c31"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="Rddace0a9895149bd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="R4784433d490a459c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="Re224eae1e74348e3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R546785db0cae47ed"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="R508bedfc088d4ab0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="R616778eb3f4048df"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="R1b211813d46540cf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="R0468122d78894ffd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="R15bd6f35db8b416c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R3060d95295644859"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="Rc44fea8e9c484584"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="Ra272775f4a1c4a4b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="Rfa95c8d2df934b7f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="Ra134f6f1cbe2423c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="Rb3da56f78ac64aea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="Rbce77a51bf844789"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="R0e68e0d0f572450a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="Rc8213526136a4798"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="R365e0d2671e44722"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="R8cacb40c99034a69"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="Rcf27fd27d4194cb3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="R8aebba1aa2fb4045"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="R1f6b1585ce4a45b9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="R5a2bec1a68c24739"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="Rc854c8764a284160"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="Rbdb62bda8e624d2e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="R53b05c0b70474353"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="Rb0bc34108a60460a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="R1260c11803ac42a2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="R19ff43afc3b64e14"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="Re9d5b186b42f4bec"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R84210047cfd44006"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="Rb9c8d6c1a10b425a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="R939c02632a664f71"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R5a4d4b3a6b414e2f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R3ee6d02c08d449c0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="R5d0170d806ad4a15"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="R674b42d1dec14a95"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="R41d80d412a2547ed"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="R453a8ee6b1b34c4e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="R406c1fb2358146bc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="R403772f3c3ca478d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="R401c4fd87279444f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="R34bbc39c50b14925"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="R317e76c04ef1448a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="Rfa967a9e5bd84e4a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="R9c005adb2d3d4ae9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="R44a89ac8e2404ef0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="Rb90ca3edc23f4239"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="Re94f0ed7dce54493"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="Rd75dabe6859a41b6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="Rd1ff5adf9baa4958"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="R2f115f07255d406a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="R51f9588e829a4a86"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="R703a126e8def4dc5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="R11e63641bd4848b5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="R7a7730ccbd114fde"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="Rf191848d6b874690"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="R6b5a56cb219e404b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="Rdba631acb3e24bbd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="R4e1e8c5c506e4d4e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="R74d9315f9f0842d0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="Ra3646439ef604f1f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="R2d51a4675bcd4f7d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="Rf840bf6864f54967"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="Rd59e04d1542244bf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="Ra7dcbfc41c27401b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="R943c29438f6048fd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="R542dd4e85d084509"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="R8737c8b9b5134a2a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="R730f6b542c3448da"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="Rc28b580037d14c3f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="R56c21a64f49148e9"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bdb21b069874527"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6be0ea4b5f0748be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20175,10 +20579,610 @@
         <x:v>Đối chiếu source/test/reports, OpenAPI/QA/RTM/backlog, DOC-065/066/069/070 và ZIP/Drive</x:v>
       </x:c>
     </x:row>
+    <x:row r="814" ht="80" customHeight="1">
+      <x:c r="A814" s="24" t="str">
+        <x:v>F17</x:v>
+      </x:c>
+      <x:c r="B814" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C814" s="24" t="str">
+        <x:v>DOC-072</x:v>
+      </x:c>
+      <x:c r="D814" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E814" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F814" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="815" ht="80" customHeight="1">
+      <x:c r="A815" s="24" t="str">
+        <x:v>F18</x:v>
+      </x:c>
+      <x:c r="B815" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C815" s="24" t="str">
+        <x:v>DOC-072</x:v>
+      </x:c>
+      <x:c r="D815" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E815" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F815" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="816" ht="80" customHeight="1">
+      <x:c r="A816" s="24" t="str">
+        <x:v>F20</x:v>
+      </x:c>
+      <x:c r="B816" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C816" s="24" t="str">
+        <x:v>DOC-072</x:v>
+      </x:c>
+      <x:c r="D816" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E816" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F816" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="817" ht="80" customHeight="1">
+      <x:c r="A817" s="24" t="str">
+        <x:v>F17</x:v>
+      </x:c>
+      <x:c r="B817" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C817" s="24" t="str">
+        <x:v>DOC-073</x:v>
+      </x:c>
+      <x:c r="D817" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E817" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F817" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="818" ht="80" customHeight="1">
+      <x:c r="A818" s="24" t="str">
+        <x:v>F18</x:v>
+      </x:c>
+      <x:c r="B818" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C818" s="24" t="str">
+        <x:v>DOC-073</x:v>
+      </x:c>
+      <x:c r="D818" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E818" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F818" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="819" ht="80" customHeight="1">
+      <x:c r="A819" s="24" t="str">
+        <x:v>F20</x:v>
+      </x:c>
+      <x:c r="B819" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C819" s="24" t="str">
+        <x:v>DOC-073</x:v>
+      </x:c>
+      <x:c r="D819" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E819" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F819" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="820" ht="80" customHeight="1">
+      <x:c r="A820" s="24" t="str">
+        <x:v>F17</x:v>
+      </x:c>
+      <x:c r="B820" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C820" s="24" t="str">
+        <x:v>DOC-074</x:v>
+      </x:c>
+      <x:c r="D820" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E820" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F820" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="821" ht="80" customHeight="1">
+      <x:c r="A821" s="24" t="str">
+        <x:v>F18</x:v>
+      </x:c>
+      <x:c r="B821" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C821" s="24" t="str">
+        <x:v>DOC-074</x:v>
+      </x:c>
+      <x:c r="D821" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E821" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F821" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="822" ht="80" customHeight="1">
+      <x:c r="A822" s="24" t="str">
+        <x:v>F20</x:v>
+      </x:c>
+      <x:c r="B822" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C822" s="24" t="str">
+        <x:v>DOC-074</x:v>
+      </x:c>
+      <x:c r="D822" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E822" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F822" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="823" ht="80" customHeight="1">
+      <x:c r="A823" s="24" t="str">
+        <x:v>F17</x:v>
+      </x:c>
+      <x:c r="B823" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C823" s="24" t="str">
+        <x:v>DOC-075</x:v>
+      </x:c>
+      <x:c r="D823" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E823" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F823" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="824" ht="80" customHeight="1">
+      <x:c r="A824" s="24" t="str">
+        <x:v>F18</x:v>
+      </x:c>
+      <x:c r="B824" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C824" s="24" t="str">
+        <x:v>DOC-075</x:v>
+      </x:c>
+      <x:c r="D824" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E824" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F824" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="825" ht="80" customHeight="1">
+      <x:c r="A825" s="24" t="str">
+        <x:v>F20</x:v>
+      </x:c>
+      <x:c r="B825" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C825" s="24" t="str">
+        <x:v>DOC-075</x:v>
+      </x:c>
+      <x:c r="D825" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E825" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F825" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="826" ht="80" customHeight="1">
+      <x:c r="A826" s="24" t="str">
+        <x:v>F17</x:v>
+      </x:c>
+      <x:c r="B826" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C826" s="24" t="str">
+        <x:v>DOC-076</x:v>
+      </x:c>
+      <x:c r="D826" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E826" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F826" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="827" ht="80" customHeight="1">
+      <x:c r="A827" s="24" t="str">
+        <x:v>F18</x:v>
+      </x:c>
+      <x:c r="B827" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C827" s="24" t="str">
+        <x:v>DOC-076</x:v>
+      </x:c>
+      <x:c r="D827" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E827" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F827" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="828" ht="80" customHeight="1">
+      <x:c r="A828" s="24" t="str">
+        <x:v>F20</x:v>
+      </x:c>
+      <x:c r="B828" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C828" s="24" t="str">
+        <x:v>DOC-076</x:v>
+      </x:c>
+      <x:c r="D828" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E828" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F828" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="829" ht="80" customHeight="1">
+      <x:c r="A829" s="24" t="str">
+        <x:v>F17</x:v>
+      </x:c>
+      <x:c r="B829" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C829" s="24" t="str">
+        <x:v>DOC-077</x:v>
+      </x:c>
+      <x:c r="D829" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E829" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F829" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="830" ht="80" customHeight="1">
+      <x:c r="A830" s="24" t="str">
+        <x:v>F18</x:v>
+      </x:c>
+      <x:c r="B830" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C830" s="24" t="str">
+        <x:v>DOC-077</x:v>
+      </x:c>
+      <x:c r="D830" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E830" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F830" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="831" ht="80" customHeight="1">
+      <x:c r="A831" s="24" t="str">
+        <x:v>F20</x:v>
+      </x:c>
+      <x:c r="B831" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C831" s="24" t="str">
+        <x:v>DOC-077</x:v>
+      </x:c>
+      <x:c r="D831" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E831" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F831" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="832" ht="80" customHeight="1">
+      <x:c r="A832" s="24" t="str">
+        <x:v>F17</x:v>
+      </x:c>
+      <x:c r="B832" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C832" s="24" t="str">
+        <x:v>DOC-078</x:v>
+      </x:c>
+      <x:c r="D832" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E832" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F832" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="833" ht="80" customHeight="1">
+      <x:c r="A833" s="24" t="str">
+        <x:v>F18</x:v>
+      </x:c>
+      <x:c r="B833" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C833" s="24" t="str">
+        <x:v>DOC-078</x:v>
+      </x:c>
+      <x:c r="D833" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E833" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F833" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="834" ht="80" customHeight="1">
+      <x:c r="A834" s="24" t="str">
+        <x:v>F20</x:v>
+      </x:c>
+      <x:c r="B834" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C834" s="24" t="str">
+        <x:v>DOC-078</x:v>
+      </x:c>
+      <x:c r="D834" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E834" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F834" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="835" ht="80" customHeight="1">
+      <x:c r="A835" s="24" t="str">
+        <x:v>F17</x:v>
+      </x:c>
+      <x:c r="B835" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C835" s="24" t="str">
+        <x:v>DOC-079</x:v>
+      </x:c>
+      <x:c r="D835" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E835" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F835" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="836" ht="80" customHeight="1">
+      <x:c r="A836" s="24" t="str">
+        <x:v>F18</x:v>
+      </x:c>
+      <x:c r="B836" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C836" s="24" t="str">
+        <x:v>DOC-079</x:v>
+      </x:c>
+      <x:c r="D836" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E836" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F836" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="837" ht="80" customHeight="1">
+      <x:c r="A837" s="24" t="str">
+        <x:v>F20</x:v>
+      </x:c>
+      <x:c r="B837" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C837" s="24" t="str">
+        <x:v>DOC-079</x:v>
+      </x:c>
+      <x:c r="D837" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E837" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F837" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="838" ht="80" customHeight="1">
+      <x:c r="A838" s="24" t="str">
+        <x:v>F17</x:v>
+      </x:c>
+      <x:c r="B838" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C838" s="24" t="str">
+        <x:v>DOC-080</x:v>
+      </x:c>
+      <x:c r="D838" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E838" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F838" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="839" ht="80" customHeight="1">
+      <x:c r="A839" s="24" t="str">
+        <x:v>F18</x:v>
+      </x:c>
+      <x:c r="B839" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C839" s="24" t="str">
+        <x:v>DOC-080</x:v>
+      </x:c>
+      <x:c r="D839" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E839" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F839" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="840" ht="80" customHeight="1">
+      <x:c r="A840" s="24" t="str">
+        <x:v>F20</x:v>
+      </x:c>
+      <x:c r="B840" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C840" s="24" t="str">
+        <x:v>DOC-080</x:v>
+      </x:c>
+      <x:c r="D840" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E840" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F840" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="841" ht="80" customHeight="1">
+      <x:c r="A841" s="24" t="str">
+        <x:v>F17</x:v>
+      </x:c>
+      <x:c r="B841" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C841" s="24" t="str">
+        <x:v>DOC-081</x:v>
+      </x:c>
+      <x:c r="D841" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E841" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F841" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="842" ht="80" customHeight="1">
+      <x:c r="A842" s="24" t="str">
+        <x:v>F18</x:v>
+      </x:c>
+      <x:c r="B842" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C842" s="24" t="str">
+        <x:v>DOC-081</x:v>
+      </x:c>
+      <x:c r="D842" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E842" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F842" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="843" ht="80" customHeight="1">
+      <x:c r="A843" s="24" t="str">
+        <x:v>F20</x:v>
+      </x:c>
+      <x:c r="B843" s="24" t="str">
+        <x:v>Môi trường và hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C843" s="24" t="str">
+        <x:v>DOC-081</x:v>
+      </x:c>
+      <x:c r="D843" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="E843" s="24" t="str">
+        <x:v>Khi đổi SDK/toolchain, máy phát triển hoặc cách chạy/test</x:v>
+      </x:c>
+      <x:c r="F843" s="24" t="str">
+        <x:v>Đối chiếu source hiện hành, DOC-072–081; tái tạo ZIP và đọc lại Drive; giữ riêng kết quả thực thi.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd945b1a595a4fe6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15f16b18190e4562"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21412,14 +22416,86 @@
         <x:v>46293</x:v>
       </x:c>
     </x:row>
-    <x:row r="57">
-      <x:c r="G57" s="11"/>
-    </x:row>
-    <x:row r="58">
-      <x:c r="G58" s="11"/>
-    </x:row>
-    <x:row r="59">
-      <x:c r="G59" s="11"/>
+    <x:row r="57" ht="150" customHeight="1">
+      <x:c r="A57" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="B57" s="24" t="str">
+        <x:v>Tạo thư mục hướng dẫn phát triển mobile</x:v>
+      </x:c>
+      <x:c r="C57" s="24" t="str">
+        <x:v>Đã chốt</x:v>
+      </x:c>
+      <x:c r="D57" s="24" t="str">
+        <x:v>Chủ dự án yêu cầu hướng dẫn chi tiết và báo đã nâng macOS27; đã kiểm sw_vers27.0. Tạo docs/huong-dan-mobile và đăng ký tài liệu. Không tự suy ra đã cài tool, triển khai native hoặc duyệt thư viện navigation.</x:v>
+      </x:c>
+      <x:c r="E57" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="F57" s="24" t="str">
+        <x:v>Yêu cầu trực tiếp29/09/2026; DOC-072–081 v1.0; macOS27.0 build26A428; Xcode/Android SDK/Java/Maestro chưa sẵn sàng.</x:v>
+      </x:c>
+      <x:c r="G57" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="85" customHeight="1">
+      <x:c r="A58" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B58" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Dùng docs, bỏ lối tắt outputs</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C58" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Đã chốt</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D58" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Chủ dự án yêu cầu chỉ giữ một đường dẫn tài liệu. Bỏ symlink outputs, giữ docs; apps/ui trỏ trực tiếp ui-ux/prototype. Cập nhật đường dẫn hiện hành, giữ lịch sử; không mở rộng sang xóa các alias khác hoặc ZIP.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E58" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F17/F18/F20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F58" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Yêu cầu trực tiếp 29/09/2026; README v0.4, DOC-064 v1.4, DOC-065 v1.5, DOC-070 v1.2; kiểm symlink, bảo toàn file docs, cú pháp helper và ZIP parity.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G58" s="11">
+        <x:v>46294</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="120" customHeight="1">
+      <x:c r="A59" s="24" t="str">
+        <x:v>NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="B59" s="24" t="str">
+        <x:v>Kiểm môi trường và triển khai development build phần B</x:v>
+      </x:c>
+      <x:c r="C59" s="24" t="str">
+        <x:v>Đã chốt</x:v>
+      </x:c>
+      <x:c r="D59" s="24" t="str">
+        <x:v>Chủ dự án xác nhận đã cài Android/iOS, mở hai máy ảo và giao Codex kiểm rồi làm phần B. Thực hiện CNG/dev-client, ID/scheme, HTTP Debug-only và scripts; chưa build/cài binary hoặc nghiệm thu native E2E, không production/tiền thật.</x:v>
+      </x:c>
+      <x:c r="E59" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="F59" s="24" t="str">
+        <x:v>Yêu cầu trực tiếp29/09/2026; DOC-076 v1.1; preflight và generated config/tests PASS. Chưa commit/push.</x:v>
+      </x:c>
+      <x:c r="G59" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="G60" s="11"/>
@@ -24247,7 +25323,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c0bb58d82ef44fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51f8dead372c41b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39025,110 +40101,1497 @@
         <x:v>Không áp dụng</x:v>
       </x:c>
     </x:row>
-    <x:row r="389">
-      <x:c r="I389" s="11"/>
-    </x:row>
-    <x:row r="390">
-      <x:c r="I390" s="11"/>
-    </x:row>
-    <x:row r="391">
-      <x:c r="I391" s="11"/>
-    </x:row>
-    <x:row r="392">
-      <x:c r="I392" s="11"/>
-    </x:row>
-    <x:row r="393">
-      <x:c r="I393" s="11"/>
-    </x:row>
-    <x:row r="394">
-      <x:c r="I394" s="11"/>
-    </x:row>
-    <x:row r="395">
-      <x:c r="I395" s="11"/>
-    </x:row>
-    <x:row r="396">
-      <x:c r="I396" s="11"/>
-    </x:row>
-    <x:row r="397">
-      <x:c r="I397" s="11"/>
-    </x:row>
-    <x:row r="398">
-      <x:c r="I398" s="11"/>
-    </x:row>
-    <x:row r="399">
-      <x:c r="I399" s="11"/>
-    </x:row>
-    <x:row r="400">
-      <x:c r="I400" s="11"/>
-    </x:row>
-    <x:row r="401">
-      <x:c r="I401" s="11"/>
-    </x:row>
-    <x:row r="402">
-      <x:c r="I402" s="11"/>
-    </x:row>
-    <x:row r="403">
-      <x:c r="I403" s="11"/>
-    </x:row>
-    <x:row r="404">
-      <x:c r="I404" s="11"/>
-    </x:row>
-    <x:row r="405">
-      <x:c r="I405" s="11"/>
-    </x:row>
-    <x:row r="406">
-      <x:c r="I406" s="11"/>
-    </x:row>
-    <x:row r="407">
-      <x:c r="I407" s="11"/>
-    </x:row>
-    <x:row r="408">
-      <x:c r="I408" s="11"/>
-    </x:row>
-    <x:row r="409">
-      <x:c r="I409" s="11"/>
-    </x:row>
-    <x:row r="410">
-      <x:c r="I410" s="11"/>
-    </x:row>
-    <x:row r="411">
-      <x:c r="I411" s="11"/>
-    </x:row>
-    <x:row r="412">
-      <x:c r="I412" s="11"/>
-    </x:row>
-    <x:row r="413">
-      <x:c r="I413" s="11"/>
-    </x:row>
-    <x:row r="414">
-      <x:c r="I414" s="11"/>
-    </x:row>
-    <x:row r="415">
-      <x:c r="I415" s="11"/>
-    </x:row>
-    <x:row r="416">
-      <x:c r="I416" s="11"/>
-    </x:row>
-    <x:row r="417">
-      <x:c r="I417" s="11"/>
-    </x:row>
-    <x:row r="418">
-      <x:c r="I418" s="11"/>
-    </x:row>
-    <x:row r="419">
-      <x:c r="I419" s="11"/>
-    </x:row>
-    <x:row r="420">
-      <x:c r="I420" s="11"/>
-    </x:row>
-    <x:row r="421">
-      <x:c r="I421" s="11"/>
-    </x:row>
-    <x:row r="422">
-      <x:c r="I422" s="11"/>
-    </x:row>
-    <x:row r="423">
-      <x:c r="I423" s="11"/>
+    <x:row r="389" ht="130" customHeight="1">
+      <x:c r="A389" s="24" t="str">
+        <x:v>GUIDE-20260929</x:v>
+      </x:c>
+      <x:c r="B389" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="C389" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D389" s="24" t="str">
+        <x:v>DOC-072</x:v>
+      </x:c>
+      <x:c r="E389" s="24" t="str">
+        <x:v>Tạo hướng dẫn môi trường native, MCP và kiểm thử</x:v>
+      </x:c>
+      <x:c r="F389" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G389" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H389" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I389" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J389" s="24" t="str">
+        <x:v>DOC-072 v1.0; docs/huong-dan-mobile/README.md; 31 khối shell kiểm cú pháp; link local và ZIP parity; Drive DOC-081 đọc lại.</x:v>
+      </x:c>
+      <x:c r="K389" s="24" t="str">
+        <x:v>Không coi hướng dẫn là build/test native đã đạt.</x:v>
+      </x:c>
+      <x:c r="L389" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="390" ht="130" customHeight="1">
+      <x:c r="A390" s="24" t="str">
+        <x:v>GUIDE-20260929</x:v>
+      </x:c>
+      <x:c r="B390" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="C390" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D390" s="24" t="str">
+        <x:v>DOC-073</x:v>
+      </x:c>
+      <x:c r="E390" s="24" t="str">
+        <x:v>Tạo hướng dẫn môi trường native, MCP và kiểm thử</x:v>
+      </x:c>
+      <x:c r="F390" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G390" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H390" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I390" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J390" s="24" t="str">
+        <x:v>DOC-073 v1.0; docs/huong-dan-mobile/01-chuan-bi-may.md; 31 khối shell kiểm cú pháp; link local và ZIP parity; Drive DOC-081 đọc lại.</x:v>
+      </x:c>
+      <x:c r="K390" s="24" t="str">
+        <x:v>Không coi hướng dẫn là build/test native đã đạt.</x:v>
+      </x:c>
+      <x:c r="L390" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="391" ht="130" customHeight="1">
+      <x:c r="A391" s="24" t="str">
+        <x:v>GUIDE-20260929</x:v>
+      </x:c>
+      <x:c r="B391" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="C391" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D391" s="24" t="str">
+        <x:v>DOC-074</x:v>
+      </x:c>
+      <x:c r="E391" s="24" t="str">
+        <x:v>Tạo hướng dẫn môi trường native, MCP và kiểm thử</x:v>
+      </x:c>
+      <x:c r="F391" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G391" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H391" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I391" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J391" s="24" t="str">
+        <x:v>DOC-074 v1.0; docs/huong-dan-mobile/02-android.md; 31 khối shell kiểm cú pháp; link local và ZIP parity; Drive DOC-081 đọc lại.</x:v>
+      </x:c>
+      <x:c r="K391" s="24" t="str">
+        <x:v>Không coi hướng dẫn là build/test native đã đạt.</x:v>
+      </x:c>
+      <x:c r="L391" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="392" ht="130" customHeight="1">
+      <x:c r="A392" s="24" t="str">
+        <x:v>GUIDE-20260929</x:v>
+      </x:c>
+      <x:c r="B392" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="C392" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D392" s="24" t="str">
+        <x:v>DOC-075</x:v>
+      </x:c>
+      <x:c r="E392" s="24" t="str">
+        <x:v>Tạo hướng dẫn môi trường native, MCP và kiểm thử</x:v>
+      </x:c>
+      <x:c r="F392" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G392" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H392" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I392" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J392" s="24" t="str">
+        <x:v>DOC-075 v1.0; docs/huong-dan-mobile/03-ios.md; 31 khối shell kiểm cú pháp; link local và ZIP parity; Drive DOC-081 đọc lại.</x:v>
+      </x:c>
+      <x:c r="K392" s="24" t="str">
+        <x:v>Không coi hướng dẫn là build/test native đã đạt.</x:v>
+      </x:c>
+      <x:c r="L392" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="393" ht="130" customHeight="1">
+      <x:c r="A393" s="24" t="str">
+        <x:v>GUIDE-20260929</x:v>
+      </x:c>
+      <x:c r="B393" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="C393" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D393" s="24" t="str">
+        <x:v>DOC-076</x:v>
+      </x:c>
+      <x:c r="E393" s="24" t="str">
+        <x:v>Tạo hướng dẫn môi trường native, MCP và kiểm thử</x:v>
+      </x:c>
+      <x:c r="F393" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G393" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H393" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I393" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J393" s="24" t="str">
+        <x:v>DOC-076 v1.0; docs/huong-dan-mobile/04-chay-app.md; 31 khối shell kiểm cú pháp; link local và ZIP parity; Drive DOC-081 đọc lại.</x:v>
+      </x:c>
+      <x:c r="K393" s="24" t="str">
+        <x:v>Không coi hướng dẫn là build/test native đã đạt.</x:v>
+      </x:c>
+      <x:c r="L393" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="394" ht="130" customHeight="1">
+      <x:c r="A394" s="24" t="str">
+        <x:v>GUIDE-20260929</x:v>
+      </x:c>
+      <x:c r="B394" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="C394" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D394" s="24" t="str">
+        <x:v>DOC-077</x:v>
+      </x:c>
+      <x:c r="E394" s="24" t="str">
+        <x:v>Tạo hướng dẫn môi trường native, MCP và kiểm thử</x:v>
+      </x:c>
+      <x:c r="F394" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G394" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H394" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I394" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J394" s="24" t="str">
+        <x:v>DOC-077 v1.0; docs/huong-dan-mobile/05-mcp.md; 31 khối shell kiểm cú pháp; link local và ZIP parity; Drive DOC-081 đọc lại.</x:v>
+      </x:c>
+      <x:c r="K394" s="24" t="str">
+        <x:v>Không coi hướng dẫn là build/test native đã đạt.</x:v>
+      </x:c>
+      <x:c r="L394" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="395" ht="130" customHeight="1">
+      <x:c r="A395" s="24" t="str">
+        <x:v>GUIDE-20260929</x:v>
+      </x:c>
+      <x:c r="B395" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="C395" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D395" s="24" t="str">
+        <x:v>DOC-078</x:v>
+      </x:c>
+      <x:c r="E395" s="24" t="str">
+        <x:v>Tạo hướng dẫn môi trường native, MCP và kiểm thử</x:v>
+      </x:c>
+      <x:c r="F395" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G395" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H395" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I395" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J395" s="24" t="str">
+        <x:v>DOC-078 v1.0; docs/huong-dan-mobile/06-kiem-thu-log.md; 31 khối shell kiểm cú pháp; link local và ZIP parity; Drive DOC-081 đọc lại.</x:v>
+      </x:c>
+      <x:c r="K395" s="24" t="str">
+        <x:v>Không coi hướng dẫn là build/test native đã đạt.</x:v>
+      </x:c>
+      <x:c r="L395" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="396" ht="130" customHeight="1">
+      <x:c r="A396" s="24" t="str">
+        <x:v>GUIDE-20260929</x:v>
+      </x:c>
+      <x:c r="B396" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="C396" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D396" s="24" t="str">
+        <x:v>DOC-079</x:v>
+      </x:c>
+      <x:c r="E396" s="24" t="str">
+        <x:v>Tạo hướng dẫn môi trường native, MCP và kiểm thử</x:v>
+      </x:c>
+      <x:c r="F396" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G396" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H396" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I396" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J396" s="24" t="str">
+        <x:v>DOC-079 v1.0; docs/huong-dan-mobile/07-ke-hoach-khung-app.md; 31 khối shell kiểm cú pháp; link local và ZIP parity; Drive DOC-081 đọc lại.</x:v>
+      </x:c>
+      <x:c r="K396" s="24" t="str">
+        <x:v>Không coi hướng dẫn là build/test native đã đạt.</x:v>
+      </x:c>
+      <x:c r="L396" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="397" ht="130" customHeight="1">
+      <x:c r="A397" s="24" t="str">
+        <x:v>GUIDE-20260929</x:v>
+      </x:c>
+      <x:c r="B397" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="C397" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D397" s="24" t="str">
+        <x:v>DOC-080</x:v>
+      </x:c>
+      <x:c r="E397" s="24" t="str">
+        <x:v>Tạo hướng dẫn môi trường native, MCP và kiểm thử</x:v>
+      </x:c>
+      <x:c r="F397" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G397" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H397" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I397" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J397" s="24" t="str">
+        <x:v>DOC-080 v1.0; docs/huong-dan-mobile/08-xu-ly-loi.md; 31 khối shell kiểm cú pháp; link local và ZIP parity; Drive DOC-081 đọc lại.</x:v>
+      </x:c>
+      <x:c r="K397" s="24" t="str">
+        <x:v>Không coi hướng dẫn là build/test native đã đạt.</x:v>
+      </x:c>
+      <x:c r="L397" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="398" ht="130" customHeight="1">
+      <x:c r="A398" s="24" t="str">
+        <x:v>GUIDE-20260929</x:v>
+      </x:c>
+      <x:c r="B398" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="C398" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D398" s="24" t="str">
+        <x:v>DOC-081</x:v>
+      </x:c>
+      <x:c r="E398" s="24" t="str">
+        <x:v>Tạo hướng dẫn môi trường native, MCP và kiểm thử</x:v>
+      </x:c>
+      <x:c r="F398" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G398" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H398" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I398" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J398" s="24" t="str">
+        <x:v>DOC-081 v1.0; docs/huong-dan-mobile/huong-dan-mobile-v1.0.zip; 31 khối shell kiểm cú pháp; link local và ZIP parity; Drive DOC-081 đọc lại.</x:v>
+      </x:c>
+      <x:c r="K398" s="24" t="str">
+        <x:v>Không coi hướng dẫn là build/test native đã đạt.</x:v>
+      </x:c>
+      <x:c r="L398" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="399" ht="130" customHeight="1">
+      <x:c r="A399" s="24" t="str">
+        <x:v>GUIDE-20260929</x:v>
+      </x:c>
+      <x:c r="B399" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="C399" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D399" s="24" t="str">
+        <x:v>DOC-054/064/065/066/069/070/071</x:v>
+      </x:c>
+      <x:c r="E399" s="24" t="str">
+        <x:v>Rà phụ thuộc hướng dẫn hiện hành</x:v>
+      </x:c>
+      <x:c r="F399" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
+      <x:c r="G399" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H399" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I399" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J399" s="24" t="str">
+        <x:v>Đã đối chiếu package/scripts/config, DOC-064/065/070/071. Không đổi code/cách chạy hiện có; guide ghi rõ bước chuẩn bị chưa thực hiện.</x:v>
+      </x:c>
+      <x:c r="K399" s="24" t="str">
+        <x:v>Giữ các runbook và ZIP kỹ thuật 28/09 làm bằng chứng theo đợt. Bộ hướng dẫn mới DOC-072–081 độc lập.</x:v>
+      </x:c>
+      <x:c r="L399" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="400" ht="130" customHeight="1">
+      <x:c r="A400" s="24" t="str">
+        <x:v>GUIDE-20260929</x:v>
+      </x:c>
+      <x:c r="B400" s="24" t="str">
+        <x:v>MOBILE-GUIDE-01</x:v>
+      </x:c>
+      <x:c r="C400" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D400" s="24" t="str">
+        <x:v>BRD/PRD/FR/SRS/UX/ERD/API/QA/prototype</x:v>
+      </x:c>
+      <x:c r="E400" s="24" t="str">
+        <x:v>Rà tác động nghiệp vụ và bản xuất</x:v>
+      </x:c>
+      <x:c r="F400" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
+      <x:c r="G400" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H400" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I400" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J400" s="24" t="str">
+        <x:v>Chỉ bổ sung hướng dẫn cài/chạy/test; không đổi contract, DB, quyền, nghiệp vụ hoặc kết quả nghiệm thu.</x:v>
+      </x:c>
+      <x:c r="K400" s="24" t="str">
+        <x:v>Không tạo lại HTML/localhost/ZIP thiết kế vì nguồn không đổi; guide chỉ có Markdown và DOC-081 ZIP.</x:v>
+      </x:c>
+      <x:c r="L400" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="401" ht="85" customHeight="1">
+      <x:c r="A401" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-20260929</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B401" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C401" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F17/F18/F20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D401" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">DOC-011</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E401" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Bỏ alias outputs; đồng bộ đường dẫn và bản xuất liên quan</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F401" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Đã cập nhật</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G401" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Có</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H401" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Codex</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I401" s="11">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J401" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">v0.1.1 / PATH-01; docs/project-docs/01-danh-muc-ho-so.md; kiểm local + ZIP parity; Drive cùng ID đã đọc lại metadata/kích thước.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K401" s="24"/>
+      <x:c r="L401" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Hoàn tất</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="402" ht="85" customHeight="1">
+      <x:c r="A402" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-20260929</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B402" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C402" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F17/F18/F20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D402" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">DOC-018</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E402" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Bỏ alias outputs; đồng bộ đường dẫn và bản xuất liên quan</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F402" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Đã cập nhật</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G402" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Có</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H402" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Codex</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I402" s="11">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J402" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">v0.1.1 / PATH-01; docs/project-docs/architecture-source-v0.1.1.zip; kiểm local + ZIP parity; Drive cùng ID đã đọc lại metadata/kích thước.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K402" s="24"/>
+      <x:c r="L402" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Hoàn tất</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="403" ht="85" customHeight="1">
+      <x:c r="A403" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-20260929</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B403" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C403" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F17/F18/F20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D403" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">DOC-040</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E403" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Bỏ alias outputs; đồng bộ đường dẫn và bản xuất liên quan</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F403" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Đã cập nhật</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G403" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Có</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H403" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Codex</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I403" s="11">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J403" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">v0.1.1 / PATH-01; docs/technical-design/technical-design-v0.1.1.zip; kiểm local + ZIP parity; Drive cùng ID đã đọc lại metadata/kích thước.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K403" s="24"/>
+      <x:c r="L403" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Hoàn tất</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="404" ht="85" customHeight="1">
+      <x:c r="A404" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-20260929</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B404" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C404" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F17/F18/F20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D404" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">DOC-050</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E404" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Bỏ alias outputs; đồng bộ đường dẫn và bản xuất liên quan</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F404" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Đã cập nhật</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G404" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Có</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H404" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Codex</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I404" s="11">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J404" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">v0.15 / gói PATH-01; ui-ux/exports/UI-UX-v0.19.zip; kiểm local + ZIP parity; Drive cùng ID đã đọc lại metadata/kích thước.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K404" s="24"/>
+      <x:c r="L404" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Hoàn tất</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="405" ht="85" customHeight="1">
+      <x:c r="A405" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-20260929</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B405" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C405" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F17/F18/F20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D405" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">DOC-054</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E405" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Bỏ alias outputs; đồng bộ đường dẫn và bản xuất liên quan</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F405" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Đã cập nhật</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G405" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Có</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H405" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Codex</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I405" s="11">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J405" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">v0.4 / PATH-01; README.md trong DOC-040 và UI-UX-v0.19.zip; kiểm local + ZIP parity; Drive cùng ID đã đọc lại metadata/kích thước.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K405" s="24"/>
+      <x:c r="L405" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Hoàn tất</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="406" ht="85" customHeight="1">
+      <x:c r="A406" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-20260929</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B406" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C406" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F17/F18/F20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D406" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">DOC-064</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E406" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Bỏ alias outputs; đồng bộ đường dẫn và bản xuất liên quan</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F406" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Đã cập nhật</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G406" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Có</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H406" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Codex</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I406" s="11">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J406" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">v1.4; docs/handoff/CODEX-IMPLEMENTATION-PROMPT.md; kiểm local + ZIP parity; Drive cùng ID đã đọc lại metadata/kích thước.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K406" s="24"/>
+      <x:c r="L406" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Hoàn tất</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="407" ht="85" customHeight="1">
+      <x:c r="A407" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-20260929</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B407" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C407" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F17/F18/F20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D407" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">DOC-065</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E407" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Bỏ alias outputs; đồng bộ đường dẫn và bản xuất liên quan</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F407" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Đã cập nhật</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G407" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Có</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H407" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Codex</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I407" s="11">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J407" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">v1.5; docs/implementation/dot-1.md; kiểm local + ZIP parity; Drive cùng ID đã đọc lại metadata/kích thước.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K407" s="24"/>
+      <x:c r="L407" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Hoàn tất</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="408" ht="85" customHeight="1">
+      <x:c r="A408" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-20260929</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B408" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C408" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F17/F18/F20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D408" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">DOC-070</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E408" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Bỏ alias outputs; đồng bộ đường dẫn và bản xuất liên quan</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F408" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Đã cập nhật</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G408" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Có</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H408" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Codex</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I408" s="11">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J408" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">v1.2; docs/implementation/project-structure.md; kiểm local + ZIP parity; Drive cùng ID đã đọc lại metadata/kích thước.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K408" s="24"/>
+      <x:c r="L408" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Hoàn tất</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="409" ht="85" customHeight="1">
+      <x:c r="A409" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-20260929</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B409" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C409" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F17/F18/F20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D409" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">BRD/PRD/FR/NFR/SRS/UX/API/ERD/QA/mobile guide</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E409" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Rà phạm vi nghiệp vụ, HTML và hướng dẫn native</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F409" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Không áp dụng</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G409" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Có</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H409" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Codex</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I409" s="11">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J409" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Không đổi code app/API, contract hoặc nội dung nghiệp vụ. Đường dẫn build/outputs/apk trong hướng dẫn Android thuộc Gradle, giữ nguyên.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K409" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Thay đổi alias thư mục local; nội dung nguồn các tài liệu này không đổi.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L409" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Không áp dụng</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="410" ht="85" customHeight="1">
+      <x:c r="A410" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-20260929</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B410" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">PATH-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C410" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">F17/F18/F20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D410" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Archive / ZIP cũ / baseline / tools</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E410" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Rà lịch sử và công cụ nội bộ</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F410" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Đã cập nhật</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G410" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Có</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H410" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Codex</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I410" s="11">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J410" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Sửa helper dùng đường dẫn local hiện tại; kiểm cú pháp Python/Node. Archive, baseline, biên nhận và script migration cũ giữ nguyên; không chạy lại builder lịch sử.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K410" s="24"/>
+      <x:c r="L410" s="24" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Hoàn tất</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="411" ht="120" customHeight="1">
+      <x:c r="A411" s="24" t="str">
+        <x:v>NATIVE-B-20260929</x:v>
+      </x:c>
+      <x:c r="B411" s="24" t="str">
+        <x:v>NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="C411" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D411" s="24" t="str">
+        <x:v>DOC-065</x:v>
+      </x:c>
+      <x:c r="E411" s="24" t="str">
+        <x:v>Đồng bộ cấu hình và kết quả kiểm phần B</x:v>
+      </x:c>
+      <x:c r="F411" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G411" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H411" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I411" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J411" s="24" t="str">
+        <x:v>v1.6; /Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/implementation/dot-1.md; Drive cùng ID 1JjfKtYYgYGHlLSZCKZ21hqWiscQxoFpT; đọc lại byte/hash. DOC-076 ghi kiểm môi trường/config, không nhận là native E2E.</x:v>
+      </x:c>
+      <x:c r="K411" s="24"/>
+      <x:c r="L411" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="412" ht="120" customHeight="1">
+      <x:c r="A412" s="24" t="str">
+        <x:v>NATIVE-B-20260929</x:v>
+      </x:c>
+      <x:c r="B412" s="24" t="str">
+        <x:v>NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="C412" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D412" s="24" t="str">
+        <x:v>DOC-070</x:v>
+      </x:c>
+      <x:c r="E412" s="24" t="str">
+        <x:v>Đồng bộ cấu hình và kết quả kiểm phần B</x:v>
+      </x:c>
+      <x:c r="F412" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G412" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H412" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I412" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J412" s="24" t="str">
+        <x:v>v1.3; /Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/implementation/project-structure.md; Drive cùng ID 1pWijvZgP7U3mpjq5Wualaa1mdPCDk_Ge; đọc lại byte/hash. DOC-076 ghi kiểm môi trường/config, không nhận là native E2E.</x:v>
+      </x:c>
+      <x:c r="K412" s="24"/>
+      <x:c r="L412" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="413" ht="120" customHeight="1">
+      <x:c r="A413" s="24" t="str">
+        <x:v>NATIVE-B-20260929</x:v>
+      </x:c>
+      <x:c r="B413" s="24" t="str">
+        <x:v>NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="C413" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D413" s="24" t="str">
+        <x:v>DOC-071</x:v>
+      </x:c>
+      <x:c r="E413" s="24" t="str">
+        <x:v>Đồng bộ cấu hình và kết quả kiểm phần B</x:v>
+      </x:c>
+      <x:c r="F413" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G413" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H413" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I413" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J413" s="24" t="str">
+        <x:v>v1.1; /Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/implementation/logging-testing.md; Drive cùng ID 1m7nrDRbwKj7HPH3TQoWUIsT4zSKn_ldK; đọc lại byte/hash. DOC-076 ghi kiểm môi trường/config, không nhận là native E2E.</x:v>
+      </x:c>
+      <x:c r="K413" s="24"/>
+      <x:c r="L413" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="414" ht="120" customHeight="1">
+      <x:c r="A414" s="24" t="str">
+        <x:v>NATIVE-B-20260929</x:v>
+      </x:c>
+      <x:c r="B414" s="24" t="str">
+        <x:v>NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="C414" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D414" s="24" t="str">
+        <x:v>DOC-072</x:v>
+      </x:c>
+      <x:c r="E414" s="24" t="str">
+        <x:v>Đồng bộ cấu hình và kết quả kiểm phần B</x:v>
+      </x:c>
+      <x:c r="F414" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G414" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H414" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I414" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J414" s="24" t="str">
+        <x:v>v1.1; /Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/README.md; Drive cùng ID 10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u; đọc lại byte/hash. DOC-076 ghi kiểm môi trường/config, không nhận là native E2E.</x:v>
+      </x:c>
+      <x:c r="K414" s="24"/>
+      <x:c r="L414" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="415" ht="120" customHeight="1">
+      <x:c r="A415" s="24" t="str">
+        <x:v>NATIVE-B-20260929</x:v>
+      </x:c>
+      <x:c r="B415" s="24" t="str">
+        <x:v>NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="C415" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D415" s="24" t="str">
+        <x:v>DOC-075</x:v>
+      </x:c>
+      <x:c r="E415" s="24" t="str">
+        <x:v>Đồng bộ cấu hình và kết quả kiểm phần B</x:v>
+      </x:c>
+      <x:c r="F415" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G415" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H415" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I415" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J415" s="24" t="str">
+        <x:v>v1.1; /Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/03-ios.md; Drive cùng ID 10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u; đọc lại byte/hash. DOC-076 ghi kiểm môi trường/config, không nhận là native E2E.</x:v>
+      </x:c>
+      <x:c r="K415" s="24"/>
+      <x:c r="L415" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="416" ht="120" customHeight="1">
+      <x:c r="A416" s="24" t="str">
+        <x:v>NATIVE-B-20260929</x:v>
+      </x:c>
+      <x:c r="B416" s="24" t="str">
+        <x:v>NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="C416" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D416" s="24" t="str">
+        <x:v>DOC-076</x:v>
+      </x:c>
+      <x:c r="E416" s="24" t="str">
+        <x:v>Đồng bộ cấu hình và kết quả kiểm phần B</x:v>
+      </x:c>
+      <x:c r="F416" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G416" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H416" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I416" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J416" s="24" t="str">
+        <x:v>v1.1; /Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/04-chay-app.md; Drive cùng ID 10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u; đọc lại byte/hash. DOC-076 ghi kiểm môi trường/config, không nhận là native E2E.</x:v>
+      </x:c>
+      <x:c r="K416" s="24"/>
+      <x:c r="L416" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="417" ht="120" customHeight="1">
+      <x:c r="A417" s="24" t="str">
+        <x:v>NATIVE-B-20260929</x:v>
+      </x:c>
+      <x:c r="B417" s="24" t="str">
+        <x:v>NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="C417" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D417" s="24" t="str">
+        <x:v>DOC-079</x:v>
+      </x:c>
+      <x:c r="E417" s="24" t="str">
+        <x:v>Đồng bộ cấu hình và kết quả kiểm phần B</x:v>
+      </x:c>
+      <x:c r="F417" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G417" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H417" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I417" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J417" s="24" t="str">
+        <x:v>v1.1; /Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/07-ke-hoach-khung-app.md; Drive cùng ID 10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u; đọc lại byte/hash. DOC-076 ghi kiểm môi trường/config, không nhận là native E2E.</x:v>
+      </x:c>
+      <x:c r="K417" s="24"/>
+      <x:c r="L417" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="418" ht="120" customHeight="1">
+      <x:c r="A418" s="24" t="str">
+        <x:v>NATIVE-B-20260929</x:v>
+      </x:c>
+      <x:c r="B418" s="24" t="str">
+        <x:v>NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="C418" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D418" s="24" t="str">
+        <x:v>DOC-080</x:v>
+      </x:c>
+      <x:c r="E418" s="24" t="str">
+        <x:v>Đồng bộ cấu hình và kết quả kiểm phần B</x:v>
+      </x:c>
+      <x:c r="F418" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G418" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H418" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I418" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J418" s="24" t="str">
+        <x:v>v1.1; /Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/08-xu-ly-loi.md; Drive cùng ID 10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u; đọc lại byte/hash. DOC-076 ghi kiểm môi trường/config, không nhận là native E2E.</x:v>
+      </x:c>
+      <x:c r="K418" s="24"/>
+      <x:c r="L418" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="419" ht="120" customHeight="1">
+      <x:c r="A419" s="24" t="str">
+        <x:v>NATIVE-B-20260929</x:v>
+      </x:c>
+      <x:c r="B419" s="24" t="str">
+        <x:v>NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="C419" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D419" s="24" t="str">
+        <x:v>DOC-081</x:v>
+      </x:c>
+      <x:c r="E419" s="24" t="str">
+        <x:v>Đồng bộ cấu hình và kết quả kiểm phần B</x:v>
+      </x:c>
+      <x:c r="F419" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G419" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H419" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I419" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J419" s="24" t="str">
+        <x:v>v1.1; /Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/huong-dan-mobile-v1.1.zip; Drive cùng ID 10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u; đọc lại byte/hash. DOC-076 ghi kiểm môi trường/config, không nhận là native E2E.</x:v>
+      </x:c>
+      <x:c r="K419" s="24"/>
+      <x:c r="L419" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="420" ht="120" customHeight="1">
+      <x:c r="A420" s="24" t="str">
+        <x:v>NATIVE-B-20260929</x:v>
+      </x:c>
+      <x:c r="B420" s="24" t="str">
+        <x:v>NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="C420" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D420" s="24" t="str">
+        <x:v>DOC-018</x:v>
+      </x:c>
+      <x:c r="E420" s="24" t="str">
+        <x:v>Đồng bộ cấu hình và kết quả kiểm phần B</x:v>
+      </x:c>
+      <x:c r="F420" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G420" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H420" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I420" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J420" s="24" t="str">
+        <x:v>v0.1.1 / NATIVE-B-01; /Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/project-docs/architecture-source-v0.1.1.zip; Drive cùng ID 1QFvCWLng19VPnOoXcCZ2i0PUCsmlexMC; đọc lại byte/hash. DOC-076 ghi kiểm môi trường/config, không nhận là native E2E.</x:v>
+      </x:c>
+      <x:c r="K420" s="24"/>
+      <x:c r="L420" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="421" ht="120" customHeight="1">
+      <x:c r="A421" s="24" t="str">
+        <x:v>NATIVE-B-20260929</x:v>
+      </x:c>
+      <x:c r="B421" s="24" t="str">
+        <x:v>NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="C421" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D421" s="24" t="str">
+        <x:v>DOC-040</x:v>
+      </x:c>
+      <x:c r="E421" s="24" t="str">
+        <x:v>Đồng bộ cấu hình và kết quả kiểm phần B</x:v>
+      </x:c>
+      <x:c r="F421" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G421" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H421" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I421" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J421" s="24" t="str">
+        <x:v>v0.1.1 / NATIVE-B-01; /Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/technical-design/technical-design-v0.1.1.zip; Drive cùng ID 18z-ReFxGP-RhX5_cOVTidcHJJGFfB48D; đọc lại byte/hash. DOC-076 ghi kiểm môi trường/config, không nhận là native E2E.</x:v>
+      </x:c>
+      <x:c r="K421" s="24"/>
+      <x:c r="L421" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="422" ht="120" customHeight="1">
+      <x:c r="A422" s="24" t="str">
+        <x:v>NATIVE-B-20260929</x:v>
+      </x:c>
+      <x:c r="B422" s="24" t="str">
+        <x:v>NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="C422" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D422" s="24" t="str">
+        <x:v>DOC-054/064; BRD/PRD/FR/NFR/SRS/UX/ERD/API/QA; DOC-073/074/077/078</x:v>
+      </x:c>
+      <x:c r="E422" s="24" t="str">
+        <x:v>Rà ảnh hưởng</x:v>
+      </x:c>
+      <x:c r="F422" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
+      <x:c r="G422" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H422" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I422" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J422" s="24" t="str">
+        <x:v>Không đổi nghiệp vụ/contract/UI; handoff/README vẫn yêu cầu nghiệm thu native. Bài01 giữ snapshot ban đầu; bài02/05/06 là quy trình còn đúng. K trạng thái dẫn DOC-076 mới; không giả kết quả runtime.</x:v>
+      </x:c>
+      <x:c r="K422" s="24" t="str">
+        <x:v>Phần B cấu hình build local, không triển khai chức năng/MCP/Maestro.</x:v>
+      </x:c>
+      <x:c r="L422" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="423" ht="120" customHeight="1">
+      <x:c r="A423" s="24" t="str">
+        <x:v>NATIVE-B-20260929</x:v>
+      </x:c>
+      <x:c r="B423" s="24" t="str">
+        <x:v>NATIVE-B-01</x:v>
+      </x:c>
+      <x:c r="C423" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D423" s="24" t="str">
+        <x:v>HTML/localhost; archive; UI-UX-v0.19.zip</x:v>
+      </x:c>
+      <x:c r="E423" s="24" t="str">
+        <x:v>Rà bản phục vụ và lịch sử</x:v>
+      </x:c>
+      <x:c r="F423" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
+      <x:c r="G423" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H423" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I423" s="25" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J423" s="24" t="str">
+        <x:v>Nguồn bị sửa là Markdown/code, không có bản HTML phục vụ riêng; UI ZIP không chứa các nguồn thay đổi. Giữ ZIP mobile v1.0 làm lịch sử.</x:v>
+      </x:c>
+      <x:c r="K423" s="24" t="str">
+        <x:v>Không thay prototype/UI hoặc tài liệu lịch sử.</x:v>
+      </x:c>
+      <x:c r="L423" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
     </x:row>
     <x:row r="424">
       <x:c r="I424" s="11"/>
@@ -40875,7 +43338,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc79d16519e4a4bb4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1e5d84f4cf84a7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41117,7 +43580,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a48a53dad144706"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc86cf20cc07a4bd5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore: checkpoint mobile setup and iOS scene support
</commit_message>
<xml_diff>
--- a/docs/project-control/So-quan-ly-tai-lieu.xlsx
+++ b/docs/project-control/So-quan-ly-tai-lieu.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bat dau" sheetId="1" r:id="R0150bbbdf20e48e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh muc" sheetId="2" r:id="R8e59ba579f244fd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anh huong" sheetId="3" r:id="R8733cef6ebee4de4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quyet dinh" sheetId="4" r:id="Rb200d66dd94042c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dong bo" sheetId="5" r:id="R0bffdca58a61443a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quy trinh" sheetId="6" r:id="R8a5f932cac484ad4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bat dau" sheetId="1" r:id="Ree2c41d13e1c491b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh muc" sheetId="2" r:id="R7b961588da9c43c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anh huong" sheetId="3" r:id="R879bda15ecaf4cd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quyet dinh" sheetId="4" r:id="Rf2e38f2a70d648e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dong bo" sheetId="5" r:id="Rb954a11b73794324"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quy trinh" sheetId="6" r:id="R719ffd65792a4c6b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -215,7 +215,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="87" name="Tbl3" displayName="Tbl3" ref="A5:G59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="87" name="Tbl3" displayName="Tbl3" ref="A5:G61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Mã quyết định"/>
     <x:tableColumn id="2" name="Chủ đề"/>
@@ -230,7 +230,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="88" name="Tbl4" displayName="Tbl4" ref="A5:L423" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="88" name="Tbl4" displayName="Tbl4" ref="A5:L435" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Mã đợt"/>
     <x:tableColumn id="2" name="Quyết định"/>
@@ -489,7 +489,7 @@
     <x:row r="3">
       <x:c r="A3" s="1"/>
       <x:c r="B3" s="1" t="str">
-        <x:v>Phiên bản 1.37 · 29/09/2026 · NATIVE-B-01: kiểm môi trường Android/iOS và triển khai phần B; giữ PATH-01</x:v>
+        <x:v>Phiên bản 1.39 · 30/09/2026 · EXPO-MCP-01: kết nối Expo MCP chỉ dùng công cụ miễn phí; giữ MCP-01/NATIVE-B-01</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>
@@ -550,7 +550,7 @@
       </x:c>
       <x:c r="C8" s="13" t="n">
         <x:f>COUNTIFS('Dong bo'!L6:L1000,"Hoàn tất")</x:f>
-        <x:v>357</x:v>
+        <x:v>365</x:v>
       </x:c>
       <x:c r="D8" s="1"/>
       <x:c r="E8" s="1"/>
@@ -751,7 +751,7 @@
     <x:hyperlink ref="B14" location="'Quyet dinh'!A1"/>
     <x:hyperlink ref="B15" location="'Dong bo'!A1"/>
     <x:hyperlink ref="B16" location="'Quy trinh'!A1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="Rade9e0e4cbdd4596"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="R16206824dd1f40b9"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -887,7 +887,7 @@
         <x:v>Quản lý hồ sơ</x:v>
       </x:c>
       <x:c r="D6" s="8" t="str">
-        <x:v>v1.37</x:v>
+        <x:v>v1.39</x:v>
       </x:c>
       <x:c r="E6" s="8" t="str">
         <x:v>Sổ quản lý chính</x:v>
@@ -896,7 +896,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G6" s="8" t="str">
-        <x:v>RULE-01; STRUCTURE-01; LOGTEST-01; MOBILE-GUIDE-01; PATH-01; NATIVE-B-01</x:v>
+        <x:v>RULE-01; STRUCTURE-01; LOGTEST-01; MOBILE-GUIDE-01; PATH-01; NATIVE-B-01; MCP-01; EXPO-MCP-01</x:v>
       </x:c>
       <x:c r="H6" s="9" t="str">
         <x:v>Mở tài liệu</x:v>
@@ -906,10 +906,10 @@
       </x:c>
       <x:c r="J6" s="8" t="str"/>
       <x:c r="K6" s="8" t="str">
-        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+        <x:v>EXPO-MCP-01: Expo OAuth/CLI đã đăng nhập; expo-mcp0.2.4 devDependency. Allowlist chỉ tài liệu/thư viện/local; read_documentation/add_library qua Codex PASS. 31 mobile tests, lint/typecheck/dependency check PASS. Native app UI chờ build; mở phiên Codex mới, bật lại Metro khi dùng local.</x:v>
       </x:c>
       <x:c r="L6" s="10" t="n">
-        <x:v>46294</x:v>
+        <x:v>46295</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="68" customHeight="1">
@@ -1545,7 +1545,7 @@
         <x:v>Gói nguồn hồ sơ</x:v>
       </x:c>
       <x:c r="D24" s="8" t="str">
-        <x:v>v0.1.1 / NATIVE-B-01</x:v>
+        <x:v>v0.1.1 / EXPO-MCP-01</x:v>
       </x:c>
       <x:c r="E24" s="8" t="str">
         <x:v>Gói xuất</x:v>
@@ -1554,7 +1554,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G24" s="8" t="str">
-        <x:v>Quyết định theo chức năng; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01; PATH-01; NATIVE-B-01</x:v>
+        <x:v>Quyết định theo chức năng; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01; PATH-01; NATIVE-B-01; MCP-01; EXPO-MCP-01</x:v>
       </x:c>
       <x:c r="H24" s="9" t="str">
         <x:v>Mở tài liệu</x:v>
@@ -1564,10 +1564,10 @@
       </x:c>
       <x:c r="J24" s="8" t="str"/>
       <x:c r="K24" s="8" t="str">
-        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+        <x:v>EXPO-MCP-01: Expo OAuth/CLI đã đăng nhập; expo-mcp0.2.4 devDependency. Allowlist chỉ tài liệu/thư viện/local; read_documentation/add_library qua Codex PASS. 31 mobile tests, lint/typecheck/dependency check PASS. Native app UI chờ build; mở phiên Codex mới, bật lại Metro khi dùng local.</x:v>
       </x:c>
       <x:c r="L24" s="10" t="n">
-        <x:v>46294</x:v>
+        <x:v>46295</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="38" customHeight="1">
@@ -2661,7 +2661,7 @@
         <x:v>Thiết kế kỹ thuật</x:v>
       </x:c>
       <x:c r="D55" s="20" t="str">
-        <x:v>v0.1.1 / NATIVE-B-01</x:v>
+        <x:v>v0.1.1 / EXPO-MCP-01</x:v>
       </x:c>
       <x:c r="E55" s="20" t="str">
         <x:v>Gói hiện hành</x:v>
@@ -2670,7 +2670,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G55" s="20" t="str">
-        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01; PATH-01; NATIVE-B-01</x:v>
+        <x:v>Q03; PLAN-001/002/003/008; IMPLEMENT-01; TECH-01; STRUCTURE-01; LOGTEST-01; PATH-01; NATIVE-B-01; MCP-01; EXPO-MCP-01</x:v>
       </x:c>
       <x:c r="H55" s="20" t="str">
         <x:v>https://drive.google.com/file/d/18z-ReFxGP-RhX5_cOVTidcHJJGFfB48D/view?usp=drivesdk</x:v>
@@ -2682,10 +2682,10 @@
         <x:v>Bản trên Drive</x:v>
       </x:c>
       <x:c r="K55" s="20" t="str">
-        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+        <x:v>EXPO-MCP-01: Expo OAuth/CLI đã đăng nhập; expo-mcp0.2.4 devDependency. Allowlist chỉ tài liệu/thư viện/local; read_documentation/add_library qua Codex PASS. 31 mobile tests, lint/typecheck/dependency check PASS. Native app UI chờ build; mở phiên Codex mới, bật lại Metro khi dùng local.</x:v>
       </x:c>
       <x:c r="L55" s="21" t="n">
-        <x:v>46294</x:v>
+        <x:v>46295</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="105" customHeight="1">
@@ -3891,7 +3891,7 @@
         <x:v>Hướng dẫn phát triển</x:v>
       </x:c>
       <x:c r="D87" s="24" t="str">
-        <x:v>v1.1</x:v>
+        <x:v>v1.3</x:v>
       </x:c>
       <x:c r="E87" s="24" t="str">
         <x:v>Nguồn Markdown</x:v>
@@ -3900,7 +3900,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G87" s="24" t="str">
-        <x:v>MOBILE-GUIDE-01; NATIVE-B-01</x:v>
+        <x:v>MOBILE-GUIDE-01; NATIVE-B-01; MCP-01; EXPO-MCP-01</x:v>
       </x:c>
       <x:c r="H87" s="24" t="str">
         <x:v>https://drive.google.com/file/d/10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u/view?usp=drivesdk</x:v>
@@ -3912,10 +3912,10 @@
         <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
       </x:c>
       <x:c r="K87" s="24" t="str">
-        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+        <x:v>EXPO-MCP-01: Expo OAuth/CLI đã đăng nhập; expo-mcp0.2.4 devDependency. Allowlist chỉ tài liệu/thư viện/local; read_documentation/add_library qua Codex PASS. 31 mobile tests, lint/typecheck/dependency check PASS. Native app UI chờ build; mở phiên Codex mới, bật lại Metro khi dùng local.</x:v>
       </x:c>
       <x:c r="L87" s="24" t="n">
-        <x:v>46294</x:v>
+        <x:v>46295</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="110" customHeight="1">
@@ -3950,7 +3950,7 @@
         <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
       </x:c>
       <x:c r="K88" s="24" t="str">
-        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+        <x:v>Trạng thái triển khai môi trường: xem DOC-076 v1.1 (NATIVE-B-01), DOC-077/078 v1.2 (MCP-01, EXPO-MCP-01). Native binary/E2E còn pending. Nội dung bài này không đổi trong EXPO-MCP-01.</x:v>
       </x:c>
       <x:c r="L88" s="24" t="n">
         <x:v>46294</x:v>
@@ -3988,7 +3988,7 @@
         <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
       </x:c>
       <x:c r="K89" s="24" t="str">
-        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+        <x:v>Trạng thái triển khai môi trường: xem DOC-076 v1.1 (NATIVE-B-01), DOC-077/078 v1.2 (MCP-01, EXPO-MCP-01). Native binary/E2E còn pending. Nội dung bài này không đổi trong EXPO-MCP-01.</x:v>
       </x:c>
       <x:c r="L89" s="24" t="n">
         <x:v>46294</x:v>
@@ -4026,7 +4026,7 @@
         <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
       </x:c>
       <x:c r="K90" s="24" t="str">
-        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+        <x:v>Trạng thái triển khai môi trường: xem DOC-076 v1.1 (NATIVE-B-01), DOC-077/078 v1.2 (MCP-01, EXPO-MCP-01). Native binary/E2E còn pending. Nội dung bài này không đổi trong EXPO-MCP-01.</x:v>
       </x:c>
       <x:c r="L90" s="24" t="n">
         <x:v>46294</x:v>
@@ -4064,7 +4064,7 @@
         <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
       </x:c>
       <x:c r="K91" s="24" t="str">
-        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+        <x:v>Trạng thái triển khai môi trường: xem DOC-076 v1.1 (NATIVE-B-01), DOC-077/078 v1.2 (MCP-01, EXPO-MCP-01). Native binary/E2E còn pending. Nội dung bài này không đổi trong EXPO-MCP-01.</x:v>
       </x:c>
       <x:c r="L91" s="24" t="n">
         <x:v>46294</x:v>
@@ -4081,7 +4081,7 @@
         <x:v>Hướng dẫn phát triển</x:v>
       </x:c>
       <x:c r="D92" s="24" t="str">
-        <x:v>v1.0</x:v>
+        <x:v>v1.2</x:v>
       </x:c>
       <x:c r="E92" s="24" t="str">
         <x:v>Nguồn Markdown</x:v>
@@ -4090,7 +4090,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G92" s="24" t="str">
-        <x:v>MOBILE-GUIDE-01</x:v>
+        <x:v>MOBILE-GUIDE-01; MCP-01; EXPO-MCP-01</x:v>
       </x:c>
       <x:c r="H92" s="24" t="str">
         <x:v>https://drive.google.com/file/d/10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u/view?usp=drivesdk</x:v>
@@ -4102,10 +4102,10 @@
         <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
       </x:c>
       <x:c r="K92" s="24" t="str">
-        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+        <x:v>EXPO-MCP-01: Expo OAuth/CLI đã đăng nhập; expo-mcp0.2.4 devDependency. Allowlist chỉ tài liệu/thư viện/local; read_documentation/add_library qua Codex PASS. 31 mobile tests, lint/typecheck/dependency check PASS. Native app UI chờ build; mở phiên Codex mới, bật lại Metro khi dùng local.</x:v>
       </x:c>
       <x:c r="L92" s="24" t="n">
-        <x:v>46294</x:v>
+        <x:v>46295</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="110" customHeight="1">
@@ -4119,7 +4119,7 @@
         <x:v>Hướng dẫn phát triển</x:v>
       </x:c>
       <x:c r="D93" s="24" t="str">
-        <x:v>v1.0</x:v>
+        <x:v>v1.2</x:v>
       </x:c>
       <x:c r="E93" s="24" t="str">
         <x:v>Nguồn Markdown</x:v>
@@ -4128,7 +4128,7 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G93" s="24" t="str">
-        <x:v>MOBILE-GUIDE-01</x:v>
+        <x:v>MOBILE-GUIDE-01; MCP-01; EXPO-MCP-01</x:v>
       </x:c>
       <x:c r="H93" s="24" t="str">
         <x:v>https://drive.google.com/file/d/10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u/view?usp=drivesdk</x:v>
@@ -4140,10 +4140,10 @@
         <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
       </x:c>
       <x:c r="K93" s="24" t="str">
-        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+        <x:v>EXPO-MCP-01: Expo OAuth/CLI đã đăng nhập; expo-mcp0.2.4 devDependency. Allowlist chỉ tài liệu/thư viện/local; read_documentation/add_library qua Codex PASS. 31 mobile tests, lint/typecheck/dependency check PASS. Native app UI chờ build; mở phiên Codex mới, bật lại Metro khi dùng local.</x:v>
       </x:c>
       <x:c r="L93" s="24" t="n">
-        <x:v>46294</x:v>
+        <x:v>46295</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="110" customHeight="1">
@@ -4178,7 +4178,7 @@
         <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
       </x:c>
       <x:c r="K94" s="24" t="str">
-        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+        <x:v>Trạng thái triển khai môi trường: xem DOC-076 v1.1 (NATIVE-B-01), DOC-077/078 v1.2 (MCP-01, EXPO-MCP-01). Native binary/E2E còn pending. Nội dung bài này không đổi trong EXPO-MCP-01.</x:v>
       </x:c>
       <x:c r="L94" s="24" t="n">
         <x:v>46294</x:v>
@@ -4216,7 +4216,7 @@
         <x:v>DOC-081 chứa 9 Markdown; giải nén vào docs/huong-dan-mobile</x:v>
       </x:c>
       <x:c r="K95" s="24" t="str">
-        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+        <x:v>Trạng thái triển khai môi trường: xem DOC-076 v1.1 (NATIVE-B-01), DOC-077/078 v1.2 (MCP-01, EXPO-MCP-01). Native binary/E2E còn pending. Nội dung bài này không đổi trong EXPO-MCP-01.</x:v>
       </x:c>
       <x:c r="L95" s="24" t="n">
         <x:v>46294</x:v>
@@ -4227,13 +4227,13 @@
         <x:v>DOC-081</x:v>
       </x:c>
       <x:c r="B96" s="24" t="str">
-        <x:v>Gói hướng dẫn phát triển mobile v1.1</x:v>
+        <x:v>Gói hướng dẫn phát triển mobile v1.3</x:v>
       </x:c>
       <x:c r="C96" s="24" t="str">
         <x:v>Hướng dẫn phát triển</x:v>
       </x:c>
       <x:c r="D96" s="24" t="str">
-        <x:v>v1.1</x:v>
+        <x:v>v1.3</x:v>
       </x:c>
       <x:c r="E96" s="24" t="str">
         <x:v>Gói xuất</x:v>
@@ -4242,22 +4242,22 @@
         <x:v>Mới nhất</x:v>
       </x:c>
       <x:c r="G96" s="24" t="str">
-        <x:v>MOBILE-GUIDE-01; NATIVE-B-01</x:v>
+        <x:v>MOBILE-GUIDE-01; NATIVE-B-01; MCP-01; EXPO-MCP-01</x:v>
       </x:c>
       <x:c r="H96" s="24" t="str">
         <x:v>https://drive.google.com/file/d/10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u/view?usp=drivesdk</x:v>
       </x:c>
       <x:c r="I96" s="24" t="str">
-        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/huong-dan-mobile-v1.1.zip</x:v>
+        <x:v>/Users/j2866/Documents/anhthai/dich-vu-quanh-ban/docs/huong-dan-mobile/huong-dan-mobile-v1.3.zip</x:v>
       </x:c>
       <x:c r="J96" s="24" t="str">
-        <x:v>9 Markdown hiện hành; v1.0 giữ lịch sử, đã thay thế</x:v>
+        <x:v>9 Markdown hiện hành; v1.0/v1.1/v1.2 giữ lịch sử, đã thay thế</x:v>
       </x:c>
       <x:c r="K96" s="24" t="str">
-        <x:v>NATIVE-B-01: hai máy ảo booted; dev-client57.0.19/Expo57.0.26, CNG, app ID/scheme và HTTP Debug-only đã kiểm. 31 mobile tests, lint/typecheck/bundle/config và kiểm âm Release PASS. Chưa build/cài APK/.app hoặc nghiệm thu native E2E; Maestro chưa có. DOC-076 v1.1 ghi bằng chứng và bước C.</x:v>
+        <x:v>EXPO-MCP-01: Expo OAuth/CLI đã đăng nhập; expo-mcp0.2.4 devDependency. Allowlist chỉ tài liệu/thư viện/local; read_documentation/add_library qua Codex PASS. 31 mobile tests, lint/typecheck/dependency check PASS. Native app UI chờ build; mở phiên Codex mới, bật lại Metro khi dùng local.</x:v>
       </x:c>
       <x:c r="L96" s="24" t="n">
-        <x:v>46294</x:v>
+        <x:v>46295</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4272,81 +4272,81 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="Re224eae1e74348e3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R546785db0cae47ed"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="R508bedfc088d4ab0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="R616778eb3f4048df"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="R1b211813d46540cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="R0468122d78894ffd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="R15bd6f35db8b416c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="R3060d95295644859"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="Rc44fea8e9c484584"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="Ra272775f4a1c4a4b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="Rfa95c8d2df934b7f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="Ra134f6f1cbe2423c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="Rb3da56f78ac64aea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="Rbce77a51bf844789"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="R0e68e0d0f572450a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="Rc8213526136a4798"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="R365e0d2671e44722"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="R8cacb40c99034a69"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="Rcf27fd27d4194cb3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="R8aebba1aa2fb4045"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="R1f6b1585ce4a45b9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="R5a2bec1a68c24739"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="Rc854c8764a284160"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="Rbdb62bda8e624d2e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="R53b05c0b70474353"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="Rb0bc34108a60460a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="R1260c11803ac42a2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="R19ff43afc3b64e14"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="Re9d5b186b42f4bec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R84210047cfd44006"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="Rb9c8d6c1a10b425a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="R939c02632a664f71"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="R5a4d4b3a6b414e2f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R3ee6d02c08d449c0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="R5d0170d806ad4a15"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="R674b42d1dec14a95"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="R41d80d412a2547ed"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="R453a8ee6b1b34c4e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="R406c1fb2358146bc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="R403772f3c3ca478d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="R401c4fd87279444f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="R34bbc39c50b14925"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="R317e76c04ef1448a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="Rfa967a9e5bd84e4a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="R9c005adb2d3d4ae9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="R44a89ac8e2404ef0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="Rb90ca3edc23f4239"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="Re94f0ed7dce54493"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="Rd75dabe6859a41b6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="Rd1ff5adf9baa4958"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="R2f115f07255d406a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="R51f9588e829a4a86"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="R703a126e8def4dc5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="R11e63641bd4848b5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="R7a7730ccbd114fde"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="Rf191848d6b874690"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="R6b5a56cb219e404b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="Rdba631acb3e24bbd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="R4e1e8c5c506e4d4e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="R74d9315f9f0842d0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="Ra3646439ef604f1f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="R2d51a4675bcd4f7d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="Rf840bf6864f54967"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="Rd59e04d1542244bf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="Ra7dcbfc41c27401b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="R943c29438f6048fd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="R542dd4e85d084509"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="R8737c8b9b5134a2a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="R730f6b542c3448da"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="Rc28b580037d14c3f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="R56c21a64f49148e9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="R3f284589c1414a41"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R27129cdb708b49f5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="R50fda4574d564ddd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="Rea62fcbd98614dd7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="Rf96ba5f546c84833"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="Re621a2f147824706"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="Rbf5cae1d0a41424f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="Ra72391a244934f15"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="R27a40306e10a4b38"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="R0fc98bda7de443e9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="Ra894431175864ba4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="R49865ed40f574dec"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="R225c5b5b50d64253"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="R004e3d3172d74c8a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="R3b4bacb1cee64dd0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="R467af5fa0aa54804"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="R9d53a0dd5adb4fc3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="R6af6aa870e014325"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="R3e72430f2f274b79"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="Rb905e97fddbd49ec"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="Rb82a5ebdbd054b89"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="R441284a6dd2f44f9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="Rf10f174361d14914"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="Ra6f7a4d1551447d7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="R7968b71e3726421d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="R6e83a49f795648e0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="R27a5fb96b1d54401"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="R8278eecffe4c4907"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="R8c3e76adbbfb4445"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="R28006b8c3d194cb3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="Ra0f088a2acef4f68"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="Rc36ec6bb049a4727"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="Rae8e46d83fb6493a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="R0bd2ccbb186843de"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="R4ac9ef0081f645c9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="R48b86cf6c00c4bc4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="Rd31f7e3046e844d7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="R24a4dd8e83de4b3a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="Rf1687f7596c84876"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="R043af0f4c2ad4bd9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="R0394adc1bee0460e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="Rc98dac23404f4f8b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="R7e716923d3c441e6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="Red104c59be3f4757"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="R3c5e3b151d504855"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="R3d3d4103f7cf40f2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="Re7350a6cfe794afe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="R09270fab28cf4878"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="Ra86d9f9946004fd4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="R6048c4c23e194140"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="R3cdfe5effb074b67"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="Rd5cf65280688410e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="R925009212e224be3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="R92052a49bc704656"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="R2184649a3be54754"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="R7e7cb80f49c2429d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="Ra34314f0d5814e27"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="R231b76117d494577"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="Rb8ef5bfe8ef04aee"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="R3229ac14b2e6470a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="Rb2b887508f5f49bf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="Re36addc95b7b45bd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="Raf36a229ab354078"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="R3edc97d4ca5c4943"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="R2ecdb4a67e7a42db"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="Re6215b4bb8b94315"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="R991d6666fddb458f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="Rf81a465b6aa54873"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="R1e4eed0aa2da4f9f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="R33b3232295d74a7a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="R5182d0dacc484b59"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6be0ea4b5f0748be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85e16a5234ea4968"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21182,7 +21182,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15f16b18190e4562"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a24aa06b86e40bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22497,11 +22497,51 @@
         <x:v>46294</x:v>
       </x:c>
     </x:row>
-    <x:row r="60">
-      <x:c r="G60" s="11"/>
-    </x:row>
-    <x:row r="61">
-      <x:c r="G61" s="11"/>
+    <x:row r="60" ht="150" customHeight="1">
+      <x:c r="A60" s="24" t="str">
+        <x:v>MCP-01</x:v>
+      </x:c>
+      <x:c r="B60" s="24" t="str">
+        <x:v>Kết nối Mobile MCP tới Codex</x:v>
+      </x:c>
+      <x:c r="C60" s="24" t="str">
+        <x:v>Đã chốt</x:v>
+      </x:c>
+      <x:c r="D60" s="24" t="str">
+        <x:v>Chủ dự án yêu cầu làm bài05. Kết nối Mobile MCP local và kiểm Android/iOS. Expo MCP tùy chọn chưa cài; không production/tiền thật.</x:v>
+      </x:c>
+      <x:c r="E60" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="F60" s="24" t="str">
+        <x:v>Yêu cầu trực tiếp30/09/2026; DOC-077/078 v1.1. Server/tool qua stdio PASS; tool trong phiên IDE mới cần nạp lại.</x:v>
+      </x:c>
+      <x:c r="G60" s="25" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="150" customHeight="1">
+      <x:c r="A61" s="24" t="str">
+        <x:v>EXPO-MCP-01</x:v>
+      </x:c>
+      <x:c r="B61" s="24" t="str">
+        <x:v>Cài Expo MCP, chỉ dùng tính năng miễn phí</x:v>
+      </x:c>
+      <x:c r="C61" s="24" t="str">
+        <x:v>Đã chốt</x:v>
+      </x:c>
+      <x:c r="D61" s="24" t="str">
+        <x:v>Chủ dự án yêu cầu cài và dùng tính năng miễn phí, hoàn tất OAuth/CLI. Bật allowlist tài liệu/thư viện/local; không search trả phí, build cloud hoặc publish.</x:v>
+      </x:c>
+      <x:c r="E61" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="F61" s="24" t="str">
+        <x:v>Yêu cầu trực tiếp30/09/2026; DOC-077/078 v1.2. Kiểm bằng Codex MCP; thao tác UI app chờ binary.</x:v>
+      </x:c>
+      <x:c r="G61" s="25" t="n">
+        <x:v>46295</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="G62" s="11"/>
@@ -25323,7 +25363,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51f8dead372c41b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e5ea893249e40c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41593,41 +41633,445 @@
         <x:v>Không áp dụng</x:v>
       </x:c>
     </x:row>
-    <x:row r="424">
-      <x:c r="I424" s="11"/>
-    </x:row>
-    <x:row r="425">
-      <x:c r="I425" s="11"/>
-    </x:row>
-    <x:row r="426">
-      <x:c r="I426" s="11"/>
-    </x:row>
-    <x:row r="427">
-      <x:c r="I427" s="11"/>
-    </x:row>
-    <x:row r="428">
-      <x:c r="I428" s="11"/>
-    </x:row>
-    <x:row r="429">
-      <x:c r="I429" s="11"/>
-    </x:row>
-    <x:row r="430">
-      <x:c r="I430" s="11"/>
-    </x:row>
-    <x:row r="431">
-      <x:c r="I431" s="11"/>
-    </x:row>
-    <x:row r="432">
-      <x:c r="I432" s="11"/>
-    </x:row>
-    <x:row r="433">
-      <x:c r="I433" s="11"/>
-    </x:row>
-    <x:row r="434">
-      <x:c r="I434" s="11"/>
-    </x:row>
-    <x:row r="435">
-      <x:c r="I435" s="11"/>
+    <x:row r="424" ht="165" customHeight="1">
+      <x:c r="A424" s="24" t="str">
+        <x:v>MCP-20260930</x:v>
+      </x:c>
+      <x:c r="B424" s="24" t="str">
+        <x:v>MCP-01</x:v>
+      </x:c>
+      <x:c r="C424" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D424" s="24" t="str">
+        <x:v>DOC-072/077/078</x:v>
+      </x:c>
+      <x:c r="E424" s="24" t="str">
+        <x:v>Cấu hình và kiểm MCP, phân biệt E2E sản phẩm</x:v>
+      </x:c>
+      <x:c r="F424" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G424" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H424" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I424" s="25" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="J424" s="24" t="str">
+        <x:v>DOC-072 v1.2; DOC-077/078 v1.1; test-results/mcp/2026-09-30/result.json và ảnh Android/iOS. Markdown/ZIP khớp; Drive trong DOC-081 cùng ID.</x:v>
+      </x:c>
+      <x:c r="K424" s="24"/>
+      <x:c r="L424" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="425" ht="165" customHeight="1">
+      <x:c r="A425" s="24" t="str">
+        <x:v>MCP-20260930</x:v>
+      </x:c>
+      <x:c r="B425" s="24" t="str">
+        <x:v>MCP-01</x:v>
+      </x:c>
+      <x:c r="C425" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D425" s="24" t="str">
+        <x:v>DOC-081</x:v>
+      </x:c>
+      <x:c r="E425" s="24" t="str">
+        <x:v>Tái tạo gói mobile v1.2</x:v>
+      </x:c>
+      <x:c r="F425" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G425" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H425" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I425" s="25" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="J425" s="24" t="str">
+        <x:v>docs/huong-dan-mobile/huong-dan-mobile-v1.2.zip, 9 nguồn Markdown khớp bytes; Drive10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u đọc lại khớp.</x:v>
+      </x:c>
+      <x:c r="K425" s="24"/>
+      <x:c r="L425" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="426" ht="165" customHeight="1">
+      <x:c r="A426" s="24" t="str">
+        <x:v>MCP-20260930</x:v>
+      </x:c>
+      <x:c r="B426" s="24" t="str">
+        <x:v>MCP-01</x:v>
+      </x:c>
+      <x:c r="C426" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D426" s="24" t="str">
+        <x:v>DOC-018/040</x:v>
+      </x:c>
+      <x:c r="E426" s="24" t="str">
+        <x:v>Đồng bộ nguồn hướng dẫn trong gói kỹ thuật</x:v>
+      </x:c>
+      <x:c r="F426" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G426" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H426" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I426" s="25" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="J426" s="24" t="str">
+        <x:v>architecture-source-v0.1.1.zip và technical-design-v0.1.1.zip / MCP-01; cập nhật 3 Markdown và ghi revision MCP-01.txt, bảo toàn entry khác. Drive cùng ID, đọc lại bytes.</x:v>
+      </x:c>
+      <x:c r="K426" s="24"/>
+      <x:c r="L426" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="427" ht="165" customHeight="1">
+      <x:c r="A427" s="24" t="str">
+        <x:v>MCP-20260930</x:v>
+      </x:c>
+      <x:c r="B427" s="24" t="str">
+        <x:v>MCP-01</x:v>
+      </x:c>
+      <x:c r="C427" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D427" s="24" t="str">
+        <x:v>DOC-000</x:v>
+      </x:c>
+      <x:c r="E427" s="24" t="str">
+        <x:v>Sổ quản lý v1.38</x:v>
+      </x:c>
+      <x:c r="F427" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G427" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H427" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I427" s="25" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="J427" s="24" t="str">
+        <x:v>Danh muc/Quyet dinh/Dong bo; Anh huong F17/F18/F20 đã có DOC-072–081. Bảo toàn công thức/style và nội dung ngoài phạm vi; Drive18eWx9ObcWbpRNSIsxKs7YTwBpR-ZPjQq cùng ID, đọc lại.</x:v>
+      </x:c>
+      <x:c r="K427" s="24"/>
+      <x:c r="L427" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="428" ht="165" customHeight="1">
+      <x:c r="A428" s="24" t="str">
+        <x:v>MCP-20260930</x:v>
+      </x:c>
+      <x:c r="B428" s="24" t="str">
+        <x:v>MCP-01</x:v>
+      </x:c>
+      <x:c r="C428" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D428" s="24" t="str">
+        <x:v>DOC-073/074/075/076/079/080; DOC-064/065/070/071; BRD/PRD/FR/NFR/SRS/UX/ERD/API/QA</x:v>
+      </x:c>
+      <x:c r="E428" s="24" t="str">
+        <x:v>Rà ảnh hưởng</x:v>
+      </x:c>
+      <x:c r="F428" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
+      <x:c r="G428" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H428" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I428" s="25" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="J428" s="24" t="str">
+        <x:v>Cross-search MCP/native: bài01 giữ snapshot; bài04 B và các runbook vẫn đúng. Native E2E sản phẩm giữ pending.</x:v>
+      </x:c>
+      <x:c r="K428" s="24" t="str">
+        <x:v>Chỉ kết nối công cụ máy phát triển; không sửa code, nghiệp vụ, UI/contract, SDK/build hoặc kế hoạch.</x:v>
+      </x:c>
+      <x:c r="L428" s="24" t="str">
+        <x:v>Không áp dụng có lý do</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="429" ht="165" customHeight="1">
+      <x:c r="A429" s="24" t="str">
+        <x:v>MCP-20260930</x:v>
+      </x:c>
+      <x:c r="B429" s="24" t="str">
+        <x:v>MCP-01</x:v>
+      </x:c>
+      <x:c r="C429" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D429" s="24" t="str">
+        <x:v>HTML/localhost; UI-UX ZIP; archive</x:v>
+      </x:c>
+      <x:c r="E429" s="24" t="str">
+        <x:v>Rà bản phục vụ và lịch sử</x:v>
+      </x:c>
+      <x:c r="F429" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
+      <x:c r="G429" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H429" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I429" s="25" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="J429" s="24" t="str">
+        <x:v>3 Markdown thay đổi không có bản HTML/localhost riêng; UI ZIP không chứa nguồn hướng dẫn. Guide v1.0/v1.1 giữ nguyên.</x:v>
+      </x:c>
+      <x:c r="K429" s="24" t="str">
+        <x:v>Không sửa prototype, không tạo bản phục vụ mới, không sửa lịch sử.</x:v>
+      </x:c>
+      <x:c r="L429" s="24" t="str">
+        <x:v>Không áp dụng có lý do</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="430" ht="165" customHeight="1">
+      <x:c r="A430" s="24" t="str">
+        <x:v>EXPO-MCP-20260930</x:v>
+      </x:c>
+      <x:c r="B430" s="24" t="str">
+        <x:v>EXPO-MCP-01</x:v>
+      </x:c>
+      <x:c r="C430" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D430" s="24" t="str">
+        <x:v>DOC-072/077/078</x:v>
+      </x:c>
+      <x:c r="E430" s="24" t="str">
+        <x:v>Cài Expo MCP và chỉ dùng công cụ miễn phí</x:v>
+      </x:c>
+      <x:c r="F430" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G430" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H430" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I430" s="25" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="J430" s="24" t="str">
+        <x:v>DOC-072 v1.3; DOC-077/078 v1.2. test-results/mcp/expo-2026-09-30: Codex connected/OAuth, read_documentation/add_library PASS. Local tools expose; app UI chờ binary.</x:v>
+      </x:c>
+      <x:c r="K430" s="24"/>
+      <x:c r="L430" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="431" ht="165" customHeight="1">
+      <x:c r="A431" s="24" t="str">
+        <x:v>EXPO-MCP-20260930</x:v>
+      </x:c>
+      <x:c r="B431" s="24" t="str">
+        <x:v>EXPO-MCP-01</x:v>
+      </x:c>
+      <x:c r="C431" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D431" s="24" t="str">
+        <x:v>DOC-081</x:v>
+      </x:c>
+      <x:c r="E431" s="24" t="str">
+        <x:v>Gói hướng dẫn v1.3</x:v>
+      </x:c>
+      <x:c r="F431" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G431" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H431" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I431" s="25" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="J431" s="24" t="str">
+        <x:v>docs/huong-dan-mobile/huong-dan-mobile-v1.3.zip; 9 Markdown khớp nguồn. Drive10gU2AUdgJLgIZH1UNs1Q2AE225sRlD-u cùng ID, đọc lại khớp.</x:v>
+      </x:c>
+      <x:c r="K431" s="24"/>
+      <x:c r="L431" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="432" ht="165" customHeight="1">
+      <x:c r="A432" s="24" t="str">
+        <x:v>EXPO-MCP-20260930</x:v>
+      </x:c>
+      <x:c r="B432" s="24" t="str">
+        <x:v>EXPO-MCP-01</x:v>
+      </x:c>
+      <x:c r="C432" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D432" s="24" t="str">
+        <x:v>DOC-018/040</x:v>
+      </x:c>
+      <x:c r="E432" s="24" t="str">
+        <x:v>Gói kỹ thuật / EXPO-MCP-01</x:v>
+      </x:c>
+      <x:c r="F432" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G432" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H432" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I432" s="25" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="J432" s="24" t="str">
+        <x:v>Cập nhật nguồn hướng dẫn và dependency liên quan nếu có trong ZIP, EXPO-MCP-01.txt; giữ entry khác. Drive cùng ID, đọc lại khớp.</x:v>
+      </x:c>
+      <x:c r="K432" s="24"/>
+      <x:c r="L432" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="433" ht="165" customHeight="1">
+      <x:c r="A433" s="24" t="str">
+        <x:v>EXPO-MCP-20260930</x:v>
+      </x:c>
+      <x:c r="B433" s="24" t="str">
+        <x:v>EXPO-MCP-01</x:v>
+      </x:c>
+      <x:c r="C433" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D433" s="24" t="str">
+        <x:v>DOC-000</x:v>
+      </x:c>
+      <x:c r="E433" s="24" t="str">
+        <x:v>Sổ quản lý v1.39</x:v>
+      </x:c>
+      <x:c r="F433" s="24" t="str">
+        <x:v>Đã cập nhật</x:v>
+      </x:c>
+      <x:c r="G433" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H433" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I433" s="25" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="J433" s="24" t="str">
+        <x:v>Danh muc/Quyet dinh/Dong bo; giữ Anh huong F17/F18/F20 đã có. Công thức/định dạng giữ nguyên; Drive cùng ID đọc lại. Chuẩn hóa kết quả MCP-01 về Hoàn tất/Không áp dụng có lý do để bộ đếm hiện có nhận đúng.</x:v>
+      </x:c>
+      <x:c r="K433" s="24"/>
+      <x:c r="L433" s="24" t="str">
+        <x:v>Hoàn tất</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="434" ht="165" customHeight="1">
+      <x:c r="A434" s="24" t="str">
+        <x:v>EXPO-MCP-20260930</x:v>
+      </x:c>
+      <x:c r="B434" s="24" t="str">
+        <x:v>EXPO-MCP-01</x:v>
+      </x:c>
+      <x:c r="C434" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D434" s="24" t="str">
+        <x:v>DOC-073/074/075/076/079/080; DOC-064/065/070/071; BRD/PRD/FR/NFR/SRS/UX/ERD/API/QA</x:v>
+      </x:c>
+      <x:c r="E434" s="24" t="str">
+        <x:v>Rà ảnh hưởng</x:v>
+      </x:c>
+      <x:c r="F434" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
+      <x:c r="G434" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H434" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I434" s="25" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="J434" s="24" t="str">
+        <x:v>Chỉ thêm devDependency expo-mcp và cấu hình Codex trên máy. DOC-077/078 ghi giới hạn miễn phí; binary/E2E vẫn pending.</x:v>
+      </x:c>
+      <x:c r="K434" s="24" t="str">
+        <x:v>Không đổi chức năng/UI/contract hoặc quy trình build/test cũ; không sửa tài liệu nghiệp vụ.</x:v>
+      </x:c>
+      <x:c r="L434" s="24" t="str">
+        <x:v>Không áp dụng có lý do</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="435" ht="165" customHeight="1">
+      <x:c r="A435" s="24" t="str">
+        <x:v>EXPO-MCP-20260930</x:v>
+      </x:c>
+      <x:c r="B435" s="24" t="str">
+        <x:v>EXPO-MCP-01</x:v>
+      </x:c>
+      <x:c r="C435" s="24" t="str">
+        <x:v>F17/F18/F20</x:v>
+      </x:c>
+      <x:c r="D435" s="24" t="str">
+        <x:v>HTML/localhost; UI-UX ZIP; archive</x:v>
+      </x:c>
+      <x:c r="E435" s="24" t="str">
+        <x:v>Rà bản xuất khác</x:v>
+      </x:c>
+      <x:c r="F435" s="24" t="str">
+        <x:v>Không áp dụng</x:v>
+      </x:c>
+      <x:c r="G435" s="24" t="str">
+        <x:v>Có</x:v>
+      </x:c>
+      <x:c r="H435" s="24" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="I435" s="25" t="n">
+        <x:v>46295</x:v>
+      </x:c>
+      <x:c r="J435" s="24" t="str">
+        <x:v>3 Markdown không có bản HTML phục vụ riêng; UI ZIP không chứa nguồn này. Guidev1.0/v1.1/v1.2 giữ nguyên.</x:v>
+      </x:c>
+      <x:c r="K435" s="24" t="str">
+        <x:v>Không đổi prototype hoặc lịch sử.</x:v>
+      </x:c>
+      <x:c r="L435" s="24" t="str">
+        <x:v>Không áp dụng có lý do</x:v>
+      </x:c>
     </x:row>
     <x:row r="436">
       <x:c r="I436" s="11"/>
@@ -43338,7 +43782,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1e5d84f4cf84a7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40db3720e7bc4123"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43580,7 +44024,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc86cf20cc07a4bd5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbdad465e78c41e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>